<commit_message>
Trade values: guard the reception refresh against thin mid-week data; refresh to week 4
A refresh now carries forward lines for players with nothing posted yet
(tagged "carried"), warns when few fresh lines came in, and the
per-position replacement level falls back to the last known value (then
the lowest posted line) when the replacement tier has fewer than
replacement_min_lines posted, instead of collapsing to 0.0 and gutting
every other position in the zero-sum step. receptions.json now remembers
the replacement levels for the next refresh. Snapshot refreshed to 2026
week 4 (103 fresh lines, 88 carried).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TradeValueSheets/TradeValues_FullPPR_10team.xlsx
+++ b/TradeValueSheets/TradeValues_FullPPR_10team.xlsx
@@ -618,7 +618,7 @@
     </row>
     <row r="5">
       <c r="A5" s="6" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B5" s="7" t="n"/>
       <c r="C5" s="7" t="n"/>
@@ -650,15 +650,15 @@
     </row>
     <row r="7">
       <c r="A7" s="6" t="n">
-        <v>61</v>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Kenneth Walker III</t>
-        </is>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="B7" s="7" t="n"/>
       <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Jaxon Smith-Njigba</t>
+        </is>
+      </c>
       <c r="E7" s="7" t="n"/>
       <c r="F7" s="7" t="n"/>
       <c r="G7" s="7" t="n"/>
@@ -666,15 +666,15 @@
     </row>
     <row r="8">
       <c r="A8" s="6" t="n">
-        <v>60</v>
-      </c>
-      <c r="B8" s="7" t="n"/>
+        <v>61</v>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Kenneth Walker III</t>
+        </is>
+      </c>
       <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>Jaxon Smith-Njigba</t>
-        </is>
-      </c>
+      <c r="D8" s="7" t="n"/>
       <c r="E8" s="7" t="n"/>
       <c r="F8" s="7" t="n"/>
       <c r="G8" s="7" t="n"/>
@@ -682,15 +682,15 @@
     </row>
     <row r="9">
       <c r="A9" s="6" t="n">
-        <v>60</v>
-      </c>
-      <c r="B9" s="7" t="n"/>
+        <v>59</v>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Christian McCaffrey</t>
+        </is>
+      </c>
       <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>Ja'Marr Chase</t>
-        </is>
-      </c>
+      <c r="D9" s="7" t="n"/>
       <c r="E9" s="7" t="n"/>
       <c r="F9" s="7" t="n"/>
       <c r="G9" s="7" t="n"/>
@@ -700,13 +700,13 @@
       <c r="A10" s="6" t="n">
         <v>59</v>
       </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>Christian McCaffrey</t>
-        </is>
-      </c>
+      <c r="B10" s="7" t="n"/>
       <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Ja'Marr Chase</t>
+        </is>
+      </c>
       <c r="E10" s="7" t="n"/>
       <c r="F10" s="7" t="n"/>
       <c r="G10" s="7" t="n"/>
@@ -794,7 +794,7 @@
     </row>
     <row r="16">
       <c r="A16" s="6" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
@@ -810,15 +810,15 @@
     </row>
     <row r="17">
       <c r="A17" s="6" t="n">
-        <v>50</v>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>James Cook III</t>
-        </is>
-      </c>
+        <v>47</v>
+      </c>
+      <c r="B17" s="7" t="n"/>
       <c r="C17" s="7" t="n"/>
-      <c r="D17" s="7" t="n"/>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>CeeDee Lamb</t>
+        </is>
+      </c>
       <c r="E17" s="7" t="n"/>
       <c r="F17" s="7" t="n"/>
       <c r="G17" s="7" t="n"/>
@@ -826,15 +826,15 @@
     </row>
     <row r="18">
       <c r="A18" s="6" t="n">
-        <v>48</v>
-      </c>
-      <c r="B18" s="7" t="n"/>
+        <v>45</v>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>James Cook III</t>
+        </is>
+      </c>
       <c r="C18" s="7" t="n"/>
-      <c r="D18" s="7" t="inlineStr">
-        <is>
-          <t>CeeDee Lamb</t>
-        </is>
-      </c>
+      <c r="D18" s="7" t="n"/>
       <c r="E18" s="7" t="n"/>
       <c r="F18" s="7" t="n"/>
       <c r="G18" s="7" t="n"/>
@@ -970,15 +970,15 @@
     </row>
     <row r="27">
       <c r="A27" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="B27" s="7" t="n"/>
+        <v>34</v>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>D'Andre Swift</t>
+        </is>
+      </c>
       <c r="C27" s="7" t="n"/>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>Nico Collins</t>
-        </is>
-      </c>
+      <c r="D27" s="7" t="n"/>
       <c r="E27" s="7" t="n"/>
       <c r="F27" s="7" t="n"/>
       <c r="G27" s="7" t="n"/>
@@ -988,13 +988,13 @@
       <c r="A28" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="B28" s="7" t="inlineStr">
-        <is>
-          <t>Kyren Williams</t>
-        </is>
-      </c>
+      <c r="B28" s="7" t="n"/>
       <c r="C28" s="7" t="n"/>
-      <c r="D28" s="7" t="n"/>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>Nico Collins</t>
+        </is>
+      </c>
       <c r="E28" s="7" t="n"/>
       <c r="F28" s="7" t="n"/>
       <c r="G28" s="7" t="n"/>
@@ -1002,11 +1002,11 @@
     </row>
     <row r="29">
       <c r="A29" s="6" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>D'Andre Swift</t>
+          <t>Kyren Williams</t>
         </is>
       </c>
       <c r="C29" s="7" t="n"/>
@@ -1018,35 +1018,35 @@
     </row>
     <row r="30">
       <c r="A30" s="6" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B30" s="7" t="n"/>
       <c r="C30" s="7" t="n"/>
       <c r="D30" s="7" t="n"/>
       <c r="E30" s="7" t="n"/>
-      <c r="F30" s="7" t="n"/>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>Trey McBride</t>
+        </is>
+      </c>
       <c r="G30" s="7" t="n"/>
-      <c r="H30" s="7" t="inlineStr">
-        <is>
-          <t>Josh Allen</t>
-        </is>
-      </c>
+      <c r="H30" s="7" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="n">
-        <v>33</v>
-      </c>
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>Omarion Hampton</t>
-        </is>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="B31" s="7" t="n"/>
       <c r="C31" s="7" t="n"/>
       <c r="D31" s="7" t="n"/>
       <c r="E31" s="7" t="n"/>
       <c r="F31" s="7" t="n"/>
       <c r="G31" s="7" t="n"/>
-      <c r="H31" s="7" t="n"/>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Josh Allen</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="n">
@@ -1098,17 +1098,17 @@
     </row>
     <row r="35">
       <c r="A35" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="B35" s="7" t="n"/>
+        <v>29</v>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Jeremiyah Love</t>
+        </is>
+      </c>
       <c r="C35" s="7" t="n"/>
       <c r="D35" s="7" t="n"/>
       <c r="E35" s="7" t="n"/>
-      <c r="F35" s="7" t="inlineStr">
-        <is>
-          <t>Trey McBride</t>
-        </is>
-      </c>
+      <c r="F35" s="7" t="n"/>
       <c r="G35" s="7" t="n"/>
       <c r="H35" s="7" t="n"/>
     </row>
@@ -1116,13 +1116,13 @@
       <c r="A36" s="6" t="n">
         <v>29</v>
       </c>
-      <c r="B36" s="7" t="inlineStr">
-        <is>
-          <t>Jeremiyah Love</t>
-        </is>
-      </c>
+      <c r="B36" s="7" t="n"/>
       <c r="C36" s="7" t="n"/>
-      <c r="D36" s="7" t="n"/>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>Rashee Rice</t>
+        </is>
+      </c>
       <c r="E36" s="7" t="n"/>
       <c r="F36" s="7" t="n"/>
       <c r="G36" s="7" t="n"/>
@@ -1130,15 +1130,15 @@
     </row>
     <row r="37">
       <c r="A37" s="6" t="n">
-        <v>29</v>
-      </c>
-      <c r="B37" s="7" t="n"/>
+        <v>28</v>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Omarion Hampton</t>
+        </is>
+      </c>
       <c r="C37" s="7" t="n"/>
-      <c r="D37" s="7" t="inlineStr">
-        <is>
-          <t>Rashee Rice</t>
-        </is>
-      </c>
+      <c r="D37" s="7" t="n"/>
       <c r="E37" s="7" t="n"/>
       <c r="F37" s="7" t="n"/>
       <c r="G37" s="7" t="n"/>
@@ -1146,13 +1146,13 @@
     </row>
     <row r="38">
       <c r="A38" s="6" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B38" s="7" t="n"/>
       <c r="C38" s="7" t="n"/>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>Zay Flowers</t>
+          <t>Davante Adams</t>
         </is>
       </c>
       <c r="E38" s="7" t="n"/>
@@ -1168,7 +1168,7 @@
       <c r="C39" s="7" t="n"/>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>Davante Adams</t>
+          <t>Zay Flowers</t>
         </is>
       </c>
       <c r="E39" s="7" t="n"/>
@@ -1178,7 +1178,7 @@
     </row>
     <row r="40">
       <c r="A40" s="6" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B40" s="7" t="n"/>
       <c r="C40" s="7" t="n"/>
@@ -1242,7 +1242,7 @@
     </row>
     <row r="44">
       <c r="A44" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B44" s="7" t="n"/>
       <c r="C44" s="7" t="n"/>
@@ -1260,17 +1260,17 @@
       <c r="A45" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="B45" s="7" t="n"/>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Jaylen Warren</t>
+        </is>
+      </c>
       <c r="C45" s="7" t="n"/>
       <c r="D45" s="7" t="n"/>
       <c r="E45" s="7" t="n"/>
       <c r="F45" s="7" t="n"/>
       <c r="G45" s="7" t="n"/>
-      <c r="H45" s="7" t="inlineStr">
-        <is>
-          <t>Lamar Jackson</t>
-        </is>
-      </c>
+      <c r="H45" s="7" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="6" t="n">
@@ -1292,13 +1292,13 @@
       <c r="A47" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="B47" s="7" t="inlineStr">
-        <is>
-          <t>Jaylen Warren</t>
-        </is>
-      </c>
+      <c r="B47" s="7" t="n"/>
       <c r="C47" s="7" t="n"/>
-      <c r="D47" s="7" t="n"/>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>Jaylen Waddle</t>
+        </is>
+      </c>
       <c r="E47" s="7" t="n"/>
       <c r="F47" s="7" t="n"/>
       <c r="G47" s="7" t="n"/>
@@ -1306,31 +1306,31 @@
     </row>
     <row r="48">
       <c r="A48" s="6" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B48" s="7" t="n"/>
       <c r="C48" s="7" t="n"/>
-      <c r="D48" s="7" t="inlineStr">
-        <is>
-          <t>Jaylen Waddle</t>
-        </is>
-      </c>
+      <c r="D48" s="7" t="n"/>
       <c r="E48" s="7" t="n"/>
       <c r="F48" s="7" t="n"/>
       <c r="G48" s="7" t="n"/>
-      <c r="H48" s="7" t="n"/>
+      <c r="H48" s="7" t="inlineStr">
+        <is>
+          <t>Lamar Jackson</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="B49" s="7" t="n"/>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Aaron Jones Sr.</t>
+        </is>
+      </c>
       <c r="C49" s="7" t="n"/>
-      <c r="D49" s="7" t="inlineStr">
-        <is>
-          <t>Ladd McConkey</t>
-        </is>
-      </c>
+      <c r="D49" s="7" t="n"/>
       <c r="E49" s="7" t="n"/>
       <c r="F49" s="7" t="n"/>
       <c r="G49" s="7" t="n"/>
@@ -1342,7 +1342,7 @@
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>Aaron Jones Sr.</t>
+          <t>Quinshon Judkins</t>
         </is>
       </c>
       <c r="C50" s="7" t="n"/>
@@ -1370,15 +1370,15 @@
     </row>
     <row r="52">
       <c r="A52" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="B52" s="7" t="inlineStr">
-        <is>
-          <t>Quinshon Judkins</t>
-        </is>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="B52" s="7" t="n"/>
       <c r="C52" s="7" t="n"/>
-      <c r="D52" s="7" t="n"/>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>Ladd McConkey</t>
+        </is>
+      </c>
       <c r="E52" s="7" t="n"/>
       <c r="F52" s="7" t="n"/>
       <c r="G52" s="7" t="n"/>
@@ -1386,15 +1386,15 @@
     </row>
     <row r="53">
       <c r="A53" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="B53" s="7" t="n"/>
+        <v>18</v>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>David Montgomery</t>
+        </is>
+      </c>
       <c r="C53" s="7" t="n"/>
-      <c r="D53" s="7" t="inlineStr">
-        <is>
-          <t>Emeka Egbuka</t>
-        </is>
-      </c>
+      <c r="D53" s="7" t="n"/>
       <c r="E53" s="7" t="n"/>
       <c r="F53" s="7" t="n"/>
       <c r="G53" s="7" t="n"/>
@@ -1402,15 +1402,15 @@
     </row>
     <row r="54">
       <c r="A54" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="B54" s="7" t="inlineStr">
-        <is>
-          <t>Bhayshul Tuten</t>
-        </is>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="B54" s="7" t="n"/>
       <c r="C54" s="7" t="n"/>
-      <c r="D54" s="7" t="n"/>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>Christian Watson</t>
+        </is>
+      </c>
       <c r="E54" s="7" t="n"/>
       <c r="F54" s="7" t="n"/>
       <c r="G54" s="7" t="n"/>
@@ -1418,11 +1418,11 @@
     </row>
     <row r="55">
       <c r="A55" s="6" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>David Montgomery</t>
+          <t>Chuba Hubbard</t>
         </is>
       </c>
       <c r="C55" s="7" t="n"/>
@@ -1434,15 +1434,15 @@
     </row>
     <row r="56">
       <c r="A56" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="B56" s="7" t="inlineStr">
-        <is>
-          <t>Jadarian Price</t>
-        </is>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="B56" s="7" t="n"/>
       <c r="C56" s="7" t="n"/>
-      <c r="D56" s="7" t="n"/>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>Emeka Egbuka</t>
+        </is>
+      </c>
       <c r="E56" s="7" t="n"/>
       <c r="F56" s="7" t="n"/>
       <c r="G56" s="7" t="n"/>
@@ -1450,17 +1450,17 @@
     </row>
     <row r="57">
       <c r="A57" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="B57" s="7" t="inlineStr">
-        <is>
-          <t>Chuba Hubbard</t>
-        </is>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="B57" s="7" t="n"/>
       <c r="C57" s="7" t="n"/>
       <c r="D57" s="7" t="n"/>
       <c r="E57" s="7" t="n"/>
-      <c r="F57" s="7" t="n"/>
+      <c r="F57" s="7" t="inlineStr">
+        <is>
+          <t>Tyler Warren</t>
+        </is>
+      </c>
       <c r="G57" s="7" t="n"/>
       <c r="H57" s="7" t="n"/>
     </row>
@@ -1472,7 +1472,7 @@
       <c r="C58" s="7" t="n"/>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>Christian Watson</t>
+          <t>Mike Evans</t>
         </is>
       </c>
       <c r="E58" s="7" t="n"/>
@@ -1482,15 +1482,15 @@
     </row>
     <row r="59">
       <c r="A59" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="B59" s="7" t="inlineStr">
-        <is>
-          <t>MarShawn Lloyd</t>
-        </is>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="B59" s="7" t="n"/>
       <c r="C59" s="7" t="n"/>
-      <c r="D59" s="7" t="n"/>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>DJ Moore</t>
+        </is>
+      </c>
       <c r="E59" s="7" t="n"/>
       <c r="F59" s="7" t="n"/>
       <c r="G59" s="7" t="n"/>
@@ -1498,13 +1498,13 @@
     </row>
     <row r="60">
       <c r="A60" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B60" s="7" t="n"/>
       <c r="C60" s="7" t="n"/>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>Luther Burden III</t>
+          <t>Terry McLaurin</t>
         </is>
       </c>
       <c r="E60" s="7" t="n"/>
@@ -1514,27 +1514,27 @@
     </row>
     <row r="61">
       <c r="A61" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="B61" s="7" t="n"/>
+        <v>13</v>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>Bhayshul Tuten</t>
+        </is>
+      </c>
       <c r="C61" s="7" t="n"/>
       <c r="D61" s="7" t="n"/>
       <c r="E61" s="7" t="n"/>
-      <c r="F61" s="7" t="inlineStr">
-        <is>
-          <t>Tyler Warren</t>
-        </is>
-      </c>
+      <c r="F61" s="7" t="n"/>
       <c r="G61" s="7" t="n"/>
       <c r="H61" s="7" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>Rhamondre Stevenson</t>
+          <t>Jadarian Price</t>
         </is>
       </c>
       <c r="C62" s="7" t="n"/>
@@ -1546,13 +1546,13 @@
     </row>
     <row r="63">
       <c r="A63" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B63" s="7" t="n"/>
       <c r="C63" s="7" t="n"/>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>Mike Evans</t>
+          <t>Luther Burden III</t>
         </is>
       </c>
       <c r="E63" s="7" t="n"/>
@@ -1562,13 +1562,13 @@
     </row>
     <row r="64">
       <c r="A64" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B64" s="7" t="n"/>
       <c r="C64" s="7" t="n"/>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>DJ Moore</t>
+          <t>Matthew Golden</t>
         </is>
       </c>
       <c r="E64" s="7" t="n"/>
@@ -1580,27 +1580,27 @@
       <c r="A65" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="B65" s="7" t="n"/>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>Rhamondre Stevenson</t>
+        </is>
+      </c>
       <c r="C65" s="7" t="n"/>
       <c r="D65" s="7" t="n"/>
       <c r="E65" s="7" t="n"/>
       <c r="F65" s="7" t="n"/>
       <c r="G65" s="7" t="n"/>
-      <c r="H65" s="7" t="inlineStr">
-        <is>
-          <t>Joe Burrow</t>
-        </is>
-      </c>
+      <c r="H65" s="7" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B66" s="7" t="n"/>
       <c r="C66" s="7" t="n"/>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>Terry McLaurin</t>
+          <t>Michael Wilson</t>
         </is>
       </c>
       <c r="E66" s="7" t="n"/>
@@ -1610,31 +1610,31 @@
     </row>
     <row r="67">
       <c r="A67" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="B67" s="7" t="n"/>
+        <v>10</v>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>MarShawn Lloyd</t>
+        </is>
+      </c>
       <c r="C67" s="7" t="n"/>
       <c r="D67" s="7" t="n"/>
       <c r="E67" s="7" t="n"/>
       <c r="F67" s="7" t="n"/>
       <c r="G67" s="7" t="n"/>
-      <c r="H67" s="7" t="inlineStr">
-        <is>
-          <t>Drake Maye</t>
-        </is>
-      </c>
+      <c r="H67" s="7" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="B68" s="7" t="inlineStr">
-        <is>
-          <t>TreVeyon Henderson</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="B68" s="7" t="n"/>
       <c r="C68" s="7" t="n"/>
-      <c r="D68" s="7" t="n"/>
+      <c r="D68" s="7" t="inlineStr">
+        <is>
+          <t>Jameson Williams</t>
+        </is>
+      </c>
       <c r="E68" s="7" t="n"/>
       <c r="F68" s="7" t="n"/>
       <c r="G68" s="7" t="n"/>
@@ -1642,13 +1642,13 @@
     </row>
     <row r="69">
       <c r="A69" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B69" s="7" t="n"/>
       <c r="C69" s="7" t="n"/>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>Matthew Golden</t>
+          <t>De'Zhaun Stribling</t>
         </is>
       </c>
       <c r="E69" s="7" t="n"/>
@@ -1658,19 +1658,19 @@
     </row>
     <row r="70">
       <c r="A70" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B70" s="7" t="n"/>
       <c r="C70" s="7" t="n"/>
       <c r="D70" s="7" t="n"/>
       <c r="E70" s="7" t="n"/>
-      <c r="F70" s="7" t="inlineStr">
-        <is>
-          <t>Colston Loveland</t>
-        </is>
-      </c>
+      <c r="F70" s="7" t="n"/>
       <c r="G70" s="7" t="n"/>
-      <c r="H70" s="7" t="n"/>
+      <c r="H70" s="7" t="inlineStr">
+        <is>
+          <t>Joe Burrow</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="6" t="n">
@@ -1678,75 +1678,75 @@
       </c>
       <c r="B71" s="7" t="n"/>
       <c r="C71" s="7" t="n"/>
-      <c r="D71" s="7" t="n"/>
+      <c r="D71" s="7" t="inlineStr">
+        <is>
+          <t>Carnell Tate</t>
+        </is>
+      </c>
       <c r="E71" s="7" t="n"/>
-      <c r="F71" s="7" t="inlineStr">
-        <is>
-          <t>Isaiah Likely</t>
-        </is>
-      </c>
+      <c r="F71" s="7" t="n"/>
       <c r="G71" s="7" t="n"/>
       <c r="H71" s="7" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B72" s="7" t="n"/>
       <c r="C72" s="7" t="n"/>
-      <c r="D72" s="7" t="n"/>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>Alec Pierce</t>
+        </is>
+      </c>
       <c r="E72" s="7" t="n"/>
-      <c r="F72" s="7" t="inlineStr">
-        <is>
-          <t>George Kittle</t>
-        </is>
-      </c>
+      <c r="F72" s="7" t="n"/>
       <c r="G72" s="7" t="n"/>
       <c r="H72" s="7" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B73" s="7" t="n"/>
       <c r="C73" s="7" t="n"/>
-      <c r="D73" s="7" t="n"/>
+      <c r="D73" s="7" t="inlineStr">
+        <is>
+          <t>Stefon Diggs</t>
+        </is>
+      </c>
       <c r="E73" s="7" t="n"/>
       <c r="F73" s="7" t="n"/>
       <c r="G73" s="7" t="n"/>
-      <c r="H73" s="7" t="inlineStr">
-        <is>
-          <t>Jalen Hurts</t>
-        </is>
-      </c>
+      <c r="H73" s="7" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B74" s="7" t="inlineStr">
-        <is>
-          <t>Tony Pollard</t>
-        </is>
-      </c>
+      <c r="B74" s="7" t="n"/>
       <c r="C74" s="7" t="n"/>
       <c r="D74" s="7" t="n"/>
       <c r="E74" s="7" t="n"/>
       <c r="F74" s="7" t="n"/>
       <c r="G74" s="7" t="n"/>
-      <c r="H74" s="7" t="n"/>
+      <c r="H74" s="7" t="inlineStr">
+        <is>
+          <t>Drake Maye</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="B75" s="7" t="n"/>
+        <v>6</v>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>TreVeyon Henderson</t>
+        </is>
+      </c>
       <c r="C75" s="7" t="n"/>
-      <c r="D75" s="7" t="inlineStr">
-        <is>
-          <t>Rome Odunze</t>
-        </is>
-      </c>
+      <c r="D75" s="7" t="n"/>
       <c r="E75" s="7" t="n"/>
       <c r="F75" s="7" t="n"/>
       <c r="G75" s="7" t="n"/>
@@ -1754,13 +1754,13 @@
     </row>
     <row r="76">
       <c r="A76" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B76" s="7" t="n"/>
       <c r="C76" s="7" t="n"/>
       <c r="D76" s="7" t="inlineStr">
         <is>
-          <t>Jameson Williams</t>
+          <t>KC Concepcion</t>
         </is>
       </c>
       <c r="E76" s="7" t="n"/>
@@ -1770,33 +1770,33 @@
     </row>
     <row r="77">
       <c r="A77" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B77" s="7" t="n"/>
       <c r="C77" s="7" t="n"/>
-      <c r="D77" s="7" t="inlineStr">
-        <is>
-          <t>Michael Wilson</t>
-        </is>
-      </c>
+      <c r="D77" s="7" t="n"/>
       <c r="E77" s="7" t="n"/>
-      <c r="F77" s="7" t="n"/>
+      <c r="F77" s="7" t="inlineStr">
+        <is>
+          <t>Colston Loveland</t>
+        </is>
+      </c>
       <c r="G77" s="7" t="n"/>
       <c r="H77" s="7" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B78" s="7" t="n"/>
       <c r="C78" s="7" t="n"/>
-      <c r="D78" s="7" t="inlineStr">
-        <is>
-          <t>Marvin Harrison Jr.</t>
-        </is>
-      </c>
+      <c r="D78" s="7" t="n"/>
       <c r="E78" s="7" t="n"/>
-      <c r="F78" s="7" t="n"/>
+      <c r="F78" s="7" t="inlineStr">
+        <is>
+          <t>Isaiah Likely</t>
+        </is>
+      </c>
       <c r="G78" s="7" t="n"/>
       <c r="H78" s="7" t="n"/>
     </row>
@@ -1804,15 +1804,15 @@
       <c r="A79" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B79" s="7" t="inlineStr">
-        <is>
-          <t>Josh Jacobs</t>
-        </is>
-      </c>
+      <c r="B79" s="7" t="n"/>
       <c r="C79" s="7" t="n"/>
       <c r="D79" s="7" t="n"/>
       <c r="E79" s="7" t="n"/>
-      <c r="F79" s="7" t="n"/>
+      <c r="F79" s="7" t="inlineStr">
+        <is>
+          <t>George Kittle</t>
+        </is>
+      </c>
       <c r="G79" s="7" t="n"/>
       <c r="H79" s="7" t="n"/>
     </row>
@@ -1822,31 +1822,31 @@
       </c>
       <c r="B80" s="7" t="n"/>
       <c r="C80" s="7" t="n"/>
-      <c r="D80" s="7" t="inlineStr">
-        <is>
-          <t>De'Zhaun Stribling</t>
-        </is>
-      </c>
+      <c r="D80" s="7" t="n"/>
       <c r="E80" s="7" t="n"/>
       <c r="F80" s="7" t="n"/>
       <c r="G80" s="7" t="n"/>
-      <c r="H80" s="7" t="n"/>
+      <c r="H80" s="7" t="inlineStr">
+        <is>
+          <t>Jalen Hurts</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B81" s="7" t="n"/>
+        <v>5</v>
+      </c>
+      <c r="B81" s="7" t="inlineStr">
+        <is>
+          <t>Tony Pollard</t>
+        </is>
+      </c>
       <c r="C81" s="7" t="n"/>
       <c r="D81" s="7" t="n"/>
       <c r="E81" s="7" t="n"/>
       <c r="F81" s="7" t="n"/>
       <c r="G81" s="7" t="n"/>
-      <c r="H81" s="7" t="inlineStr">
-        <is>
-          <t>Jayden Daniels</t>
-        </is>
-      </c>
+      <c r="H81" s="7" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="6" t="n">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="B82" s="7" t="inlineStr">
         <is>
-          <t>Jacory Croskey-Merritt</t>
+          <t>Kenny Gainwell</t>
         </is>
       </c>
       <c r="C82" s="7" t="n"/>
@@ -1868,13 +1868,13 @@
       <c r="A83" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B83" s="7" t="inlineStr">
-        <is>
-          <t>Kenny Gainwell</t>
-        </is>
-      </c>
+      <c r="B83" s="7" t="n"/>
       <c r="C83" s="7" t="n"/>
-      <c r="D83" s="7" t="n"/>
+      <c r="D83" s="7" t="inlineStr">
+        <is>
+          <t>Rome Odunze</t>
+        </is>
+      </c>
       <c r="E83" s="7" t="n"/>
       <c r="F83" s="7" t="n"/>
       <c r="G83" s="7" t="n"/>
@@ -1886,27 +1886,27 @@
       </c>
       <c r="B84" s="7" t="n"/>
       <c r="C84" s="7" t="n"/>
-      <c r="D84" s="7" t="n"/>
+      <c r="D84" s="7" t="inlineStr">
+        <is>
+          <t>Jayden Reed</t>
+        </is>
+      </c>
       <c r="E84" s="7" t="n"/>
       <c r="F84" s="7" t="n"/>
       <c r="G84" s="7" t="n"/>
-      <c r="H84" s="7" t="inlineStr">
-        <is>
-          <t>Justin Herbert</t>
-        </is>
-      </c>
+      <c r="H84" s="7" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B85" s="7" t="inlineStr">
-        <is>
-          <t>Jordan Mason</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="B85" s="7" t="n"/>
       <c r="C85" s="7" t="n"/>
-      <c r="D85" s="7" t="n"/>
+      <c r="D85" s="7" t="inlineStr">
+        <is>
+          <t>Jordyn Tyson</t>
+        </is>
+      </c>
       <c r="E85" s="7" t="n"/>
       <c r="F85" s="7" t="n"/>
       <c r="G85" s="7" t="n"/>
@@ -1916,13 +1916,13 @@
       <c r="A86" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B86" s="7" t="n"/>
+      <c r="B86" s="7" t="inlineStr">
+        <is>
+          <t>Josh Jacobs</t>
+        </is>
+      </c>
       <c r="C86" s="7" t="n"/>
-      <c r="D86" s="7" t="inlineStr">
-        <is>
-          <t>Carnell Tate</t>
-        </is>
-      </c>
+      <c r="D86" s="7" t="n"/>
       <c r="E86" s="7" t="n"/>
       <c r="F86" s="7" t="n"/>
       <c r="G86" s="7" t="n"/>
@@ -1936,7 +1936,7 @@
       <c r="C87" s="7" t="n"/>
       <c r="D87" s="7" t="inlineStr">
         <is>
-          <t>Alec Pierce</t>
+          <t>DK Metcalf</t>
         </is>
       </c>
       <c r="E87" s="7" t="n"/>
@@ -1946,31 +1946,31 @@
     </row>
     <row r="88">
       <c r="A88" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B88" s="7" t="inlineStr">
-        <is>
-          <t>Rachaad White</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="B88" s="7" t="n"/>
       <c r="C88" s="7" t="n"/>
       <c r="D88" s="7" t="n"/>
       <c r="E88" s="7" t="n"/>
       <c r="F88" s="7" t="n"/>
       <c r="G88" s="7" t="n"/>
-      <c r="H88" s="7" t="n"/>
+      <c r="H88" s="7" t="inlineStr">
+        <is>
+          <t>Jayden Daniels</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B89" s="7" t="n"/>
+      <c r="B89" s="7" t="inlineStr">
+        <is>
+          <t>Jacory Croskey-Merritt</t>
+        </is>
+      </c>
       <c r="C89" s="7" t="n"/>
-      <c r="D89" s="7" t="inlineStr">
-        <is>
-          <t>Brian Thomas Jr.</t>
-        </is>
-      </c>
+      <c r="D89" s="7" t="n"/>
       <c r="E89" s="7" t="n"/>
       <c r="F89" s="7" t="n"/>
       <c r="G89" s="7" t="n"/>
@@ -1980,13 +1980,13 @@
       <c r="A90" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B90" s="7" t="n"/>
+      <c r="B90" s="7" t="inlineStr">
+        <is>
+          <t>Rachaad White</t>
+        </is>
+      </c>
       <c r="C90" s="7" t="n"/>
-      <c r="D90" s="7" t="inlineStr">
-        <is>
-          <t>KC Concepcion</t>
-        </is>
-      </c>
+      <c r="D90" s="7" t="n"/>
       <c r="E90" s="7" t="n"/>
       <c r="F90" s="7" t="n"/>
       <c r="G90" s="7" t="n"/>
@@ -1998,27 +1998,27 @@
       </c>
       <c r="B91" s="7" t="n"/>
       <c r="C91" s="7" t="n"/>
-      <c r="D91" s="7" t="inlineStr">
-        <is>
-          <t>Quentin Johnston</t>
-        </is>
-      </c>
+      <c r="D91" s="7" t="n"/>
       <c r="E91" s="7" t="n"/>
       <c r="F91" s="7" t="n"/>
       <c r="G91" s="7" t="n"/>
-      <c r="H91" s="7" t="n"/>
+      <c r="H91" s="7" t="inlineStr">
+        <is>
+          <t>Justin Herbert</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B92" s="7" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="B92" s="7" t="inlineStr">
+        <is>
+          <t>Jordan Mason</t>
+        </is>
+      </c>
       <c r="C92" s="7" t="n"/>
-      <c r="D92" s="7" t="inlineStr">
-        <is>
-          <t>Stefon Diggs</t>
-        </is>
-      </c>
+      <c r="D92" s="7" t="n"/>
       <c r="E92" s="7" t="n"/>
       <c r="F92" s="7" t="n"/>
       <c r="G92" s="7" t="n"/>
@@ -2026,43 +2026,43 @@
     </row>
     <row r="93">
       <c r="A93" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B93" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="B93" s="7" t="inlineStr">
+        <is>
+          <t>J.K. Dobbins</t>
+        </is>
+      </c>
       <c r="C93" s="7" t="n"/>
       <c r="D93" s="7" t="n"/>
       <c r="E93" s="7" t="n"/>
-      <c r="F93" s="7" t="inlineStr">
-        <is>
-          <t>Tucker Kraft</t>
-        </is>
-      </c>
+      <c r="F93" s="7" t="n"/>
       <c r="G93" s="7" t="n"/>
       <c r="H93" s="7" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B94" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="B94" s="7" t="inlineStr">
+        <is>
+          <t>Jonathon Brooks</t>
+        </is>
+      </c>
       <c r="C94" s="7" t="n"/>
       <c r="D94" s="7" t="n"/>
       <c r="E94" s="7" t="n"/>
-      <c r="F94" s="7" t="inlineStr">
-        <is>
-          <t>Harold Fannin Jr.</t>
-        </is>
-      </c>
+      <c r="F94" s="7" t="n"/>
       <c r="G94" s="7" t="n"/>
       <c r="H94" s="7" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B95" s="7" t="inlineStr">
         <is>
-          <t>J.K. Dobbins</t>
+          <t>Mike Washington Jr.</t>
         </is>
       </c>
       <c r="C95" s="7" t="n"/>
@@ -2074,11 +2074,11 @@
     </row>
     <row r="96">
       <c r="A96" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B96" s="7" t="inlineStr">
         <is>
-          <t>Jonathon Brooks</t>
+          <t>Rico Dowdle</t>
         </is>
       </c>
       <c r="C96" s="7" t="n"/>
@@ -2090,11 +2090,11 @@
     </row>
     <row r="97">
       <c r="A97" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B97" s="7" t="inlineStr">
         <is>
-          <t>Mike Washington Jr.</t>
+          <t>Blake Corum</t>
         </is>
       </c>
       <c r="C97" s="7" t="n"/>
@@ -2106,11 +2106,11 @@
     </row>
     <row r="98">
       <c r="A98" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B98" s="7" t="inlineStr">
         <is>
-          <t>Rico Dowdle</t>
+          <t>Woody Marks</t>
         </is>
       </c>
       <c r="C98" s="7" t="n"/>
@@ -2122,13 +2122,13 @@
     </row>
     <row r="99">
       <c r="A99" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B99" s="7" t="n"/>
       <c r="C99" s="7" t="n"/>
       <c r="D99" s="7" t="inlineStr">
         <is>
-          <t>Chris Godwin Jr.</t>
+          <t>Brian Thomas Jr.</t>
         </is>
       </c>
       <c r="E99" s="7" t="n"/>
@@ -2138,13 +2138,13 @@
     </row>
     <row r="100">
       <c r="A100" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B100" s="7" t="n"/>
       <c r="C100" s="7" t="n"/>
       <c r="D100" s="7" t="inlineStr">
         <is>
-          <t>Jayden Reed</t>
+          <t>Marvin Harrison Jr.</t>
         </is>
       </c>
       <c r="E100" s="7" t="n"/>
@@ -2154,13 +2154,13 @@
     </row>
     <row r="101">
       <c r="A101" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B101" s="7" t="n"/>
       <c r="C101" s="7" t="n"/>
       <c r="D101" s="7" t="inlineStr">
         <is>
-          <t>Jordyn Tyson</t>
+          <t>Quentin Johnston</t>
         </is>
       </c>
       <c r="E101" s="7" t="n"/>
@@ -2170,31 +2170,31 @@
     </row>
     <row r="102">
       <c r="A102" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B102" s="7" t="n"/>
       <c r="C102" s="7" t="n"/>
-      <c r="D102" s="7" t="n"/>
+      <c r="D102" s="7" t="inlineStr">
+        <is>
+          <t>Chris Godwin Jr.</t>
+        </is>
+      </c>
       <c r="E102" s="7" t="n"/>
       <c r="F102" s="7" t="n"/>
       <c r="G102" s="7" t="n"/>
-      <c r="H102" s="7" t="inlineStr">
-        <is>
-          <t>Trevor Lawrence</t>
-        </is>
-      </c>
+      <c r="H102" s="7" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B103" s="7" t="inlineStr">
-        <is>
-          <t>Blake Corum</t>
-        </is>
-      </c>
+      <c r="B103" s="7" t="n"/>
       <c r="C103" s="7" t="n"/>
-      <c r="D103" s="7" t="n"/>
+      <c r="D103" s="7" t="inlineStr">
+        <is>
+          <t>Ja'Kobi Lane</t>
+        </is>
+      </c>
       <c r="E103" s="7" t="n"/>
       <c r="F103" s="7" t="n"/>
       <c r="G103" s="7" t="n"/>
@@ -2204,15 +2204,15 @@
       <c r="A104" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B104" s="7" t="inlineStr">
-        <is>
-          <t>Woody Marks</t>
-        </is>
-      </c>
+      <c r="B104" s="7" t="n"/>
       <c r="C104" s="7" t="n"/>
       <c r="D104" s="7" t="n"/>
       <c r="E104" s="7" t="n"/>
-      <c r="F104" s="7" t="n"/>
+      <c r="F104" s="7" t="inlineStr">
+        <is>
+          <t>Tucker Kraft</t>
+        </is>
+      </c>
       <c r="G104" s="7" t="n"/>
       <c r="H104" s="7" t="n"/>
     </row>
@@ -2222,13 +2222,13 @@
       </c>
       <c r="B105" s="7" t="n"/>
       <c r="C105" s="7" t="n"/>
-      <c r="D105" s="7" t="inlineStr">
-        <is>
-          <t>DK Metcalf</t>
-        </is>
-      </c>
+      <c r="D105" s="7" t="n"/>
       <c r="E105" s="7" t="n"/>
-      <c r="F105" s="7" t="n"/>
+      <c r="F105" s="7" t="inlineStr">
+        <is>
+          <t>Harold Fannin Jr.</t>
+        </is>
+      </c>
       <c r="G105" s="7" t="n"/>
       <c r="H105" s="7" t="n"/>
     </row>
@@ -2238,15 +2238,15 @@
       </c>
       <c r="B106" s="7" t="n"/>
       <c r="C106" s="7" t="n"/>
-      <c r="D106" s="7" t="inlineStr">
-        <is>
-          <t>Ja'Kobi Lane</t>
-        </is>
-      </c>
+      <c r="D106" s="7" t="n"/>
       <c r="E106" s="7" t="n"/>
       <c r="F106" s="7" t="n"/>
       <c r="G106" s="7" t="n"/>
-      <c r="H106" s="7" t="n"/>
+      <c r="H106" s="7" t="inlineStr">
+        <is>
+          <t>Trevor Lawrence</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="6" t="n">
@@ -2401,14 +2401,14 @@
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   receptions/game = BettingPros consensus receptions line from the 2026 week 1 props; players with no line use the mean line of position peers within 10 value points.</t>
+          <t xml:space="preserve">   receptions/game = BettingPros consensus receptions line from the 2026 week 4 props; players with no line use the mean line of position peers within 10 value points.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Replacement level = average line of baseline players valued 5 or less at the position: RB 1.8, WR 3.3, TE 4.5, QB 0.0.</t>
+          <t xml:space="preserve">   Replacement level = average line of baseline players valued 5 or less at the position: RB 1.8, WR 2.9, TE 4.5, QB 0.0.</t>
         </is>
       </c>
     </row>
@@ -2435,7 +2435,7 @@
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>Largest moves vs. the baseline in this file: Puka Nacua 65-&gt;70, Ja'Marr Chase 55-&gt;60, Jaxon Smith-Njigba 56-&gt;60, Amon-Ra St. Brown 52-&gt;56, CeeDee Lamb 44-&gt;48, Chris Olave 41-&gt;45, Bijan Robinson 70-&gt;73, Jahmyr Gibbs 61-&gt;64</t>
+          <t>Largest moves vs. the baseline in this file: Puka Nacua 65-&gt;71, Jaxon Smith-Njigba 56-&gt;62, Ja'Marr Chase 55-&gt;59, Amon-Ra St. Brown 52-&gt;56, James Cook III 49-&gt;45, Derrick Henry 55-&gt;51, Omarion Hampton 32-&gt;28, Chris Olave 41-&gt;45</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Trade values: make the weekly re-seed follow the projections
Within each position the projected players are ranked by median and mapped
onto their own group's sorted sheet values (term A) blended with their
share of the group's points above replacement (term C); both are monotone
in the projection, so the published order tracks the medians (Spearman
~0.97 for RB/WR vs ~0.78 before) and the sheet only tempers the gaps.
Weight raised to 0.8. Players without a line use last week's median
(dump_projections.mjs now emits the previous week); a position under 60%
coverage keeps the sheet values. Ranking within the projected group keeps
stars from funding cheap breakouts, and the league-size step now anchors
on the re-seeded top so the #1 player is exactly 65/70/75. JSON players
now carry sheetValue, projection and projectionWeek.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TradeValueSheets/TradeValues_FullPPR_10team.xlsx
+++ b/TradeValueSheets/TradeValues_FullPPR_10team.xlsx
@@ -606,7 +606,7 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Bijan Robinson</t>
+          <t>Jahmyr Gibbs</t>
         </is>
       </c>
       <c r="C4" s="7" t="n"/>
@@ -618,13 +618,13 @@
     </row>
     <row r="5">
       <c r="A5" s="6" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B5" s="7" t="n"/>
       <c r="C5" s="7" t="n"/>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Puka Nacua</t>
+          <t>Jaxon Smith-Njigba</t>
         </is>
       </c>
       <c r="E5" s="7" t="n"/>
@@ -638,7 +638,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Jahmyr Gibbs</t>
+          <t>Bijan Robinson</t>
         </is>
       </c>
       <c r="C6" s="7" t="n"/>
@@ -650,15 +650,15 @@
     </row>
     <row r="7">
       <c r="A7" s="6" t="n">
-        <v>62</v>
-      </c>
-      <c r="B7" s="7" t="n"/>
+        <v>60</v>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Christian McCaffrey</t>
+        </is>
+      </c>
       <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>Jaxon Smith-Njigba</t>
-        </is>
-      </c>
+      <c r="D7" s="7" t="n"/>
       <c r="E7" s="7" t="n"/>
       <c r="F7" s="7" t="n"/>
       <c r="G7" s="7" t="n"/>
@@ -666,15 +666,15 @@
     </row>
     <row r="8">
       <c r="A8" s="6" t="n">
-        <v>61</v>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Kenneth Walker III</t>
-        </is>
-      </c>
+        <v>59</v>
+      </c>
+      <c r="B8" s="7" t="n"/>
       <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Ja'Marr Chase</t>
+        </is>
+      </c>
       <c r="E8" s="7" t="n"/>
       <c r="F8" s="7" t="n"/>
       <c r="G8" s="7" t="n"/>
@@ -682,15 +682,15 @@
     </row>
     <row r="9">
       <c r="A9" s="6" t="n">
-        <v>59</v>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Christian McCaffrey</t>
-        </is>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="B9" s="7" t="n"/>
       <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Amon-Ra St. Brown</t>
+        </is>
+      </c>
       <c r="E9" s="7" t="n"/>
       <c r="F9" s="7" t="n"/>
       <c r="G9" s="7" t="n"/>
@@ -698,13 +698,13 @@
     </row>
     <row r="10">
       <c r="A10" s="6" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B10" s="7" t="n"/>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Ja'Marr Chase</t>
+          <t>Puka Nacua</t>
         </is>
       </c>
       <c r="E10" s="7" t="n"/>
@@ -714,11 +714,11 @@
     </row>
     <row r="11">
       <c r="A11" s="6" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Saquon Barkley</t>
+          <t>Jonathan Taylor</t>
         </is>
       </c>
       <c r="C11" s="7" t="n"/>
@@ -730,11 +730,11 @@
     </row>
     <row r="12">
       <c r="A12" s="6" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Ashton Jeanty</t>
+          <t>Kenneth Walker III</t>
         </is>
       </c>
       <c r="C12" s="7" t="n"/>
@@ -746,13 +746,13 @@
     </row>
     <row r="13">
       <c r="A13" s="6" t="n">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B13" s="7" t="n"/>
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Justin Jefferson</t>
+          <t>Chris Olave</t>
         </is>
       </c>
       <c r="E13" s="7" t="n"/>
@@ -762,13 +762,13 @@
     </row>
     <row r="14">
       <c r="A14" s="6" t="n">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="B14" s="7" t="n"/>
       <c r="C14" s="7" t="n"/>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Amon-Ra St. Brown</t>
+          <t>CeeDee Lamb</t>
         </is>
       </c>
       <c r="E14" s="7" t="n"/>
@@ -778,11 +778,11 @@
     </row>
     <row r="15">
       <c r="A15" s="6" t="n">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Jonathan Taylor</t>
+          <t>Derrick Henry</t>
         </is>
       </c>
       <c r="C15" s="7" t="n"/>
@@ -794,11 +794,11 @@
     </row>
     <row r="16">
       <c r="A16" s="6" t="n">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Derrick Henry</t>
+          <t>Ashton Jeanty</t>
         </is>
       </c>
       <c r="C16" s="7" t="n"/>
@@ -810,15 +810,15 @@
     </row>
     <row r="17">
       <c r="A17" s="6" t="n">
-        <v>47</v>
-      </c>
-      <c r="B17" s="7" t="n"/>
+        <v>43</v>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Chase Brown</t>
+        </is>
+      </c>
       <c r="C17" s="7" t="n"/>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>CeeDee Lamb</t>
-        </is>
-      </c>
+      <c r="D17" s="7" t="n"/>
       <c r="E17" s="7" t="n"/>
       <c r="F17" s="7" t="n"/>
       <c r="G17" s="7" t="n"/>
@@ -826,31 +826,31 @@
     </row>
     <row r="18">
       <c r="A18" s="6" t="n">
-        <v>45</v>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>James Cook III</t>
-        </is>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="B18" s="7" t="n"/>
       <c r="C18" s="7" t="n"/>
       <c r="D18" s="7" t="n"/>
       <c r="E18" s="7" t="n"/>
-      <c r="F18" s="7" t="n"/>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>Trey McBride</t>
+        </is>
+      </c>
       <c r="G18" s="7" t="n"/>
       <c r="H18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="n">
-        <v>45</v>
-      </c>
-      <c r="B19" s="7" t="n"/>
+        <v>41</v>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>James Cook III</t>
+        </is>
+      </c>
       <c r="C19" s="7" t="n"/>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>Chris Olave</t>
-        </is>
-      </c>
+      <c r="D19" s="7" t="n"/>
       <c r="E19" s="7" t="n"/>
       <c r="F19" s="7" t="n"/>
       <c r="G19" s="7" t="n"/>
@@ -858,15 +858,15 @@
     </row>
     <row r="20">
       <c r="A20" s="6" t="n">
-        <v>44</v>
-      </c>
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>Chase Brown</t>
-        </is>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="B20" s="7" t="n"/>
       <c r="C20" s="7" t="n"/>
-      <c r="D20" s="7" t="n"/>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Justin Jefferson</t>
+        </is>
+      </c>
       <c r="E20" s="7" t="n"/>
       <c r="F20" s="7" t="n"/>
       <c r="G20" s="7" t="n"/>
@@ -874,15 +874,15 @@
     </row>
     <row r="21">
       <c r="A21" s="6" t="n">
-        <v>44</v>
-      </c>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>De'Von Achane</t>
-        </is>
-      </c>
+        <v>38</v>
+      </c>
+      <c r="B21" s="7" t="n"/>
       <c r="C21" s="7" t="n"/>
-      <c r="D21" s="7" t="n"/>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Garrett Wilson</t>
+        </is>
+      </c>
       <c r="E21" s="7" t="n"/>
       <c r="F21" s="7" t="n"/>
       <c r="G21" s="7" t="n"/>
@@ -890,13 +890,13 @@
     </row>
     <row r="22">
       <c r="A22" s="6" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B22" s="7" t="n"/>
       <c r="C22" s="7" t="n"/>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>A.J. Brown</t>
+          <t>Davante Adams</t>
         </is>
       </c>
       <c r="E22" s="7" t="n"/>
@@ -906,15 +906,15 @@
     </row>
     <row r="23">
       <c r="A23" s="6" t="n">
-        <v>40</v>
-      </c>
-      <c r="B23" s="7" t="n"/>
+        <v>36</v>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>De'Von Achane</t>
+        </is>
+      </c>
       <c r="C23" s="7" t="n"/>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>Drake London</t>
-        </is>
-      </c>
+      <c r="D23" s="7" t="n"/>
       <c r="E23" s="7" t="n"/>
       <c r="F23" s="7" t="n"/>
       <c r="G23" s="7" t="n"/>
@@ -922,15 +922,15 @@
     </row>
     <row r="24">
       <c r="A24" s="6" t="n">
-        <v>38</v>
-      </c>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>Breece Hall</t>
-        </is>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="B24" s="7" t="n"/>
       <c r="C24" s="7" t="n"/>
-      <c r="D24" s="7" t="n"/>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Parker Washington</t>
+        </is>
+      </c>
       <c r="E24" s="7" t="n"/>
       <c r="F24" s="7" t="n"/>
       <c r="G24" s="7" t="n"/>
@@ -938,27 +938,27 @@
     </row>
     <row r="25">
       <c r="A25" s="6" t="n">
-        <v>38</v>
-      </c>
-      <c r="B25" s="7" t="n"/>
+        <v>31</v>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Breece Hall</t>
+        </is>
+      </c>
       <c r="C25" s="7" t="n"/>
       <c r="D25" s="7" t="n"/>
       <c r="E25" s="7" t="n"/>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>Brock Bowers</t>
-        </is>
-      </c>
+      <c r="F25" s="7" t="n"/>
       <c r="G25" s="7" t="n"/>
       <c r="H25" s="7" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Javonte Williams</t>
+          <t>Jaylen Warren</t>
         </is>
       </c>
       <c r="C26" s="7" t="n"/>
@@ -970,11 +970,11 @@
     </row>
     <row r="27">
       <c r="A27" s="6" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>D'Andre Swift</t>
+          <t>Aaron Jones Sr.</t>
         </is>
       </c>
       <c r="C27" s="7" t="n"/>
@@ -986,7 +986,7 @@
     </row>
     <row r="28">
       <c r="A28" s="6" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B28" s="7" t="n"/>
       <c r="C28" s="7" t="n"/>
@@ -1002,11 +1002,11 @@
     </row>
     <row r="29">
       <c r="A29" s="6" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Kyren Williams</t>
+          <t>D'Andre Swift</t>
         </is>
       </c>
       <c r="C29" s="7" t="n"/>
@@ -1018,47 +1018,47 @@
     </row>
     <row r="30">
       <c r="A30" s="6" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B30" s="7" t="n"/>
       <c r="C30" s="7" t="n"/>
       <c r="D30" s="7" t="n"/>
       <c r="E30" s="7" t="n"/>
-      <c r="F30" s="7" t="inlineStr">
-        <is>
-          <t>Trey McBride</t>
-        </is>
-      </c>
+      <c r="F30" s="7" t="n"/>
       <c r="G30" s="7" t="n"/>
-      <c r="H30" s="7" t="n"/>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>Josh Allen</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="n">
-        <v>32</v>
-      </c>
-      <c r="B31" s="7" t="n"/>
+        <v>29</v>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Cam Skattebo</t>
+        </is>
+      </c>
       <c r="C31" s="7" t="n"/>
       <c r="D31" s="7" t="n"/>
       <c r="E31" s="7" t="n"/>
       <c r="F31" s="7" t="n"/>
       <c r="G31" s="7" t="n"/>
-      <c r="H31" s="7" t="inlineStr">
-        <is>
-          <t>Josh Allen</t>
-        </is>
-      </c>
+      <c r="H31" s="7" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="6" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" s="7" t="n"/>
+        <v>28</v>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Javonte Williams</t>
+        </is>
+      </c>
       <c r="C32" s="7" t="n"/>
-      <c r="D32" s="7" t="inlineStr">
-        <is>
-          <t>George Pickens</t>
-        </is>
-      </c>
+      <c r="D32" s="7" t="n"/>
       <c r="E32" s="7" t="n"/>
       <c r="F32" s="7" t="n"/>
       <c r="G32" s="7" t="n"/>
@@ -1066,13 +1066,13 @@
     </row>
     <row r="33">
       <c r="A33" s="6" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B33" s="7" t="n"/>
       <c r="C33" s="7" t="n"/>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>Garrett Wilson</t>
+          <t>DeVonta Smith</t>
         </is>
       </c>
       <c r="E33" s="7" t="n"/>
@@ -1082,13 +1082,13 @@
     </row>
     <row r="34">
       <c r="A34" s="6" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B34" s="7" t="n"/>
       <c r="C34" s="7" t="n"/>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>DeVonta Smith</t>
+          <t>Drake London</t>
         </is>
       </c>
       <c r="E34" s="7" t="n"/>
@@ -1098,11 +1098,11 @@
     </row>
     <row r="35">
       <c r="A35" s="6" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>Jeremiyah Love</t>
+          <t>Saquon Barkley</t>
         </is>
       </c>
       <c r="C35" s="7" t="n"/>
@@ -1114,13 +1114,13 @@
     </row>
     <row r="36">
       <c r="A36" s="6" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B36" s="7" t="n"/>
       <c r="C36" s="7" t="n"/>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>Rashee Rice</t>
+          <t>Tetairoa McMillan</t>
         </is>
       </c>
       <c r="E36" s="7" t="n"/>
@@ -1130,11 +1130,11 @@
     </row>
     <row r="37">
       <c r="A37" s="6" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>Omarion Hampton</t>
+          <t>Chuba Hubbard</t>
         </is>
       </c>
       <c r="C37" s="7" t="n"/>
@@ -1146,13 +1146,13 @@
     </row>
     <row r="38">
       <c r="A38" s="6" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="B38" s="7" t="n"/>
       <c r="C38" s="7" t="n"/>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>Davante Adams</t>
+          <t>George Pickens</t>
         </is>
       </c>
       <c r="E38" s="7" t="n"/>
@@ -1162,43 +1162,43 @@
     </row>
     <row r="39">
       <c r="A39" s="6" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B39" s="7" t="n"/>
       <c r="C39" s="7" t="n"/>
-      <c r="D39" s="7" t="inlineStr">
-        <is>
-          <t>Zay Flowers</t>
-        </is>
-      </c>
+      <c r="D39" s="7" t="n"/>
       <c r="E39" s="7" t="n"/>
-      <c r="F39" s="7" t="n"/>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>George Kittle</t>
+        </is>
+      </c>
       <c r="G39" s="7" t="n"/>
       <c r="H39" s="7" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="6" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B40" s="7" t="n"/>
       <c r="C40" s="7" t="n"/>
-      <c r="D40" s="7" t="inlineStr">
-        <is>
-          <t>Malik Nabers</t>
-        </is>
-      </c>
+      <c r="D40" s="7" t="n"/>
       <c r="E40" s="7" t="n"/>
       <c r="F40" s="7" t="n"/>
       <c r="G40" s="7" t="n"/>
-      <c r="H40" s="7" t="n"/>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>Lamar Jackson</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>Cam Skattebo</t>
+          <t>Jeremiyah Love</t>
         </is>
       </c>
       <c r="C41" s="7" t="n"/>
@@ -1210,7 +1210,7 @@
     </row>
     <row r="42">
       <c r="A42" s="6" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B42" s="7" t="n"/>
       <c r="C42" s="7" t="n"/>
@@ -1226,13 +1226,13 @@
     </row>
     <row r="43">
       <c r="A43" s="6" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B43" s="7" t="n"/>
       <c r="C43" s="7" t="n"/>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>Tetairoa McMillan</t>
+          <t>A.J. Brown</t>
         </is>
       </c>
       <c r="E43" s="7" t="n"/>
@@ -1242,13 +1242,13 @@
     </row>
     <row r="44">
       <c r="A44" s="6" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B44" s="7" t="n"/>
       <c r="C44" s="7" t="n"/>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Parker Washington</t>
+          <t>Christian Watson</t>
         </is>
       </c>
       <c r="E44" s="7" t="n"/>
@@ -1258,15 +1258,15 @@
     </row>
     <row r="45">
       <c r="A45" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="B45" s="7" t="inlineStr">
-        <is>
-          <t>Jaylen Warren</t>
-        </is>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="B45" s="7" t="n"/>
       <c r="C45" s="7" t="n"/>
-      <c r="D45" s="7" t="n"/>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>Malik Nabers</t>
+        </is>
+      </c>
       <c r="E45" s="7" t="n"/>
       <c r="F45" s="7" t="n"/>
       <c r="G45" s="7" t="n"/>
@@ -1274,31 +1274,31 @@
     </row>
     <row r="46">
       <c r="A46" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="B46" s="7" t="inlineStr">
-        <is>
-          <t>Bucky Irving</t>
-        </is>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="B46" s="7" t="n"/>
       <c r="C46" s="7" t="n"/>
       <c r="D46" s="7" t="n"/>
       <c r="E46" s="7" t="n"/>
-      <c r="F46" s="7" t="n"/>
+      <c r="F46" s="7" t="inlineStr">
+        <is>
+          <t>Tyler Warren</t>
+        </is>
+      </c>
       <c r="G46" s="7" t="n"/>
       <c r="H46" s="7" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="B47" s="7" t="n"/>
+        <v>15</v>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Bucky Irving</t>
+        </is>
+      </c>
       <c r="C47" s="7" t="n"/>
-      <c r="D47" s="7" t="inlineStr">
-        <is>
-          <t>Jaylen Waddle</t>
-        </is>
-      </c>
+      <c r="D47" s="7" t="n"/>
       <c r="E47" s="7" t="n"/>
       <c r="F47" s="7" t="n"/>
       <c r="G47" s="7" t="n"/>
@@ -1306,27 +1306,27 @@
     </row>
     <row r="48">
       <c r="A48" s="6" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B48" s="7" t="n"/>
       <c r="C48" s="7" t="n"/>
       <c r="D48" s="7" t="n"/>
       <c r="E48" s="7" t="n"/>
-      <c r="F48" s="7" t="n"/>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>Brock Bowers</t>
+        </is>
+      </c>
       <c r="G48" s="7" t="n"/>
-      <c r="H48" s="7" t="inlineStr">
-        <is>
-          <t>Lamar Jackson</t>
-        </is>
-      </c>
+      <c r="H48" s="7" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="6" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>Aaron Jones Sr.</t>
+          <t>Kyren Williams</t>
         </is>
       </c>
       <c r="C49" s="7" t="n"/>
@@ -1338,7 +1338,7 @@
     </row>
     <row r="50">
       <c r="A50" s="6" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
@@ -1354,15 +1354,15 @@
     </row>
     <row r="51">
       <c r="A51" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="B51" s="7" t="inlineStr">
-        <is>
-          <t>Travis Etienne Jr.</t>
-        </is>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="B51" s="7" t="n"/>
       <c r="C51" s="7" t="n"/>
-      <c r="D51" s="7" t="n"/>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>Jaylen Waddle</t>
+        </is>
+      </c>
       <c r="E51" s="7" t="n"/>
       <c r="F51" s="7" t="n"/>
       <c r="G51" s="7" t="n"/>
@@ -1370,15 +1370,15 @@
     </row>
     <row r="52">
       <c r="A52" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="B52" s="7" t="n"/>
+        <v>11</v>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>David Montgomery</t>
+        </is>
+      </c>
       <c r="C52" s="7" t="n"/>
-      <c r="D52" s="7" t="inlineStr">
-        <is>
-          <t>Ladd McConkey</t>
-        </is>
-      </c>
+      <c r="D52" s="7" t="n"/>
       <c r="E52" s="7" t="n"/>
       <c r="F52" s="7" t="n"/>
       <c r="G52" s="7" t="n"/>
@@ -1386,15 +1386,15 @@
     </row>
     <row r="53">
       <c r="A53" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="B53" s="7" t="inlineStr">
-        <is>
-          <t>David Montgomery</t>
-        </is>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="B53" s="7" t="n"/>
       <c r="C53" s="7" t="n"/>
-      <c r="D53" s="7" t="n"/>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>Rashee Rice</t>
+        </is>
+      </c>
       <c r="E53" s="7" t="n"/>
       <c r="F53" s="7" t="n"/>
       <c r="G53" s="7" t="n"/>
@@ -1402,15 +1402,15 @@
     </row>
     <row r="54">
       <c r="A54" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="B54" s="7" t="n"/>
+        <v>10</v>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>Omarion Hampton</t>
+        </is>
+      </c>
       <c r="C54" s="7" t="n"/>
-      <c r="D54" s="7" t="inlineStr">
-        <is>
-          <t>Christian Watson</t>
-        </is>
-      </c>
+      <c r="D54" s="7" t="n"/>
       <c r="E54" s="7" t="n"/>
       <c r="F54" s="7" t="n"/>
       <c r="G54" s="7" t="n"/>
@@ -1418,15 +1418,15 @@
     </row>
     <row r="55">
       <c r="A55" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="B55" s="7" t="inlineStr">
-        <is>
-          <t>Chuba Hubbard</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="B55" s="7" t="n"/>
       <c r="C55" s="7" t="n"/>
-      <c r="D55" s="7" t="n"/>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>Matthew Golden</t>
+        </is>
+      </c>
       <c r="E55" s="7" t="n"/>
       <c r="F55" s="7" t="n"/>
       <c r="G55" s="7" t="n"/>
@@ -1434,13 +1434,13 @@
     </row>
     <row r="56">
       <c r="A56" s="6" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B56" s="7" t="n"/>
       <c r="C56" s="7" t="n"/>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>Emeka Egbuka</t>
+          <t>Zay Flowers</t>
         </is>
       </c>
       <c r="E56" s="7" t="n"/>
@@ -1450,29 +1450,29 @@
     </row>
     <row r="57">
       <c r="A57" s="6" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B57" s="7" t="n"/>
       <c r="C57" s="7" t="n"/>
-      <c r="D57" s="7" t="n"/>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>Mike Evans</t>
+        </is>
+      </c>
       <c r="E57" s="7" t="n"/>
-      <c r="F57" s="7" t="inlineStr">
-        <is>
-          <t>Tyler Warren</t>
-        </is>
-      </c>
+      <c r="F57" s="7" t="n"/>
       <c r="G57" s="7" t="n"/>
       <c r="H57" s="7" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="6" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B58" s="7" t="n"/>
       <c r="C58" s="7" t="n"/>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>Mike Evans</t>
+          <t>Terry McLaurin</t>
         </is>
       </c>
       <c r="E58" s="7" t="n"/>
@@ -1482,15 +1482,15 @@
     </row>
     <row r="59">
       <c r="A59" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="B59" s="7" t="n"/>
+        <v>6</v>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>Bhayshul Tuten</t>
+        </is>
+      </c>
       <c r="C59" s="7" t="n"/>
-      <c r="D59" s="7" t="inlineStr">
-        <is>
-          <t>DJ Moore</t>
-        </is>
-      </c>
+      <c r="D59" s="7" t="n"/>
       <c r="E59" s="7" t="n"/>
       <c r="F59" s="7" t="n"/>
       <c r="G59" s="7" t="n"/>
@@ -1498,15 +1498,15 @@
     </row>
     <row r="60">
       <c r="A60" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="B60" s="7" t="n"/>
+        <v>6</v>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>Travis Etienne Jr.</t>
+        </is>
+      </c>
       <c r="C60" s="7" t="n"/>
-      <c r="D60" s="7" t="inlineStr">
-        <is>
-          <t>Terry McLaurin</t>
-        </is>
-      </c>
+      <c r="D60" s="7" t="n"/>
       <c r="E60" s="7" t="n"/>
       <c r="F60" s="7" t="n"/>
       <c r="G60" s="7" t="n"/>
@@ -1514,15 +1514,15 @@
     </row>
     <row r="61">
       <c r="A61" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="B61" s="7" t="inlineStr">
-        <is>
-          <t>Bhayshul Tuten</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="B61" s="7" t="n"/>
       <c r="C61" s="7" t="n"/>
-      <c r="D61" s="7" t="n"/>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>Michael Wilson</t>
+        </is>
+      </c>
       <c r="E61" s="7" t="n"/>
       <c r="F61" s="7" t="n"/>
       <c r="G61" s="7" t="n"/>
@@ -1530,47 +1530,47 @@
     </row>
     <row r="62">
       <c r="A62" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="B62" s="7" t="inlineStr">
-        <is>
-          <t>Jadarian Price</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="B62" s="7" t="n"/>
       <c r="C62" s="7" t="n"/>
       <c r="D62" s="7" t="n"/>
       <c r="E62" s="7" t="n"/>
-      <c r="F62" s="7" t="n"/>
+      <c r="F62" s="7" t="inlineStr">
+        <is>
+          <t>Isaiah Likely</t>
+        </is>
+      </c>
       <c r="G62" s="7" t="n"/>
       <c r="H62" s="7" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="6" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B63" s="7" t="n"/>
       <c r="C63" s="7" t="n"/>
-      <c r="D63" s="7" t="inlineStr">
-        <is>
-          <t>Luther Burden III</t>
-        </is>
-      </c>
+      <c r="D63" s="7" t="n"/>
       <c r="E63" s="7" t="n"/>
       <c r="F63" s="7" t="n"/>
       <c r="G63" s="7" t="n"/>
-      <c r="H63" s="7" t="n"/>
+      <c r="H63" s="7" t="inlineStr">
+        <is>
+          <t>Drake Maye</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="B64" s="7" t="n"/>
+        <v>5</v>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>Rhamondre Stevenson</t>
+        </is>
+      </c>
       <c r="C64" s="7" t="n"/>
-      <c r="D64" s="7" t="inlineStr">
-        <is>
-          <t>Matthew Golden</t>
-        </is>
-      </c>
+      <c r="D64" s="7" t="n"/>
       <c r="E64" s="7" t="n"/>
       <c r="F64" s="7" t="n"/>
       <c r="G64" s="7" t="n"/>
@@ -1578,15 +1578,15 @@
     </row>
     <row r="65">
       <c r="A65" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="B65" s="7" t="inlineStr">
-        <is>
-          <t>Rhamondre Stevenson</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="B65" s="7" t="n"/>
       <c r="C65" s="7" t="n"/>
-      <c r="D65" s="7" t="n"/>
+      <c r="D65" s="7" t="inlineStr">
+        <is>
+          <t>Ladd McConkey</t>
+        </is>
+      </c>
       <c r="E65" s="7" t="n"/>
       <c r="F65" s="7" t="n"/>
       <c r="G65" s="7" t="n"/>
@@ -1594,13 +1594,13 @@
     </row>
     <row r="66">
       <c r="A66" s="6" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="B66" s="7" t="n"/>
       <c r="C66" s="7" t="n"/>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>Michael Wilson</t>
+          <t>DJ Moore</t>
         </is>
       </c>
       <c r="E66" s="7" t="n"/>
@@ -1610,15 +1610,15 @@
     </row>
     <row r="67">
       <c r="A67" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="B67" s="7" t="inlineStr">
-        <is>
-          <t>MarShawn Lloyd</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="B67" s="7" t="n"/>
       <c r="C67" s="7" t="n"/>
-      <c r="D67" s="7" t="n"/>
+      <c r="D67" s="7" t="inlineStr">
+        <is>
+          <t>Luther Burden III</t>
+        </is>
+      </c>
       <c r="E67" s="7" t="n"/>
       <c r="F67" s="7" t="n"/>
       <c r="G67" s="7" t="n"/>
@@ -1626,13 +1626,13 @@
     </row>
     <row r="68">
       <c r="A68" s="6" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B68" s="7" t="n"/>
       <c r="C68" s="7" t="n"/>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>Jameson Williams</t>
+          <t>Carnell Tate</t>
         </is>
       </c>
       <c r="E68" s="7" t="n"/>
@@ -1642,13 +1642,13 @@
     </row>
     <row r="69">
       <c r="A69" s="6" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B69" s="7" t="n"/>
       <c r="C69" s="7" t="n"/>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>De'Zhaun Stribling</t>
+          <t>Stefon Diggs</t>
         </is>
       </c>
       <c r="E69" s="7" t="n"/>
@@ -1658,7 +1658,7 @@
     </row>
     <row r="70">
       <c r="A70" s="6" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B70" s="7" t="n"/>
       <c r="C70" s="7" t="n"/>
@@ -1668,21 +1668,21 @@
       <c r="G70" s="7" t="n"/>
       <c r="H70" s="7" t="inlineStr">
         <is>
-          <t>Joe Burrow</t>
+          <t>Dak Prescott</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="B71" s="7" t="n"/>
+        <v>4</v>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>Josh Jacobs</t>
+        </is>
+      </c>
       <c r="C71" s="7" t="n"/>
-      <c r="D71" s="7" t="inlineStr">
-        <is>
-          <t>Carnell Tate</t>
-        </is>
-      </c>
+      <c r="D71" s="7" t="n"/>
       <c r="E71" s="7" t="n"/>
       <c r="F71" s="7" t="n"/>
       <c r="G71" s="7" t="n"/>
@@ -1690,13 +1690,13 @@
     </row>
     <row r="72">
       <c r="A72" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B72" s="7" t="n"/>
       <c r="C72" s="7" t="n"/>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>Alec Pierce</t>
+          <t>Emeka Egbuka</t>
         </is>
       </c>
       <c r="E72" s="7" t="n"/>
@@ -1706,13 +1706,13 @@
     </row>
     <row r="73">
       <c r="A73" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B73" s="7" t="n"/>
       <c r="C73" s="7" t="n"/>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>Stefon Diggs</t>
+          <t>De'Zhaun Stribling</t>
         </is>
       </c>
       <c r="E73" s="7" t="n"/>
@@ -1722,47 +1722,47 @@
     </row>
     <row r="74">
       <c r="A74" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B74" s="7" t="n"/>
       <c r="C74" s="7" t="n"/>
       <c r="D74" s="7" t="n"/>
       <c r="E74" s="7" t="n"/>
-      <c r="F74" s="7" t="n"/>
+      <c r="F74" s="7" t="inlineStr">
+        <is>
+          <t>Harold Fannin Jr.</t>
+        </is>
+      </c>
       <c r="G74" s="7" t="n"/>
-      <c r="H74" s="7" t="inlineStr">
-        <is>
-          <t>Drake Maye</t>
-        </is>
-      </c>
+      <c r="H74" s="7" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B75" s="7" t="inlineStr">
-        <is>
-          <t>TreVeyon Henderson</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="B75" s="7" t="n"/>
       <c r="C75" s="7" t="n"/>
       <c r="D75" s="7" t="n"/>
       <c r="E75" s="7" t="n"/>
       <c r="F75" s="7" t="n"/>
       <c r="G75" s="7" t="n"/>
-      <c r="H75" s="7" t="n"/>
+      <c r="H75" s="7" t="inlineStr">
+        <is>
+          <t>Jayden Daniels</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B76" s="7" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="B76" s="7" t="inlineStr">
+        <is>
+          <t>Jadarian Price</t>
+        </is>
+      </c>
       <c r="C76" s="7" t="n"/>
-      <c r="D76" s="7" t="inlineStr">
-        <is>
-          <t>KC Concepcion</t>
-        </is>
-      </c>
+      <c r="D76" s="7" t="n"/>
       <c r="E76" s="7" t="n"/>
       <c r="F76" s="7" t="n"/>
       <c r="G76" s="7" t="n"/>
@@ -1770,79 +1770,79 @@
     </row>
     <row r="77">
       <c r="A77" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B77" s="7" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>Kenny Gainwell</t>
+        </is>
+      </c>
       <c r="C77" s="7" t="n"/>
       <c r="D77" s="7" t="n"/>
       <c r="E77" s="7" t="n"/>
-      <c r="F77" s="7" t="inlineStr">
-        <is>
-          <t>Colston Loveland</t>
-        </is>
-      </c>
+      <c r="F77" s="7" t="n"/>
       <c r="G77" s="7" t="n"/>
       <c r="H77" s="7" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B78" s="7" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="B78" s="7" t="inlineStr">
+        <is>
+          <t>Jordan Mason</t>
+        </is>
+      </c>
       <c r="C78" s="7" t="n"/>
       <c r="D78" s="7" t="n"/>
       <c r="E78" s="7" t="n"/>
-      <c r="F78" s="7" t="inlineStr">
-        <is>
-          <t>Isaiah Likely</t>
-        </is>
-      </c>
+      <c r="F78" s="7" t="n"/>
       <c r="G78" s="7" t="n"/>
       <c r="H78" s="7" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B79" s="7" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="B79" s="7" t="inlineStr">
+        <is>
+          <t>Tony Pollard</t>
+        </is>
+      </c>
       <c r="C79" s="7" t="n"/>
       <c r="D79" s="7" t="n"/>
       <c r="E79" s="7" t="n"/>
-      <c r="F79" s="7" t="inlineStr">
-        <is>
-          <t>George Kittle</t>
-        </is>
-      </c>
+      <c r="F79" s="7" t="n"/>
       <c r="G79" s="7" t="n"/>
       <c r="H79" s="7" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="6" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="B80" s="7" t="n"/>
       <c r="C80" s="7" t="n"/>
-      <c r="D80" s="7" t="n"/>
+      <c r="D80" s="7" t="inlineStr">
+        <is>
+          <t>Jameson Williams</t>
+        </is>
+      </c>
       <c r="E80" s="7" t="n"/>
       <c r="F80" s="7" t="n"/>
       <c r="G80" s="7" t="n"/>
-      <c r="H80" s="7" t="inlineStr">
-        <is>
-          <t>Jalen Hurts</t>
-        </is>
-      </c>
+      <c r="H80" s="7" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B81" s="7" t="inlineStr">
-        <is>
-          <t>Tony Pollard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="B81" s="7" t="n"/>
       <c r="C81" s="7" t="n"/>
-      <c r="D81" s="7" t="n"/>
+      <c r="D81" s="7" t="inlineStr">
+        <is>
+          <t>Alec Pierce</t>
+        </is>
+      </c>
       <c r="E81" s="7" t="n"/>
       <c r="F81" s="7" t="n"/>
       <c r="G81" s="7" t="n"/>
@@ -1850,11 +1850,11 @@
     </row>
     <row r="82">
       <c r="A82" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B82" s="7" t="inlineStr">
         <is>
-          <t>Kenny Gainwell</t>
+          <t>MarShawn Lloyd</t>
         </is>
       </c>
       <c r="C82" s="7" t="n"/>
@@ -1866,15 +1866,15 @@
     </row>
     <row r="83">
       <c r="A83" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B83" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="B83" s="7" t="inlineStr">
+        <is>
+          <t>TreVeyon Henderson</t>
+        </is>
+      </c>
       <c r="C83" s="7" t="n"/>
-      <c r="D83" s="7" t="inlineStr">
-        <is>
-          <t>Rome Odunze</t>
-        </is>
-      </c>
+      <c r="D83" s="7" t="n"/>
       <c r="E83" s="7" t="n"/>
       <c r="F83" s="7" t="n"/>
       <c r="G83" s="7" t="n"/>
@@ -1882,15 +1882,15 @@
     </row>
     <row r="84">
       <c r="A84" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B84" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="B84" s="7" t="inlineStr">
+        <is>
+          <t>Jonathon Brooks</t>
+        </is>
+      </c>
       <c r="C84" s="7" t="n"/>
-      <c r="D84" s="7" t="inlineStr">
-        <is>
-          <t>Jayden Reed</t>
-        </is>
-      </c>
+      <c r="D84" s="7" t="n"/>
       <c r="E84" s="7" t="n"/>
       <c r="F84" s="7" t="n"/>
       <c r="G84" s="7" t="n"/>
@@ -1898,15 +1898,15 @@
     </row>
     <row r="85">
       <c r="A85" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B85" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="B85" s="7" t="inlineStr">
+        <is>
+          <t>Mike Washington Jr.</t>
+        </is>
+      </c>
       <c r="C85" s="7" t="n"/>
-      <c r="D85" s="7" t="inlineStr">
-        <is>
-          <t>Jordyn Tyson</t>
-        </is>
-      </c>
+      <c r="D85" s="7" t="n"/>
       <c r="E85" s="7" t="n"/>
       <c r="F85" s="7" t="n"/>
       <c r="G85" s="7" t="n"/>
@@ -1914,11 +1914,11 @@
     </row>
     <row r="86">
       <c r="A86" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B86" s="7" t="inlineStr">
         <is>
-          <t>Josh Jacobs</t>
+          <t>Rico Dowdle</t>
         </is>
       </c>
       <c r="C86" s="7" t="n"/>
@@ -1930,15 +1930,15 @@
     </row>
     <row r="87">
       <c r="A87" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B87" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="B87" s="7" t="inlineStr">
+        <is>
+          <t>Jacory Croskey-Merritt</t>
+        </is>
+      </c>
       <c r="C87" s="7" t="n"/>
-      <c r="D87" s="7" t="inlineStr">
-        <is>
-          <t>DK Metcalf</t>
-        </is>
-      </c>
+      <c r="D87" s="7" t="n"/>
       <c r="E87" s="7" t="n"/>
       <c r="F87" s="7" t="n"/>
       <c r="G87" s="7" t="n"/>
@@ -1946,27 +1946,27 @@
     </row>
     <row r="88">
       <c r="A88" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B88" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="B88" s="7" t="inlineStr">
+        <is>
+          <t>J.K. Dobbins</t>
+        </is>
+      </c>
       <c r="C88" s="7" t="n"/>
       <c r="D88" s="7" t="n"/>
       <c r="E88" s="7" t="n"/>
       <c r="F88" s="7" t="n"/>
       <c r="G88" s="7" t="n"/>
-      <c r="H88" s="7" t="inlineStr">
-        <is>
-          <t>Jayden Daniels</t>
-        </is>
-      </c>
+      <c r="H88" s="7" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B89" s="7" t="inlineStr">
         <is>
-          <t>Jacory Croskey-Merritt</t>
+          <t>Blake Corum</t>
         </is>
       </c>
       <c r="C89" s="7" t="n"/>
@@ -1978,11 +1978,11 @@
     </row>
     <row r="90">
       <c r="A90" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B90" s="7" t="inlineStr">
         <is>
-          <t>Rachaad White</t>
+          <t>Woody Marks</t>
         </is>
       </c>
       <c r="C90" s="7" t="n"/>
@@ -1994,31 +1994,31 @@
     </row>
     <row r="91">
       <c r="A91" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B91" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="B91" s="7" t="inlineStr">
+        <is>
+          <t>Rachaad White</t>
+        </is>
+      </c>
       <c r="C91" s="7" t="n"/>
       <c r="D91" s="7" t="n"/>
       <c r="E91" s="7" t="n"/>
       <c r="F91" s="7" t="n"/>
       <c r="G91" s="7" t="n"/>
-      <c r="H91" s="7" t="inlineStr">
-        <is>
-          <t>Justin Herbert</t>
-        </is>
-      </c>
+      <c r="H91" s="7" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B92" s="7" t="inlineStr">
-        <is>
-          <t>Jordan Mason</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="B92" s="7" t="n"/>
       <c r="C92" s="7" t="n"/>
-      <c r="D92" s="7" t="n"/>
+      <c r="D92" s="7" t="inlineStr">
+        <is>
+          <t>Rome Odunze</t>
+        </is>
+      </c>
       <c r="E92" s="7" t="n"/>
       <c r="F92" s="7" t="n"/>
       <c r="G92" s="7" t="n"/>
@@ -2028,13 +2028,13 @@
       <c r="A93" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B93" s="7" t="inlineStr">
-        <is>
-          <t>J.K. Dobbins</t>
-        </is>
-      </c>
+      <c r="B93" s="7" t="n"/>
       <c r="C93" s="7" t="n"/>
-      <c r="D93" s="7" t="n"/>
+      <c r="D93" s="7" t="inlineStr">
+        <is>
+          <t>Jayden Reed</t>
+        </is>
+      </c>
       <c r="E93" s="7" t="n"/>
       <c r="F93" s="7" t="n"/>
       <c r="G93" s="7" t="n"/>
@@ -2044,13 +2044,13 @@
       <c r="A94" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B94" s="7" t="inlineStr">
-        <is>
-          <t>Jonathon Brooks</t>
-        </is>
-      </c>
+      <c r="B94" s="7" t="n"/>
       <c r="C94" s="7" t="n"/>
-      <c r="D94" s="7" t="n"/>
+      <c r="D94" s="7" t="inlineStr">
+        <is>
+          <t>Jordyn Tyson</t>
+        </is>
+      </c>
       <c r="E94" s="7" t="n"/>
       <c r="F94" s="7" t="n"/>
       <c r="G94" s="7" t="n"/>
@@ -2060,13 +2060,13 @@
       <c r="A95" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B95" s="7" t="inlineStr">
-        <is>
-          <t>Mike Washington Jr.</t>
-        </is>
-      </c>
+      <c r="B95" s="7" t="n"/>
       <c r="C95" s="7" t="n"/>
-      <c r="D95" s="7" t="n"/>
+      <c r="D95" s="7" t="inlineStr">
+        <is>
+          <t>Marvin Harrison Jr.</t>
+        </is>
+      </c>
       <c r="E95" s="7" t="n"/>
       <c r="F95" s="7" t="n"/>
       <c r="G95" s="7" t="n"/>
@@ -2076,13 +2076,13 @@
       <c r="A96" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B96" s="7" t="inlineStr">
-        <is>
-          <t>Rico Dowdle</t>
-        </is>
-      </c>
+      <c r="B96" s="7" t="n"/>
       <c r="C96" s="7" t="n"/>
-      <c r="D96" s="7" t="n"/>
+      <c r="D96" s="7" t="inlineStr">
+        <is>
+          <t>KC Concepcion</t>
+        </is>
+      </c>
       <c r="E96" s="7" t="n"/>
       <c r="F96" s="7" t="n"/>
       <c r="G96" s="7" t="n"/>
@@ -2092,13 +2092,13 @@
       <c r="A97" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B97" s="7" t="inlineStr">
-        <is>
-          <t>Blake Corum</t>
-        </is>
-      </c>
+      <c r="B97" s="7" t="n"/>
       <c r="C97" s="7" t="n"/>
-      <c r="D97" s="7" t="n"/>
+      <c r="D97" s="7" t="inlineStr">
+        <is>
+          <t>Quentin Johnston</t>
+        </is>
+      </c>
       <c r="E97" s="7" t="n"/>
       <c r="F97" s="7" t="n"/>
       <c r="G97" s="7" t="n"/>
@@ -2108,13 +2108,13 @@
       <c r="A98" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B98" s="7" t="inlineStr">
-        <is>
-          <t>Woody Marks</t>
-        </is>
-      </c>
+      <c r="B98" s="7" t="n"/>
       <c r="C98" s="7" t="n"/>
-      <c r="D98" s="7" t="n"/>
+      <c r="D98" s="7" t="inlineStr">
+        <is>
+          <t>Chris Godwin Jr.</t>
+        </is>
+      </c>
       <c r="E98" s="7" t="n"/>
       <c r="F98" s="7" t="n"/>
       <c r="G98" s="7" t="n"/>
@@ -2128,7 +2128,7 @@
       <c r="C99" s="7" t="n"/>
       <c r="D99" s="7" t="inlineStr">
         <is>
-          <t>Brian Thomas Jr.</t>
+          <t>DK Metcalf</t>
         </is>
       </c>
       <c r="E99" s="7" t="n"/>
@@ -2144,7 +2144,7 @@
       <c r="C100" s="7" t="n"/>
       <c r="D100" s="7" t="inlineStr">
         <is>
-          <t>Marvin Harrison Jr.</t>
+          <t>Brian Thomas Jr.</t>
         </is>
       </c>
       <c r="E100" s="7" t="n"/>
@@ -2160,7 +2160,7 @@
       <c r="C101" s="7" t="n"/>
       <c r="D101" s="7" t="inlineStr">
         <is>
-          <t>Quentin Johnston</t>
+          <t>Ja'Kobi Lane</t>
         </is>
       </c>
       <c r="E101" s="7" t="n"/>
@@ -2174,13 +2174,13 @@
       </c>
       <c r="B102" s="7" t="n"/>
       <c r="C102" s="7" t="n"/>
-      <c r="D102" s="7" t="inlineStr">
-        <is>
-          <t>Chris Godwin Jr.</t>
-        </is>
-      </c>
+      <c r="D102" s="7" t="n"/>
       <c r="E102" s="7" t="n"/>
-      <c r="F102" s="7" t="n"/>
+      <c r="F102" s="7" t="inlineStr">
+        <is>
+          <t>Colston Loveland</t>
+        </is>
+      </c>
       <c r="G102" s="7" t="n"/>
       <c r="H102" s="7" t="n"/>
     </row>
@@ -2190,13 +2190,13 @@
       </c>
       <c r="B103" s="7" t="n"/>
       <c r="C103" s="7" t="n"/>
-      <c r="D103" s="7" t="inlineStr">
-        <is>
-          <t>Ja'Kobi Lane</t>
-        </is>
-      </c>
+      <c r="D103" s="7" t="n"/>
       <c r="E103" s="7" t="n"/>
-      <c r="F103" s="7" t="n"/>
+      <c r="F103" s="7" t="inlineStr">
+        <is>
+          <t>Tucker Kraft</t>
+        </is>
+      </c>
       <c r="G103" s="7" t="n"/>
       <c r="H103" s="7" t="n"/>
     </row>
@@ -2208,13 +2208,13 @@
       <c r="C104" s="7" t="n"/>
       <c r="D104" s="7" t="n"/>
       <c r="E104" s="7" t="n"/>
-      <c r="F104" s="7" t="inlineStr">
-        <is>
-          <t>Tucker Kraft</t>
-        </is>
-      </c>
+      <c r="F104" s="7" t="n"/>
       <c r="G104" s="7" t="n"/>
-      <c r="H104" s="7" t="n"/>
+      <c r="H104" s="7" t="inlineStr">
+        <is>
+          <t>Joe Burrow</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="6" t="n">
@@ -2224,13 +2224,13 @@
       <c r="C105" s="7" t="n"/>
       <c r="D105" s="7" t="n"/>
       <c r="E105" s="7" t="n"/>
-      <c r="F105" s="7" t="inlineStr">
-        <is>
-          <t>Harold Fannin Jr.</t>
-        </is>
-      </c>
+      <c r="F105" s="7" t="n"/>
       <c r="G105" s="7" t="n"/>
-      <c r="H105" s="7" t="n"/>
+      <c r="H105" s="7" t="inlineStr">
+        <is>
+          <t>Trevor Lawrence</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="6" t="n">
@@ -2244,7 +2244,7 @@
       <c r="G106" s="7" t="n"/>
       <c r="H106" s="7" t="inlineStr">
         <is>
-          <t>Trevor Lawrence</t>
+          <t>Jalen Hurts</t>
         </is>
       </c>
     </row>
@@ -2260,7 +2260,7 @@
       <c r="G107" s="7" t="n"/>
       <c r="H107" s="7" t="inlineStr">
         <is>
-          <t>Dak Prescott</t>
+          <t>Justin Herbert</t>
         </is>
       </c>
     </row>
@@ -2311,7 +2311,7 @@
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>Baseline: the live Trade Values Google Sheet (Half PPR, 10-team), 105 players, top value 70.</t>
+          <t>Baseline: the live Trade Values Google Sheet (Half PPR, 10-team), 105 players, top value 85.</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2335,7 @@
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   (Projections page snapshot 0): implied = average of the sheet value at the player's projection-rank slot</t>
+          <t xml:space="preserve">   (Projections page snapshot 0; 32 players used week 3 medians): implied = average of the seed value at the player's projection-rank slot among the projected players at the position</t>
         </is>
       </c>
     </row>
@@ -2349,14 +2349,14 @@
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   new = sheet + 0.4 x (implied - sheet), then rescaled so the total equals the sheet total. 55 players moved.</t>
+          <t xml:space="preserve">   new = sheet + 0.8 x (implied - sheet), then rescaled so the total equals the sheet total. 80 players moved.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   No projection this week (value kept): Bijan Robinson, Puka Nacua, Kenneth Walker III, Saquon Barkley, Ashton Jeanty, Derrick Henry, Justin Jefferson, De'Von Achane, Chris Olave, A.J. Brown, Breece Hall, Drake London, Brock Bowers, Kyren Williams, Josh Allen, Rashee Rice, Zay Flowers, Lamar Jackson, Travis Etienne Jr., Jadarian Price, MarShawn Lloyd, Mike Evans, Joe Burrow, Drake Maye, Luther Burden III, Josh Jacobs, De'Zhaun Stribling, Jayden Daniels, Jordan Mason, Alec Pierce, J.K. Dobbins, Chris Godwin Jr., Jonathon Brooks, Jayden Reed, Mike Washington Jr., Jordyn Tyson, Trevor Lawrence, Rico Dowdle, Dak Prescott, Blake Corum, Kenny Gainwell, Jaxson Dart, Rachaad White, Ja'Kobi Lane, Woody Marks.</t>
+          <t xml:space="preserve">   No projection this week (value kept): Puka Nacua, Josh Jacobs, De'Zhaun Stribling, Jayden Daniels, Jordan Mason, Alec Pierce, Jonathon Brooks, Jayden Reed, Mike Washington Jr., Jordyn Tyson, Rico Dowdle, Jaxson Dart, Ja'Kobi Lane.</t>
         </is>
       </c>
     </row>
@@ -2408,7 +2408,7 @@
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Replacement level = average line of baseline players valued 5 or less at the position: RB 1.8, WR 2.9, TE 4.5, QB 0.0.</t>
+          <t xml:space="preserve">   Replacement level = average line of baseline players valued 5 or less at the position: RB 1.9, WR 3.2, TE 3.5, QB 0.0.</t>
         </is>
       </c>
     </row>
@@ -2435,7 +2435,7 @@
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>Largest moves vs. the baseline in this file: Puka Nacua 65-&gt;71, Jaxon Smith-Njigba 56-&gt;62, Ja'Marr Chase 55-&gt;59, Amon-Ra St. Brown 52-&gt;56, James Cook III 49-&gt;45, Derrick Henry 55-&gt;51, Omarion Hampton 32-&gt;28, Chris Olave 41-&gt;45</t>
+          <t>Largest moves vs. the baseline in this file: Derrick Henry 57-&gt;44, Jahmyr Gibbs 85-&gt;73, James Cook III 53-&gt;41, Jonathan Taylor 66-&gt;55, Kenneth Walker III 64-&gt;53, Bijan Robinson 74-&gt;64, Jaxon Smith-Njigba 82-&gt;72, Christian McCaffrey 69-&gt;60</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Trade values: weight 0.6 and rank_share 0.7 to flatten the bottom
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TradeValueSheets/TradeValues_FullPPR_10team.xlsx
+++ b/TradeValueSheets/TradeValues_FullPPR_10team.xlsx
@@ -618,7 +618,7 @@
     </row>
     <row r="5">
       <c r="A5" s="6" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B5" s="7" t="n"/>
       <c r="C5" s="7" t="n"/>
@@ -634,7 +634,7 @@
     </row>
     <row r="6">
       <c r="A6" s="6" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
@@ -650,7 +650,7 @@
     </row>
     <row r="7">
       <c r="A7" s="6" t="n">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
@@ -666,13 +666,13 @@
     </row>
     <row r="8">
       <c r="A8" s="6" t="n">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="B8" s="7" t="n"/>
       <c r="C8" s="7" t="n"/>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Ja'Marr Chase</t>
+          <t>Puka Nacua</t>
         </is>
       </c>
       <c r="E8" s="7" t="n"/>
@@ -682,13 +682,13 @@
     </row>
     <row r="9">
       <c r="A9" s="6" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B9" s="7" t="n"/>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Amon-Ra St. Brown</t>
+          <t>Ja'Marr Chase</t>
         </is>
       </c>
       <c r="E9" s="7" t="n"/>
@@ -698,13 +698,13 @@
     </row>
     <row r="10">
       <c r="A10" s="6" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B10" s="7" t="n"/>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Puka Nacua</t>
+          <t>Amon-Ra St. Brown</t>
         </is>
       </c>
       <c r="E10" s="7" t="n"/>
@@ -714,7 +714,7 @@
     </row>
     <row r="11">
       <c r="A11" s="6" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
     </row>
     <row r="12">
       <c r="A12" s="6" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
@@ -748,13 +748,13 @@
       <c r="A13" s="6" t="n">
         <v>50</v>
       </c>
-      <c r="B13" s="7" t="n"/>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Derrick Henry</t>
+        </is>
+      </c>
       <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>Chris Olave</t>
-        </is>
-      </c>
+      <c r="D13" s="7" t="n"/>
       <c r="E13" s="7" t="n"/>
       <c r="F13" s="7" t="n"/>
       <c r="G13" s="7" t="n"/>
@@ -762,15 +762,15 @@
     </row>
     <row r="14">
       <c r="A14" s="6" t="n">
-        <v>47</v>
-      </c>
-      <c r="B14" s="7" t="n"/>
+        <v>50</v>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Ashton Jeanty</t>
+        </is>
+      </c>
       <c r="C14" s="7" t="n"/>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>CeeDee Lamb</t>
-        </is>
-      </c>
+      <c r="D14" s="7" t="n"/>
       <c r="E14" s="7" t="n"/>
       <c r="F14" s="7" t="n"/>
       <c r="G14" s="7" t="n"/>
@@ -778,11 +778,11 @@
     </row>
     <row r="15">
       <c r="A15" s="6" t="n">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Derrick Henry</t>
+          <t>James Cook III</t>
         </is>
       </c>
       <c r="C15" s="7" t="n"/>
@@ -794,15 +794,15 @@
     </row>
     <row r="16">
       <c r="A16" s="6" t="n">
-        <v>44</v>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>Ashton Jeanty</t>
-        </is>
-      </c>
+        <v>49</v>
+      </c>
+      <c r="B16" s="7" t="n"/>
       <c r="C16" s="7" t="n"/>
-      <c r="D16" s="7" t="n"/>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Chris Olave</t>
+        </is>
+      </c>
       <c r="E16" s="7" t="n"/>
       <c r="F16" s="7" t="n"/>
       <c r="G16" s="7" t="n"/>
@@ -810,15 +810,15 @@
     </row>
     <row r="17">
       <c r="A17" s="6" t="n">
-        <v>43</v>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>Chase Brown</t>
-        </is>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="B17" s="7" t="n"/>
       <c r="C17" s="7" t="n"/>
-      <c r="D17" s="7" t="n"/>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>CeeDee Lamb</t>
+        </is>
+      </c>
       <c r="E17" s="7" t="n"/>
       <c r="F17" s="7" t="n"/>
       <c r="G17" s="7" t="n"/>
@@ -826,31 +826,31 @@
     </row>
     <row r="18">
       <c r="A18" s="6" t="n">
-        <v>43</v>
-      </c>
-      <c r="B18" s="7" t="n"/>
+        <v>47</v>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Chase Brown</t>
+        </is>
+      </c>
       <c r="C18" s="7" t="n"/>
       <c r="D18" s="7" t="n"/>
       <c r="E18" s="7" t="n"/>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>Trey McBride</t>
-        </is>
-      </c>
+      <c r="F18" s="7" t="n"/>
       <c r="G18" s="7" t="n"/>
       <c r="H18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="n">
-        <v>41</v>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>James Cook III</t>
-        </is>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="B19" s="7" t="n"/>
       <c r="C19" s="7" t="n"/>
-      <c r="D19" s="7" t="n"/>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Justin Jefferson</t>
+        </is>
+      </c>
       <c r="E19" s="7" t="n"/>
       <c r="F19" s="7" t="n"/>
       <c r="G19" s="7" t="n"/>
@@ -858,15 +858,15 @@
     </row>
     <row r="20">
       <c r="A20" s="6" t="n">
-        <v>41</v>
-      </c>
-      <c r="B20" s="7" t="n"/>
+        <v>40</v>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>De'Von Achane</t>
+        </is>
+      </c>
       <c r="C20" s="7" t="n"/>
-      <c r="D20" s="7" t="inlineStr">
-        <is>
-          <t>Justin Jefferson</t>
-        </is>
-      </c>
+      <c r="D20" s="7" t="n"/>
       <c r="E20" s="7" t="n"/>
       <c r="F20" s="7" t="n"/>
       <c r="G20" s="7" t="n"/>
@@ -874,29 +874,29 @@
     </row>
     <row r="21">
       <c r="A21" s="6" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B21" s="7" t="n"/>
       <c r="C21" s="7" t="n"/>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>Garrett Wilson</t>
-        </is>
-      </c>
+      <c r="D21" s="7" t="n"/>
       <c r="E21" s="7" t="n"/>
-      <c r="F21" s="7" t="n"/>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>Trey McBride</t>
+        </is>
+      </c>
       <c r="G21" s="7" t="n"/>
       <c r="H21" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B22" s="7" t="n"/>
       <c r="C22" s="7" t="n"/>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Davante Adams</t>
+          <t>Garrett Wilson</t>
         </is>
       </c>
       <c r="E22" s="7" t="n"/>
@@ -906,11 +906,11 @@
     </row>
     <row r="23">
       <c r="A23" s="6" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>De'Von Achane</t>
+          <t>Breece Hall</t>
         </is>
       </c>
       <c r="C23" s="7" t="n"/>
@@ -922,13 +922,13 @@
     </row>
     <row r="24">
       <c r="A24" s="6" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B24" s="7" t="n"/>
       <c r="C24" s="7" t="n"/>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Parker Washington</t>
+          <t>Davante Adams</t>
         </is>
       </c>
       <c r="E24" s="7" t="n"/>
@@ -938,11 +938,11 @@
     </row>
     <row r="25">
       <c r="A25" s="6" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Breece Hall</t>
+          <t>Saquon Barkley</t>
         </is>
       </c>
       <c r="C25" s="7" t="n"/>
@@ -954,11 +954,11 @@
     </row>
     <row r="26">
       <c r="A26" s="6" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Jaylen Warren</t>
+          <t>D'Andre Swift</t>
         </is>
       </c>
       <c r="C26" s="7" t="n"/>
@@ -970,11 +970,11 @@
     </row>
     <row r="27">
       <c r="A27" s="6" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Aaron Jones Sr.</t>
+          <t>Javonte Williams</t>
         </is>
       </c>
       <c r="C27" s="7" t="n"/>
@@ -986,7 +986,7 @@
     </row>
     <row r="28">
       <c r="A28" s="6" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B28" s="7" t="n"/>
       <c r="C28" s="7" t="n"/>
@@ -1002,15 +1002,15 @@
     </row>
     <row r="29">
       <c r="A29" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t>D'Andre Swift</t>
-        </is>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="B29" s="7" t="n"/>
       <c r="C29" s="7" t="n"/>
-      <c r="D29" s="7" t="n"/>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Drake London</t>
+        </is>
+      </c>
       <c r="E29" s="7" t="n"/>
       <c r="F29" s="7" t="n"/>
       <c r="G29" s="7" t="n"/>
@@ -1018,7 +1018,7 @@
     </row>
     <row r="30">
       <c r="A30" s="6" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B30" s="7" t="n"/>
       <c r="C30" s="7" t="n"/>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Cam Skattebo</t>
+          <t>Jaylen Warren</t>
         </is>
       </c>
       <c r="C31" s="7" t="n"/>
@@ -1050,15 +1050,15 @@
     </row>
     <row r="32">
       <c r="A32" s="6" t="n">
-        <v>28</v>
-      </c>
-      <c r="B32" s="7" t="inlineStr">
-        <is>
-          <t>Javonte Williams</t>
-        </is>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="B32" s="7" t="n"/>
       <c r="C32" s="7" t="n"/>
-      <c r="D32" s="7" t="n"/>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>DeVonta Smith</t>
+        </is>
+      </c>
       <c r="E32" s="7" t="n"/>
       <c r="F32" s="7" t="n"/>
       <c r="G32" s="7" t="n"/>
@@ -1066,13 +1066,13 @@
     </row>
     <row r="33">
       <c r="A33" s="6" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B33" s="7" t="n"/>
       <c r="C33" s="7" t="n"/>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>DeVonta Smith</t>
+          <t>Parker Washington</t>
         </is>
       </c>
       <c r="E33" s="7" t="n"/>
@@ -1082,15 +1082,15 @@
     </row>
     <row r="34">
       <c r="A34" s="6" t="n">
-        <v>27</v>
-      </c>
-      <c r="B34" s="7" t="n"/>
+        <v>28</v>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Cam Skattebo</t>
+        </is>
+      </c>
       <c r="C34" s="7" t="n"/>
-      <c r="D34" s="7" t="inlineStr">
-        <is>
-          <t>Drake London</t>
-        </is>
-      </c>
+      <c r="D34" s="7" t="n"/>
       <c r="E34" s="7" t="n"/>
       <c r="F34" s="7" t="n"/>
       <c r="G34" s="7" t="n"/>
@@ -1098,11 +1098,11 @@
     </row>
     <row r="35">
       <c r="A35" s="6" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>Saquon Barkley</t>
+          <t>Aaron Jones Sr.</t>
         </is>
       </c>
       <c r="C35" s="7" t="n"/>
@@ -1114,13 +1114,13 @@
     </row>
     <row r="36">
       <c r="A36" s="6" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B36" s="7" t="n"/>
       <c r="C36" s="7" t="n"/>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>Tetairoa McMillan</t>
+          <t>George Pickens</t>
         </is>
       </c>
       <c r="E36" s="7" t="n"/>
@@ -1130,15 +1130,15 @@
     </row>
     <row r="37">
       <c r="A37" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="B37" s="7" t="inlineStr">
-        <is>
-          <t>Chuba Hubbard</t>
-        </is>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="B37" s="7" t="n"/>
       <c r="C37" s="7" t="n"/>
-      <c r="D37" s="7" t="n"/>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>A.J. Brown</t>
+        </is>
+      </c>
       <c r="E37" s="7" t="n"/>
       <c r="F37" s="7" t="n"/>
       <c r="G37" s="7" t="n"/>
@@ -1146,13 +1146,13 @@
     </row>
     <row r="38">
       <c r="A38" s="6" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B38" s="7" t="n"/>
       <c r="C38" s="7" t="n"/>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>George Pickens</t>
+          <t>Tetairoa McMillan</t>
         </is>
       </c>
       <c r="E38" s="7" t="n"/>
@@ -1164,41 +1164,41 @@
       <c r="A39" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="B39" s="7" t="n"/>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Jeremiyah Love</t>
+        </is>
+      </c>
       <c r="C39" s="7" t="n"/>
       <c r="D39" s="7" t="n"/>
       <c r="E39" s="7" t="n"/>
-      <c r="F39" s="7" t="inlineStr">
-        <is>
-          <t>George Kittle</t>
-        </is>
-      </c>
+      <c r="F39" s="7" t="n"/>
       <c r="G39" s="7" t="n"/>
       <c r="H39" s="7" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B40" s="7" t="n"/>
       <c r="C40" s="7" t="n"/>
-      <c r="D40" s="7" t="n"/>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>Tee Higgins</t>
+        </is>
+      </c>
       <c r="E40" s="7" t="n"/>
       <c r="F40" s="7" t="n"/>
       <c r="G40" s="7" t="n"/>
-      <c r="H40" s="7" t="inlineStr">
-        <is>
-          <t>Lamar Jackson</t>
-        </is>
-      </c>
+      <c r="H40" s="7" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="6" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>Jeremiyah Love</t>
+          <t>Chuba Hubbard</t>
         </is>
       </c>
       <c r="C41" s="7" t="n"/>
@@ -1210,13 +1210,13 @@
     </row>
     <row r="42">
       <c r="A42" s="6" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B42" s="7" t="n"/>
       <c r="C42" s="7" t="n"/>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>Tee Higgins</t>
+          <t>Malik Nabers</t>
         </is>
       </c>
       <c r="E42" s="7" t="n"/>
@@ -1226,47 +1226,47 @@
     </row>
     <row r="43">
       <c r="A43" s="6" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B43" s="7" t="n"/>
       <c r="C43" s="7" t="n"/>
-      <c r="D43" s="7" t="inlineStr">
-        <is>
-          <t>A.J. Brown</t>
-        </is>
-      </c>
+      <c r="D43" s="7" t="n"/>
       <c r="E43" s="7" t="n"/>
       <c r="F43" s="7" t="n"/>
       <c r="G43" s="7" t="n"/>
-      <c r="H43" s="7" t="n"/>
+      <c r="H43" s="7" t="inlineStr">
+        <is>
+          <t>Lamar Jackson</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B44" s="7" t="n"/>
       <c r="C44" s="7" t="n"/>
-      <c r="D44" s="7" t="inlineStr">
-        <is>
-          <t>Christian Watson</t>
-        </is>
-      </c>
+      <c r="D44" s="7" t="n"/>
       <c r="E44" s="7" t="n"/>
-      <c r="F44" s="7" t="n"/>
+      <c r="F44" s="7" t="inlineStr">
+        <is>
+          <t>Brock Bowers</t>
+        </is>
+      </c>
       <c r="G44" s="7" t="n"/>
       <c r="H44" s="7" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="B45" s="7" t="n"/>
+        <v>19</v>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Omarion Hampton</t>
+        </is>
+      </c>
       <c r="C45" s="7" t="n"/>
-      <c r="D45" s="7" t="inlineStr">
-        <is>
-          <t>Malik Nabers</t>
-        </is>
-      </c>
+      <c r="D45" s="7" t="n"/>
       <c r="E45" s="7" t="n"/>
       <c r="F45" s="7" t="n"/>
       <c r="G45" s="7" t="n"/>
@@ -1274,31 +1274,31 @@
     </row>
     <row r="46">
       <c r="A46" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="B46" s="7" t="n"/>
+        <v>19</v>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>Kyren Williams</t>
+        </is>
+      </c>
       <c r="C46" s="7" t="n"/>
       <c r="D46" s="7" t="n"/>
       <c r="E46" s="7" t="n"/>
-      <c r="F46" s="7" t="inlineStr">
-        <is>
-          <t>Tyler Warren</t>
-        </is>
-      </c>
+      <c r="F46" s="7" t="n"/>
       <c r="G46" s="7" t="n"/>
       <c r="H46" s="7" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="B47" s="7" t="inlineStr">
-        <is>
-          <t>Bucky Irving</t>
-        </is>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="B47" s="7" t="n"/>
       <c r="C47" s="7" t="n"/>
-      <c r="D47" s="7" t="n"/>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>Christian Watson</t>
+        </is>
+      </c>
       <c r="E47" s="7" t="n"/>
       <c r="F47" s="7" t="n"/>
       <c r="G47" s="7" t="n"/>
@@ -1306,43 +1306,43 @@
     </row>
     <row r="48">
       <c r="A48" s="6" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B48" s="7" t="n"/>
       <c r="C48" s="7" t="n"/>
-      <c r="D48" s="7" t="n"/>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>Jaylen Waddle</t>
+        </is>
+      </c>
       <c r="E48" s="7" t="n"/>
-      <c r="F48" s="7" t="inlineStr">
-        <is>
-          <t>Brock Bowers</t>
-        </is>
-      </c>
+      <c r="F48" s="7" t="n"/>
       <c r="G48" s="7" t="n"/>
       <c r="H48" s="7" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="B49" s="7" t="inlineStr">
-        <is>
-          <t>Kyren Williams</t>
-        </is>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="B49" s="7" t="n"/>
       <c r="C49" s="7" t="n"/>
       <c r="D49" s="7" t="n"/>
       <c r="E49" s="7" t="n"/>
-      <c r="F49" s="7" t="n"/>
+      <c r="F49" s="7" t="inlineStr">
+        <is>
+          <t>Tyler Warren</t>
+        </is>
+      </c>
       <c r="G49" s="7" t="n"/>
       <c r="H49" s="7" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="6" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>Quinshon Judkins</t>
+          <t>Bucky Irving</t>
         </is>
       </c>
       <c r="C50" s="7" t="n"/>
@@ -1354,13 +1354,13 @@
     </row>
     <row r="51">
       <c r="A51" s="6" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B51" s="7" t="n"/>
       <c r="C51" s="7" t="n"/>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>Jaylen Waddle</t>
+          <t>Rashee Rice</t>
         </is>
       </c>
       <c r="E51" s="7" t="n"/>
@@ -1370,29 +1370,29 @@
     </row>
     <row r="52">
       <c r="A52" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="B52" s="7" t="inlineStr">
-        <is>
-          <t>David Montgomery</t>
-        </is>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="B52" s="7" t="n"/>
       <c r="C52" s="7" t="n"/>
       <c r="D52" s="7" t="n"/>
       <c r="E52" s="7" t="n"/>
-      <c r="F52" s="7" t="n"/>
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>George Kittle</t>
+        </is>
+      </c>
       <c r="G52" s="7" t="n"/>
       <c r="H52" s="7" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B53" s="7" t="n"/>
       <c r="C53" s="7" t="n"/>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>Rashee Rice</t>
+          <t>Zay Flowers</t>
         </is>
       </c>
       <c r="E53" s="7" t="n"/>
@@ -1402,11 +1402,11 @@
     </row>
     <row r="54">
       <c r="A54" s="6" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>Omarion Hampton</t>
+          <t>Quinshon Judkins</t>
         </is>
       </c>
       <c r="C54" s="7" t="n"/>
@@ -1418,15 +1418,15 @@
     </row>
     <row r="55">
       <c r="A55" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="B55" s="7" t="n"/>
+        <v>13</v>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>David Montgomery</t>
+        </is>
+      </c>
       <c r="C55" s="7" t="n"/>
-      <c r="D55" s="7" t="inlineStr">
-        <is>
-          <t>Matthew Golden</t>
-        </is>
-      </c>
+      <c r="D55" s="7" t="n"/>
       <c r="E55" s="7" t="n"/>
       <c r="F55" s="7" t="n"/>
       <c r="G55" s="7" t="n"/>
@@ -1434,13 +1434,13 @@
     </row>
     <row r="56">
       <c r="A56" s="6" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B56" s="7" t="n"/>
       <c r="C56" s="7" t="n"/>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>Zay Flowers</t>
+          <t>Matthew Golden</t>
         </is>
       </c>
       <c r="E56" s="7" t="n"/>
@@ -1450,13 +1450,13 @@
     </row>
     <row r="57">
       <c r="A57" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B57" s="7" t="n"/>
       <c r="C57" s="7" t="n"/>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>Mike Evans</t>
+          <t>Terry McLaurin</t>
         </is>
       </c>
       <c r="E57" s="7" t="n"/>
@@ -1466,13 +1466,13 @@
     </row>
     <row r="58">
       <c r="A58" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B58" s="7" t="n"/>
       <c r="C58" s="7" t="n"/>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>Terry McLaurin</t>
+          <t>Mike Evans</t>
         </is>
       </c>
       <c r="E58" s="7" t="n"/>
@@ -1482,15 +1482,15 @@
     </row>
     <row r="59">
       <c r="A59" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B59" s="7" t="inlineStr">
-        <is>
-          <t>Bhayshul Tuten</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="B59" s="7" t="n"/>
       <c r="C59" s="7" t="n"/>
-      <c r="D59" s="7" t="n"/>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>Ladd McConkey</t>
+        </is>
+      </c>
       <c r="E59" s="7" t="n"/>
       <c r="F59" s="7" t="n"/>
       <c r="G59" s="7" t="n"/>
@@ -1498,11 +1498,11 @@
     </row>
     <row r="60">
       <c r="A60" s="6" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>Travis Etienne Jr.</t>
+          <t>Bhayshul Tuten</t>
         </is>
       </c>
       <c r="C60" s="7" t="n"/>
@@ -1514,15 +1514,15 @@
     </row>
     <row r="61">
       <c r="A61" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B61" s="7" t="n"/>
+        <v>9</v>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>Travis Etienne Jr.</t>
+        </is>
+      </c>
       <c r="C61" s="7" t="n"/>
-      <c r="D61" s="7" t="inlineStr">
-        <is>
-          <t>Michael Wilson</t>
-        </is>
-      </c>
+      <c r="D61" s="7" t="n"/>
       <c r="E61" s="7" t="n"/>
       <c r="F61" s="7" t="n"/>
       <c r="G61" s="7" t="n"/>
@@ -1530,47 +1530,47 @@
     </row>
     <row r="62">
       <c r="A62" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B62" s="7" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>Jadarian Price</t>
+        </is>
+      </c>
       <c r="C62" s="7" t="n"/>
       <c r="D62" s="7" t="n"/>
       <c r="E62" s="7" t="n"/>
-      <c r="F62" s="7" t="inlineStr">
-        <is>
-          <t>Isaiah Likely</t>
-        </is>
-      </c>
+      <c r="F62" s="7" t="n"/>
       <c r="G62" s="7" t="n"/>
       <c r="H62" s="7" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B63" s="7" t="n"/>
       <c r="C63" s="7" t="n"/>
-      <c r="D63" s="7" t="n"/>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>Emeka Egbuka</t>
+        </is>
+      </c>
       <c r="E63" s="7" t="n"/>
       <c r="F63" s="7" t="n"/>
       <c r="G63" s="7" t="n"/>
-      <c r="H63" s="7" t="inlineStr">
-        <is>
-          <t>Drake Maye</t>
-        </is>
-      </c>
+      <c r="H63" s="7" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B64" s="7" t="inlineStr">
-        <is>
-          <t>Rhamondre Stevenson</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="B64" s="7" t="n"/>
       <c r="C64" s="7" t="n"/>
-      <c r="D64" s="7" t="n"/>
+      <c r="D64" s="7" t="inlineStr">
+        <is>
+          <t>Michael Wilson</t>
+        </is>
+      </c>
       <c r="E64" s="7" t="n"/>
       <c r="F64" s="7" t="n"/>
       <c r="G64" s="7" t="n"/>
@@ -1578,13 +1578,13 @@
     </row>
     <row r="65">
       <c r="A65" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B65" s="7" t="n"/>
       <c r="C65" s="7" t="n"/>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>Ladd McConkey</t>
+          <t>DJ Moore</t>
         </is>
       </c>
       <c r="E65" s="7" t="n"/>
@@ -1594,13 +1594,13 @@
     </row>
     <row r="66">
       <c r="A66" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B66" s="7" t="n"/>
       <c r="C66" s="7" t="n"/>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>DJ Moore</t>
+          <t>Luther Burden III</t>
         </is>
       </c>
       <c r="E66" s="7" t="n"/>
@@ -1610,31 +1610,31 @@
     </row>
     <row r="67">
       <c r="A67" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B67" s="7" t="n"/>
       <c r="C67" s="7" t="n"/>
-      <c r="D67" s="7" t="inlineStr">
-        <is>
-          <t>Luther Burden III</t>
-        </is>
-      </c>
+      <c r="D67" s="7" t="n"/>
       <c r="E67" s="7" t="n"/>
       <c r="F67" s="7" t="n"/>
       <c r="G67" s="7" t="n"/>
-      <c r="H67" s="7" t="n"/>
+      <c r="H67" s="7" t="inlineStr">
+        <is>
+          <t>Drake Maye</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B68" s="7" t="n"/>
+        <v>6</v>
+      </c>
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>Rhamondre Stevenson</t>
+        </is>
+      </c>
       <c r="C68" s="7" t="n"/>
-      <c r="D68" s="7" t="inlineStr">
-        <is>
-          <t>Carnell Tate</t>
-        </is>
-      </c>
+      <c r="D68" s="7" t="n"/>
       <c r="E68" s="7" t="n"/>
       <c r="F68" s="7" t="n"/>
       <c r="G68" s="7" t="n"/>
@@ -1642,13 +1642,13 @@
     </row>
     <row r="69">
       <c r="A69" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B69" s="7" t="n"/>
       <c r="C69" s="7" t="n"/>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>Stefon Diggs</t>
+          <t>Carnell Tate</t>
         </is>
       </c>
       <c r="E69" s="7" t="n"/>
@@ -1658,23 +1658,23 @@
     </row>
     <row r="70">
       <c r="A70" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B70" s="7" t="n"/>
       <c r="C70" s="7" t="n"/>
-      <c r="D70" s="7" t="n"/>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>Stefon Diggs</t>
+        </is>
+      </c>
       <c r="E70" s="7" t="n"/>
       <c r="F70" s="7" t="n"/>
       <c r="G70" s="7" t="n"/>
-      <c r="H70" s="7" t="inlineStr">
-        <is>
-          <t>Dak Prescott</t>
-        </is>
-      </c>
+      <c r="H70" s="7" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
@@ -1690,13 +1690,13 @@
     </row>
     <row r="72">
       <c r="A72" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B72" s="7" t="n"/>
       <c r="C72" s="7" t="n"/>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>Emeka Egbuka</t>
+          <t>Jameson Williams</t>
         </is>
       </c>
       <c r="E72" s="7" t="n"/>
@@ -1706,7 +1706,7 @@
     </row>
     <row r="73">
       <c r="A73" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B73" s="7" t="n"/>
       <c r="C73" s="7" t="n"/>
@@ -1722,7 +1722,7 @@
     </row>
     <row r="74">
       <c r="A74" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B74" s="7" t="n"/>
       <c r="C74" s="7" t="n"/>
@@ -1730,7 +1730,7 @@
       <c r="E74" s="7" t="n"/>
       <c r="F74" s="7" t="inlineStr">
         <is>
-          <t>Harold Fannin Jr.</t>
+          <t>Colston Loveland</t>
         </is>
       </c>
       <c r="G74" s="7" t="n"/>
@@ -1738,59 +1738,59 @@
     </row>
     <row r="75">
       <c r="A75" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B75" s="7" t="n"/>
       <c r="C75" s="7" t="n"/>
       <c r="D75" s="7" t="n"/>
       <c r="E75" s="7" t="n"/>
-      <c r="F75" s="7" t="n"/>
+      <c r="F75" s="7" t="inlineStr">
+        <is>
+          <t>Isaiah Likely</t>
+        </is>
+      </c>
       <c r="G75" s="7" t="n"/>
-      <c r="H75" s="7" t="inlineStr">
-        <is>
-          <t>Jayden Daniels</t>
-        </is>
-      </c>
+      <c r="H75" s="7" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B76" s="7" t="inlineStr">
-        <is>
-          <t>Jadarian Price</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="B76" s="7" t="n"/>
       <c r="C76" s="7" t="n"/>
       <c r="D76" s="7" t="n"/>
       <c r="E76" s="7" t="n"/>
       <c r="F76" s="7" t="n"/>
       <c r="G76" s="7" t="n"/>
-      <c r="H76" s="7" t="n"/>
+      <c r="H76" s="7" t="inlineStr">
+        <is>
+          <t>Jayden Daniels</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B77" s="7" t="inlineStr">
-        <is>
-          <t>Kenny Gainwell</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="B77" s="7" t="n"/>
       <c r="C77" s="7" t="n"/>
       <c r="D77" s="7" t="n"/>
       <c r="E77" s="7" t="n"/>
       <c r="F77" s="7" t="n"/>
       <c r="G77" s="7" t="n"/>
-      <c r="H77" s="7" t="n"/>
+      <c r="H77" s="7" t="inlineStr">
+        <is>
+          <t>Dak Prescott</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B78" s="7" t="inlineStr">
         <is>
-          <t>Jordan Mason</t>
+          <t>Tony Pollard</t>
         </is>
       </c>
       <c r="C78" s="7" t="n"/>
@@ -1802,11 +1802,11 @@
     </row>
     <row r="79">
       <c r="A79" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B79" s="7" t="inlineStr">
         <is>
-          <t>Tony Pollard</t>
+          <t>Kenny Gainwell</t>
         </is>
       </c>
       <c r="C79" s="7" t="n"/>
@@ -1818,13 +1818,13 @@
     </row>
     <row r="80">
       <c r="A80" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B80" s="7" t="n"/>
       <c r="C80" s="7" t="n"/>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>Jameson Williams</t>
+          <t>Rome Odunze</t>
         </is>
       </c>
       <c r="E80" s="7" t="n"/>
@@ -1834,23 +1834,23 @@
     </row>
     <row r="81">
       <c r="A81" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B81" s="7" t="n"/>
       <c r="C81" s="7" t="n"/>
-      <c r="D81" s="7" t="inlineStr">
-        <is>
-          <t>Alec Pierce</t>
-        </is>
-      </c>
+      <c r="D81" s="7" t="n"/>
       <c r="E81" s="7" t="n"/>
       <c r="F81" s="7" t="n"/>
       <c r="G81" s="7" t="n"/>
-      <c r="H81" s="7" t="n"/>
+      <c r="H81" s="7" t="inlineStr">
+        <is>
+          <t>Joe Burrow</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B82" s="7" t="inlineStr">
         <is>
@@ -1866,7 +1866,7 @@
     </row>
     <row r="83">
       <c r="A83" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B83" s="7" t="inlineStr">
         <is>
@@ -1882,11 +1882,11 @@
     </row>
     <row r="84">
       <c r="A84" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B84" s="7" t="inlineStr">
         <is>
-          <t>Jonathon Brooks</t>
+          <t>Jordan Mason</t>
         </is>
       </c>
       <c r="C84" s="7" t="n"/>
@@ -1898,11 +1898,11 @@
     </row>
     <row r="85">
       <c r="A85" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B85" s="7" t="inlineStr">
         <is>
-          <t>Mike Washington Jr.</t>
+          <t>Rachaad White</t>
         </is>
       </c>
       <c r="C85" s="7" t="n"/>
@@ -1914,15 +1914,15 @@
     </row>
     <row r="86">
       <c r="A86" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B86" s="7" t="inlineStr">
-        <is>
-          <t>Rico Dowdle</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="B86" s="7" t="n"/>
       <c r="C86" s="7" t="n"/>
-      <c r="D86" s="7" t="n"/>
+      <c r="D86" s="7" t="inlineStr">
+        <is>
+          <t>Alec Pierce</t>
+        </is>
+      </c>
       <c r="E86" s="7" t="n"/>
       <c r="F86" s="7" t="n"/>
       <c r="G86" s="7" t="n"/>
@@ -1934,7 +1934,7 @@
       </c>
       <c r="B87" s="7" t="inlineStr">
         <is>
-          <t>Jacory Croskey-Merritt</t>
+          <t>Jonathon Brooks</t>
         </is>
       </c>
       <c r="C87" s="7" t="n"/>
@@ -1950,7 +1950,7 @@
       </c>
       <c r="B88" s="7" t="inlineStr">
         <is>
-          <t>J.K. Dobbins</t>
+          <t>Mike Washington Jr.</t>
         </is>
       </c>
       <c r="C88" s="7" t="n"/>
@@ -1966,7 +1966,7 @@
       </c>
       <c r="B89" s="7" t="inlineStr">
         <is>
-          <t>Blake Corum</t>
+          <t>Rico Dowdle</t>
         </is>
       </c>
       <c r="C89" s="7" t="n"/>
@@ -1982,7 +1982,7 @@
       </c>
       <c r="B90" s="7" t="inlineStr">
         <is>
-          <t>Woody Marks</t>
+          <t>Jacory Croskey-Merritt</t>
         </is>
       </c>
       <c r="C90" s="7" t="n"/>
@@ -1998,7 +1998,7 @@
       </c>
       <c r="B91" s="7" t="inlineStr">
         <is>
-          <t>Rachaad White</t>
+          <t>J.K. Dobbins</t>
         </is>
       </c>
       <c r="C91" s="7" t="n"/>
@@ -2012,13 +2012,13 @@
       <c r="A92" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B92" s="7" t="n"/>
+      <c r="B92" s="7" t="inlineStr">
+        <is>
+          <t>Blake Corum</t>
+        </is>
+      </c>
       <c r="C92" s="7" t="n"/>
-      <c r="D92" s="7" t="inlineStr">
-        <is>
-          <t>Rome Odunze</t>
-        </is>
-      </c>
+      <c r="D92" s="7" t="n"/>
       <c r="E92" s="7" t="n"/>
       <c r="F92" s="7" t="n"/>
       <c r="G92" s="7" t="n"/>
@@ -2028,13 +2028,13 @@
       <c r="A93" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B93" s="7" t="n"/>
+      <c r="B93" s="7" t="inlineStr">
+        <is>
+          <t>Woody Marks</t>
+        </is>
+      </c>
       <c r="C93" s="7" t="n"/>
-      <c r="D93" s="7" t="inlineStr">
-        <is>
-          <t>Jayden Reed</t>
-        </is>
-      </c>
+      <c r="D93" s="7" t="n"/>
       <c r="E93" s="7" t="n"/>
       <c r="F93" s="7" t="n"/>
       <c r="G93" s="7" t="n"/>
@@ -2048,7 +2048,7 @@
       <c r="C94" s="7" t="n"/>
       <c r="D94" s="7" t="inlineStr">
         <is>
-          <t>Jordyn Tyson</t>
+          <t>Marvin Harrison Jr.</t>
         </is>
       </c>
       <c r="E94" s="7" t="n"/>
@@ -2064,7 +2064,7 @@
       <c r="C95" s="7" t="n"/>
       <c r="D95" s="7" t="inlineStr">
         <is>
-          <t>Marvin Harrison Jr.</t>
+          <t>KC Concepcion</t>
         </is>
       </c>
       <c r="E95" s="7" t="n"/>
@@ -2080,7 +2080,7 @@
       <c r="C96" s="7" t="n"/>
       <c r="D96" s="7" t="inlineStr">
         <is>
-          <t>KC Concepcion</t>
+          <t>Quentin Johnston</t>
         </is>
       </c>
       <c r="E96" s="7" t="n"/>
@@ -2096,7 +2096,7 @@
       <c r="C97" s="7" t="n"/>
       <c r="D97" s="7" t="inlineStr">
         <is>
-          <t>Quentin Johnston</t>
+          <t>Chris Godwin Jr.</t>
         </is>
       </c>
       <c r="E97" s="7" t="n"/>
@@ -2112,7 +2112,7 @@
       <c r="C98" s="7" t="n"/>
       <c r="D98" s="7" t="inlineStr">
         <is>
-          <t>Chris Godwin Jr.</t>
+          <t>Jayden Reed</t>
         </is>
       </c>
       <c r="E98" s="7" t="n"/>
@@ -2128,7 +2128,7 @@
       <c r="C99" s="7" t="n"/>
       <c r="D99" s="7" t="inlineStr">
         <is>
-          <t>DK Metcalf</t>
+          <t>Jordyn Tyson</t>
         </is>
       </c>
       <c r="E99" s="7" t="n"/>
@@ -2160,7 +2160,7 @@
       <c r="C101" s="7" t="n"/>
       <c r="D101" s="7" t="inlineStr">
         <is>
-          <t>Ja'Kobi Lane</t>
+          <t>DK Metcalf</t>
         </is>
       </c>
       <c r="E101" s="7" t="n"/>
@@ -2174,13 +2174,13 @@
       </c>
       <c r="B102" s="7" t="n"/>
       <c r="C102" s="7" t="n"/>
-      <c r="D102" s="7" t="n"/>
+      <c r="D102" s="7" t="inlineStr">
+        <is>
+          <t>Ja'Kobi Lane</t>
+        </is>
+      </c>
       <c r="E102" s="7" t="n"/>
-      <c r="F102" s="7" t="inlineStr">
-        <is>
-          <t>Colston Loveland</t>
-        </is>
-      </c>
+      <c r="F102" s="7" t="n"/>
       <c r="G102" s="7" t="n"/>
       <c r="H102" s="7" t="n"/>
     </row>
@@ -2208,13 +2208,13 @@
       <c r="C104" s="7" t="n"/>
       <c r="D104" s="7" t="n"/>
       <c r="E104" s="7" t="n"/>
-      <c r="F104" s="7" t="n"/>
+      <c r="F104" s="7" t="inlineStr">
+        <is>
+          <t>Harold Fannin Jr.</t>
+        </is>
+      </c>
       <c r="G104" s="7" t="n"/>
-      <c r="H104" s="7" t="inlineStr">
-        <is>
-          <t>Joe Burrow</t>
-        </is>
-      </c>
+      <c r="H104" s="7" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="6" t="n">
@@ -2311,7 +2311,7 @@
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>Baseline: the live Trade Values Google Sheet (Half PPR, 10-team), 105 players, top value 85.</t>
+          <t>Baseline: the live Trade Values Google Sheet (Half PPR, 10-team), 105 players, top value 77.</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2335,7 @@
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   (Projections page snapshot 0; 32 players used week 3 medians): implied = average of the seed value at the player's projection-rank slot among the projected players at the position</t>
+          <t xml:space="preserve">   (Projections page snapshot 0; 32 players used week 3 medians): implied = 0.7 x the seed value at the player's projection-rank slot among the projected players at the position + 0.3 x</t>
         </is>
       </c>
     </row>
@@ -2349,7 +2349,7 @@
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   new = sheet + 0.8 x (implied - sheet), then rescaled so the total equals the sheet total. 80 players moved.</t>
+          <t xml:space="preserve">   new = sheet + 0.6 x (implied - sheet), then rescaled so the total equals the sheet total. 79 players moved.</t>
         </is>
       </c>
     </row>
@@ -2408,7 +2408,7 @@
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Replacement level = average line of baseline players valued 5 or less at the position: RB 1.9, WR 3.2, TE 3.5, QB 0.0.</t>
+          <t xml:space="preserve">   Replacement level = average line of baseline players valued 5 or less at the position: RB 1.9, WR 3.1, TE 4.5, QB 0.0.</t>
         </is>
       </c>
     </row>
@@ -2435,7 +2435,7 @@
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>Largest moves vs. the baseline in this file: Derrick Henry 57-&gt;44, Jahmyr Gibbs 85-&gt;73, James Cook III 53-&gt;41, Jonathan Taylor 66-&gt;55, Kenneth Walker III 64-&gt;53, Bijan Robinson 74-&gt;64, Jaxon Smith-Njigba 82-&gt;72, Christian McCaffrey 69-&gt;60</t>
+          <t>Largest moves vs. the baseline in this file: James Cook III 56-&gt;49, Derrick Henry 57-&gt;50, Josh Allen 37-&gt;31, Jonathan Taylor 63-&gt;58, Kenneth Walker III 62-&gt;57, Lamar Jackson 27-&gt;22, Bijan Robinson 72-&gt;68, Jahmyr Gibbs 77-&gt;73</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Trade values: re-seed weight 0.45
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TradeValueSheets/TradeValues_FullPPR_10team.xlsx
+++ b/TradeValueSheets/TradeValues_FullPPR_10team.xlsx
@@ -618,15 +618,15 @@
     </row>
     <row r="5">
       <c r="A5" s="6" t="n">
-        <v>70</v>
-      </c>
-      <c r="B5" s="7" t="n"/>
+        <v>71</v>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Bijan Robinson</t>
+        </is>
+      </c>
       <c r="C5" s="7" t="n"/>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>Jaxon Smith-Njigba</t>
-        </is>
-      </c>
+      <c r="D5" s="7" t="n"/>
       <c r="E5" s="7" t="n"/>
       <c r="F5" s="7" t="n"/>
       <c r="G5" s="7" t="n"/>
@@ -634,15 +634,15 @@
     </row>
     <row r="6">
       <c r="A6" s="6" t="n">
-        <v>68</v>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>Bijan Robinson</t>
-        </is>
-      </c>
+        <v>66</v>
+      </c>
+      <c r="B6" s="7" t="n"/>
       <c r="C6" s="7" t="n"/>
-      <c r="D6" s="7" t="n"/>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Jaxon Smith-Njigba</t>
+        </is>
+      </c>
       <c r="E6" s="7" t="n"/>
       <c r="F6" s="7" t="n"/>
       <c r="G6" s="7" t="n"/>
@@ -650,7 +650,7 @@
     </row>
     <row r="7">
       <c r="A7" s="6" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
@@ -666,13 +666,13 @@
     </row>
     <row r="8">
       <c r="A8" s="6" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B8" s="7" t="n"/>
       <c r="C8" s="7" t="n"/>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Puka Nacua</t>
+          <t>Ja'Marr Chase</t>
         </is>
       </c>
       <c r="E8" s="7" t="n"/>
@@ -682,13 +682,13 @@
     </row>
     <row r="9">
       <c r="A9" s="6" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B9" s="7" t="n"/>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Ja'Marr Chase</t>
+          <t>Amon-Ra St. Brown</t>
         </is>
       </c>
       <c r="E9" s="7" t="n"/>
@@ -704,7 +704,7 @@
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Amon-Ra St. Brown</t>
+          <t>Puka Nacua</t>
         </is>
       </c>
       <c r="E10" s="7" t="n"/>
@@ -714,11 +714,11 @@
     </row>
     <row r="11">
       <c r="A11" s="6" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Jonathan Taylor</t>
+          <t>Kenneth Walker III</t>
         </is>
       </c>
       <c r="C11" s="7" t="n"/>
@@ -730,11 +730,11 @@
     </row>
     <row r="12">
       <c r="A12" s="6" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Kenneth Walker III</t>
+          <t>Jonathan Taylor</t>
         </is>
       </c>
       <c r="C12" s="7" t="n"/>
@@ -746,15 +746,15 @@
     </row>
     <row r="13">
       <c r="A13" s="6" t="n">
-        <v>50</v>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Derrick Henry</t>
-        </is>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="B13" s="7" t="n"/>
       <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Chris Olave</t>
+        </is>
+      </c>
       <c r="E13" s="7" t="n"/>
       <c r="F13" s="7" t="n"/>
       <c r="G13" s="7" t="n"/>
@@ -762,7 +762,7 @@
     </row>
     <row r="14">
       <c r="A14" s="6" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
@@ -782,7 +782,7 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>James Cook III</t>
+          <t>Derrick Henry</t>
         </is>
       </c>
       <c r="C15" s="7" t="n"/>
@@ -794,13 +794,13 @@
     </row>
     <row r="16">
       <c r="A16" s="6" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B16" s="7" t="n"/>
       <c r="C16" s="7" t="n"/>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Chris Olave</t>
+          <t>Justin Jefferson</t>
         </is>
       </c>
       <c r="E16" s="7" t="n"/>
@@ -810,15 +810,15 @@
     </row>
     <row r="17">
       <c r="A17" s="6" t="n">
-        <v>48</v>
-      </c>
-      <c r="B17" s="7" t="n"/>
+        <v>45</v>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Saquon Barkley</t>
+        </is>
+      </c>
       <c r="C17" s="7" t="n"/>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>CeeDee Lamb</t>
-        </is>
-      </c>
+      <c r="D17" s="7" t="n"/>
       <c r="E17" s="7" t="n"/>
       <c r="F17" s="7" t="n"/>
       <c r="G17" s="7" t="n"/>
@@ -826,11 +826,11 @@
     </row>
     <row r="18">
       <c r="A18" s="6" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Chase Brown</t>
+          <t>James Cook III</t>
         </is>
       </c>
       <c r="C18" s="7" t="n"/>
@@ -842,15 +842,15 @@
     </row>
     <row r="19">
       <c r="A19" s="6" t="n">
-        <v>45</v>
-      </c>
-      <c r="B19" s="7" t="n"/>
+        <v>44</v>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Chase Brown</t>
+        </is>
+      </c>
       <c r="C19" s="7" t="n"/>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>Justin Jefferson</t>
-        </is>
-      </c>
+      <c r="D19" s="7" t="n"/>
       <c r="E19" s="7" t="n"/>
       <c r="F19" s="7" t="n"/>
       <c r="G19" s="7" t="n"/>
@@ -858,15 +858,15 @@
     </row>
     <row r="20">
       <c r="A20" s="6" t="n">
-        <v>40</v>
-      </c>
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>De'Von Achane</t>
-        </is>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="B20" s="7" t="n"/>
       <c r="C20" s="7" t="n"/>
-      <c r="D20" s="7" t="n"/>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>CeeDee Lamb</t>
+        </is>
+      </c>
       <c r="E20" s="7" t="n"/>
       <c r="F20" s="7" t="n"/>
       <c r="G20" s="7" t="n"/>
@@ -874,29 +874,29 @@
     </row>
     <row r="21">
       <c r="A21" s="6" t="n">
-        <v>39</v>
-      </c>
-      <c r="B21" s="7" t="n"/>
+        <v>41</v>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>De'Von Achane</t>
+        </is>
+      </c>
       <c r="C21" s="7" t="n"/>
       <c r="D21" s="7" t="n"/>
       <c r="E21" s="7" t="n"/>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>Trey McBride</t>
-        </is>
-      </c>
+      <c r="F21" s="7" t="n"/>
       <c r="G21" s="7" t="n"/>
       <c r="H21" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="B22" s="7" t="n"/>
       <c r="C22" s="7" t="n"/>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Garrett Wilson</t>
+          <t>Drake London</t>
         </is>
       </c>
       <c r="E22" s="7" t="n"/>
@@ -906,7 +906,7 @@
     </row>
     <row r="23">
       <c r="A23" s="6" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
@@ -922,13 +922,13 @@
     </row>
     <row r="24">
       <c r="A24" s="6" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B24" s="7" t="n"/>
       <c r="C24" s="7" t="n"/>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Davante Adams</t>
+          <t>Garrett Wilson</t>
         </is>
       </c>
       <c r="E24" s="7" t="n"/>
@@ -938,17 +938,17 @@
     </row>
     <row r="25">
       <c r="A25" s="6" t="n">
-        <v>33</v>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>Saquon Barkley</t>
-        </is>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="B25" s="7" t="n"/>
       <c r="C25" s="7" t="n"/>
       <c r="D25" s="7" t="n"/>
       <c r="E25" s="7" t="n"/>
-      <c r="F25" s="7" t="n"/>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>Trey McBride</t>
+        </is>
+      </c>
       <c r="G25" s="7" t="n"/>
       <c r="H25" s="7" t="n"/>
     </row>
@@ -956,13 +956,13 @@
       <c r="A26" s="6" t="n">
         <v>33</v>
       </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>D'Andre Swift</t>
-        </is>
-      </c>
+      <c r="B26" s="7" t="n"/>
       <c r="C26" s="7" t="n"/>
-      <c r="D26" s="7" t="n"/>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>Nico Collins</t>
+        </is>
+      </c>
       <c r="E26" s="7" t="n"/>
       <c r="F26" s="7" t="n"/>
       <c r="G26" s="7" t="n"/>
@@ -970,47 +970,47 @@
     </row>
     <row r="27">
       <c r="A27" s="6" t="n">
-        <v>33</v>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>Javonte Williams</t>
-        </is>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="B27" s="7" t="n"/>
       <c r="C27" s="7" t="n"/>
       <c r="D27" s="7" t="n"/>
       <c r="E27" s="7" t="n"/>
-      <c r="F27" s="7" t="n"/>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>Brock Bowers</t>
+        </is>
+      </c>
       <c r="G27" s="7" t="n"/>
       <c r="H27" s="7" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B28" s="7" t="n"/>
       <c r="C28" s="7" t="n"/>
-      <c r="D28" s="7" t="inlineStr">
-        <is>
-          <t>Nico Collins</t>
-        </is>
-      </c>
+      <c r="D28" s="7" t="n"/>
       <c r="E28" s="7" t="n"/>
       <c r="F28" s="7" t="n"/>
       <c r="G28" s="7" t="n"/>
-      <c r="H28" s="7" t="n"/>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Josh Allen</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="n">
-        <v>31</v>
-      </c>
-      <c r="B29" s="7" t="n"/>
+        <v>30</v>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Jeremiyah Love</t>
+        </is>
+      </c>
       <c r="C29" s="7" t="n"/>
-      <c r="D29" s="7" t="inlineStr">
-        <is>
-          <t>Drake London</t>
-        </is>
-      </c>
+      <c r="D29" s="7" t="n"/>
       <c r="E29" s="7" t="n"/>
       <c r="F29" s="7" t="n"/>
       <c r="G29" s="7" t="n"/>
@@ -1018,19 +1018,19 @@
     </row>
     <row r="30">
       <c r="A30" s="6" t="n">
-        <v>31</v>
-      </c>
-      <c r="B30" s="7" t="n"/>
+        <v>30</v>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Jaylen Warren</t>
+        </is>
+      </c>
       <c r="C30" s="7" t="n"/>
       <c r="D30" s="7" t="n"/>
       <c r="E30" s="7" t="n"/>
       <c r="F30" s="7" t="n"/>
       <c r="G30" s="7" t="n"/>
-      <c r="H30" s="7" t="inlineStr">
-        <is>
-          <t>Josh Allen</t>
-        </is>
-      </c>
+      <c r="H30" s="7" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="n">
@@ -1038,7 +1038,7 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Jaylen Warren</t>
+          <t>Javonte Williams</t>
         </is>
       </c>
       <c r="C31" s="7" t="n"/>
@@ -1056,7 +1056,7 @@
       <c r="C32" s="7" t="n"/>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>DeVonta Smith</t>
+          <t>George Pickens</t>
         </is>
       </c>
       <c r="E32" s="7" t="n"/>
@@ -1066,15 +1066,15 @@
     </row>
     <row r="33">
       <c r="A33" s="6" t="n">
-        <v>29</v>
-      </c>
-      <c r="B33" s="7" t="n"/>
+        <v>28</v>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>D'Andre Swift</t>
+        </is>
+      </c>
       <c r="C33" s="7" t="n"/>
-      <c r="D33" s="7" t="inlineStr">
-        <is>
-          <t>Parker Washington</t>
-        </is>
-      </c>
+      <c r="D33" s="7" t="n"/>
       <c r="E33" s="7" t="n"/>
       <c r="F33" s="7" t="n"/>
       <c r="G33" s="7" t="n"/>
@@ -1084,13 +1084,13 @@
       <c r="A34" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="B34" s="7" t="inlineStr">
-        <is>
-          <t>Cam Skattebo</t>
-        </is>
-      </c>
+      <c r="B34" s="7" t="n"/>
       <c r="C34" s="7" t="n"/>
-      <c r="D34" s="7" t="n"/>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>DeVonta Smith</t>
+        </is>
+      </c>
       <c r="E34" s="7" t="n"/>
       <c r="F34" s="7" t="n"/>
       <c r="G34" s="7" t="n"/>
@@ -1100,13 +1100,13 @@
       <c r="A35" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="B35" s="7" t="inlineStr">
-        <is>
-          <t>Aaron Jones Sr.</t>
-        </is>
-      </c>
+      <c r="B35" s="7" t="n"/>
       <c r="C35" s="7" t="n"/>
-      <c r="D35" s="7" t="n"/>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>Davante Adams</t>
+        </is>
+      </c>
       <c r="E35" s="7" t="n"/>
       <c r="F35" s="7" t="n"/>
       <c r="G35" s="7" t="n"/>
@@ -1120,7 +1120,7 @@
       <c r="C36" s="7" t="n"/>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>George Pickens</t>
+          <t>A.J. Brown</t>
         </is>
       </c>
       <c r="E36" s="7" t="n"/>
@@ -1130,13 +1130,13 @@
     </row>
     <row r="37">
       <c r="A37" s="6" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B37" s="7" t="n"/>
       <c r="C37" s="7" t="n"/>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>A.J. Brown</t>
+          <t>Zay Flowers</t>
         </is>
       </c>
       <c r="E37" s="7" t="n"/>
@@ -1148,13 +1148,13 @@
       <c r="A38" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="B38" s="7" t="n"/>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Aaron Jones Sr.</t>
+        </is>
+      </c>
       <c r="C38" s="7" t="n"/>
-      <c r="D38" s="7" t="inlineStr">
-        <is>
-          <t>Tetairoa McMillan</t>
-        </is>
-      </c>
+      <c r="D38" s="7" t="n"/>
       <c r="E38" s="7" t="n"/>
       <c r="F38" s="7" t="n"/>
       <c r="G38" s="7" t="n"/>
@@ -1162,15 +1162,15 @@
     </row>
     <row r="39">
       <c r="A39" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="B39" s="7" t="inlineStr">
-        <is>
-          <t>Jeremiyah Love</t>
-        </is>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="B39" s="7" t="n"/>
       <c r="C39" s="7" t="n"/>
-      <c r="D39" s="7" t="n"/>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>Tetairoa McMillan</t>
+        </is>
+      </c>
       <c r="E39" s="7" t="n"/>
       <c r="F39" s="7" t="n"/>
       <c r="G39" s="7" t="n"/>
@@ -1178,13 +1178,13 @@
     </row>
     <row r="40">
       <c r="A40" s="6" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B40" s="7" t="n"/>
       <c r="C40" s="7" t="n"/>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>Tee Higgins</t>
+          <t>Parker Washington</t>
         </is>
       </c>
       <c r="E40" s="7" t="n"/>
@@ -1194,15 +1194,15 @@
     </row>
     <row r="41">
       <c r="A41" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="B41" s="7" t="inlineStr">
-        <is>
-          <t>Chuba Hubbard</t>
-        </is>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="B41" s="7" t="n"/>
       <c r="C41" s="7" t="n"/>
-      <c r="D41" s="7" t="n"/>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>Tee Higgins</t>
+        </is>
+      </c>
       <c r="E41" s="7" t="n"/>
       <c r="F41" s="7" t="n"/>
       <c r="G41" s="7" t="n"/>
@@ -1216,7 +1216,7 @@
       <c r="C42" s="7" t="n"/>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>Malik Nabers</t>
+          <t>Rashee Rice</t>
         </is>
       </c>
       <c r="E42" s="7" t="n"/>
@@ -1226,47 +1226,47 @@
     </row>
     <row r="43">
       <c r="A43" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="B43" s="7" t="n"/>
+        <v>21</v>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Omarion Hampton</t>
+        </is>
+      </c>
       <c r="C43" s="7" t="n"/>
       <c r="D43" s="7" t="n"/>
       <c r="E43" s="7" t="n"/>
       <c r="F43" s="7" t="n"/>
       <c r="G43" s="7" t="n"/>
-      <c r="H43" s="7" t="inlineStr">
-        <is>
-          <t>Lamar Jackson</t>
-        </is>
-      </c>
+      <c r="H43" s="7" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="B44" s="7" t="n"/>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Cam Skattebo</t>
+        </is>
+      </c>
       <c r="C44" s="7" t="n"/>
       <c r="D44" s="7" t="n"/>
       <c r="E44" s="7" t="n"/>
-      <c r="F44" s="7" t="inlineStr">
-        <is>
-          <t>Brock Bowers</t>
-        </is>
-      </c>
+      <c r="F44" s="7" t="n"/>
       <c r="G44" s="7" t="n"/>
       <c r="H44" s="7" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="B45" s="7" t="inlineStr">
-        <is>
-          <t>Omarion Hampton</t>
-        </is>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="B45" s="7" t="n"/>
       <c r="C45" s="7" t="n"/>
-      <c r="D45" s="7" t="n"/>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>Malik Nabers</t>
+        </is>
+      </c>
       <c r="E45" s="7" t="n"/>
       <c r="F45" s="7" t="n"/>
       <c r="G45" s="7" t="n"/>
@@ -1274,7 +1274,7 @@
     </row>
     <row r="46">
       <c r="A46" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
@@ -1290,29 +1290,29 @@
     </row>
     <row r="47">
       <c r="A47" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B47" s="7" t="n"/>
       <c r="C47" s="7" t="n"/>
-      <c r="D47" s="7" t="inlineStr">
-        <is>
-          <t>Christian Watson</t>
-        </is>
-      </c>
+      <c r="D47" s="7" t="n"/>
       <c r="E47" s="7" t="n"/>
       <c r="F47" s="7" t="n"/>
       <c r="G47" s="7" t="n"/>
-      <c r="H47" s="7" t="n"/>
+      <c r="H47" s="7" t="inlineStr">
+        <is>
+          <t>Lamar Jackson</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B48" s="7" t="n"/>
       <c r="C48" s="7" t="n"/>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>Jaylen Waddle</t>
+          <t>Christian Watson</t>
         </is>
       </c>
       <c r="E48" s="7" t="n"/>
@@ -1324,29 +1324,29 @@
       <c r="A49" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="B49" s="7" t="n"/>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Chuba Hubbard</t>
+        </is>
+      </c>
       <c r="C49" s="7" t="n"/>
       <c r="D49" s="7" t="n"/>
       <c r="E49" s="7" t="n"/>
-      <c r="F49" s="7" t="inlineStr">
-        <is>
-          <t>Tyler Warren</t>
-        </is>
-      </c>
+      <c r="F49" s="7" t="n"/>
       <c r="G49" s="7" t="n"/>
       <c r="H49" s="7" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="B50" s="7" t="inlineStr">
-        <is>
-          <t>Bucky Irving</t>
-        </is>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="B50" s="7" t="n"/>
       <c r="C50" s="7" t="n"/>
-      <c r="D50" s="7" t="n"/>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>Jaylen Waddle</t>
+        </is>
+      </c>
       <c r="E50" s="7" t="n"/>
       <c r="F50" s="7" t="n"/>
       <c r="G50" s="7" t="n"/>
@@ -1356,13 +1356,13 @@
       <c r="A51" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="B51" s="7" t="n"/>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>Bucky Irving</t>
+        </is>
+      </c>
       <c r="C51" s="7" t="n"/>
-      <c r="D51" s="7" t="inlineStr">
-        <is>
-          <t>Rashee Rice</t>
-        </is>
-      </c>
+      <c r="D51" s="7" t="n"/>
       <c r="E51" s="7" t="n"/>
       <c r="F51" s="7" t="n"/>
       <c r="G51" s="7" t="n"/>
@@ -1378,7 +1378,7 @@
       <c r="E52" s="7" t="n"/>
       <c r="F52" s="7" t="inlineStr">
         <is>
-          <t>George Kittle</t>
+          <t>Tyler Warren</t>
         </is>
       </c>
       <c r="G52" s="7" t="n"/>
@@ -1388,13 +1388,13 @@
       <c r="A53" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B53" s="7" t="n"/>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>Quinshon Judkins</t>
+        </is>
+      </c>
       <c r="C53" s="7" t="n"/>
-      <c r="D53" s="7" t="inlineStr">
-        <is>
-          <t>Zay Flowers</t>
-        </is>
-      </c>
+      <c r="D53" s="7" t="n"/>
       <c r="E53" s="7" t="n"/>
       <c r="F53" s="7" t="n"/>
       <c r="G53" s="7" t="n"/>
@@ -1402,15 +1402,15 @@
     </row>
     <row r="54">
       <c r="A54" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="B54" s="7" t="inlineStr">
-        <is>
-          <t>Quinshon Judkins</t>
-        </is>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="B54" s="7" t="n"/>
       <c r="C54" s="7" t="n"/>
-      <c r="D54" s="7" t="n"/>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>Ladd McConkey</t>
+        </is>
+      </c>
       <c r="E54" s="7" t="n"/>
       <c r="F54" s="7" t="n"/>
       <c r="G54" s="7" t="n"/>
@@ -1418,11 +1418,11 @@
     </row>
     <row r="55">
       <c r="A55" s="6" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>David Montgomery</t>
+          <t>Travis Etienne Jr.</t>
         </is>
       </c>
       <c r="C55" s="7" t="n"/>
@@ -1440,7 +1440,7 @@
       <c r="C56" s="7" t="n"/>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>Matthew Golden</t>
+          <t>Mike Evans</t>
         </is>
       </c>
       <c r="E56" s="7" t="n"/>
@@ -1450,13 +1450,13 @@
     </row>
     <row r="57">
       <c r="A57" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B57" s="7" t="n"/>
       <c r="C57" s="7" t="n"/>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>Terry McLaurin</t>
+          <t>Michael Wilson</t>
         </is>
       </c>
       <c r="E57" s="7" t="n"/>
@@ -1466,15 +1466,15 @@
     </row>
     <row r="58">
       <c r="A58" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="B58" s="7" t="n"/>
+        <v>11</v>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>David Montgomery</t>
+        </is>
+      </c>
       <c r="C58" s="7" t="n"/>
-      <c r="D58" s="7" t="inlineStr">
-        <is>
-          <t>Mike Evans</t>
-        </is>
-      </c>
+      <c r="D58" s="7" t="n"/>
       <c r="E58" s="7" t="n"/>
       <c r="F58" s="7" t="n"/>
       <c r="G58" s="7" t="n"/>
@@ -1482,13 +1482,13 @@
     </row>
     <row r="59">
       <c r="A59" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B59" s="7" t="n"/>
       <c r="C59" s="7" t="n"/>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>Ladd McConkey</t>
+          <t>Emeka Egbuka</t>
         </is>
       </c>
       <c r="E59" s="7" t="n"/>
@@ -1498,15 +1498,15 @@
     </row>
     <row r="60">
       <c r="A60" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="B60" s="7" t="inlineStr">
-        <is>
-          <t>Bhayshul Tuten</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="B60" s="7" t="n"/>
       <c r="C60" s="7" t="n"/>
-      <c r="D60" s="7" t="n"/>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
+          <t>Luther Burden III</t>
+        </is>
+      </c>
       <c r="E60" s="7" t="n"/>
       <c r="F60" s="7" t="n"/>
       <c r="G60" s="7" t="n"/>
@@ -1514,15 +1514,15 @@
     </row>
     <row r="61">
       <c r="A61" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="B61" s="7" t="inlineStr">
-        <is>
-          <t>Travis Etienne Jr.</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="B61" s="7" t="n"/>
       <c r="C61" s="7" t="n"/>
-      <c r="D61" s="7" t="n"/>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>Terry McLaurin</t>
+        </is>
+      </c>
       <c r="E61" s="7" t="n"/>
       <c r="F61" s="7" t="n"/>
       <c r="G61" s="7" t="n"/>
@@ -1530,15 +1530,15 @@
     </row>
     <row r="62">
       <c r="A62" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="B62" s="7" t="inlineStr">
-        <is>
-          <t>Jadarian Price</t>
-        </is>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="B62" s="7" t="n"/>
       <c r="C62" s="7" t="n"/>
-      <c r="D62" s="7" t="n"/>
+      <c r="D62" s="7" t="inlineStr">
+        <is>
+          <t>DJ Moore</t>
+        </is>
+      </c>
       <c r="E62" s="7" t="n"/>
       <c r="F62" s="7" t="n"/>
       <c r="G62" s="7" t="n"/>
@@ -1546,13 +1546,13 @@
     </row>
     <row r="63">
       <c r="A63" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B63" s="7" t="n"/>
       <c r="C63" s="7" t="n"/>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>Emeka Egbuka</t>
+          <t>Matthew Golden</t>
         </is>
       </c>
       <c r="E63" s="7" t="n"/>
@@ -1568,7 +1568,7 @@
       <c r="C64" s="7" t="n"/>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>Michael Wilson</t>
+          <t>Jameson Williams</t>
         </is>
       </c>
       <c r="E64" s="7" t="n"/>
@@ -1578,13 +1578,13 @@
     </row>
     <row r="65">
       <c r="A65" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B65" s="7" t="n"/>
       <c r="C65" s="7" t="n"/>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>DJ Moore</t>
+          <t>De'Zhaun Stribling</t>
         </is>
       </c>
       <c r="E65" s="7" t="n"/>
@@ -1596,13 +1596,13 @@
       <c r="A66" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B66" s="7" t="n"/>
+      <c r="B66" s="7" t="inlineStr">
+        <is>
+          <t>Bhayshul Tuten</t>
+        </is>
+      </c>
       <c r="C66" s="7" t="n"/>
-      <c r="D66" s="7" t="inlineStr">
-        <is>
-          <t>Luther Burden III</t>
-        </is>
-      </c>
+      <c r="D66" s="7" t="n"/>
       <c r="E66" s="7" t="n"/>
       <c r="F66" s="7" t="n"/>
       <c r="G66" s="7" t="n"/>
@@ -1612,29 +1612,29 @@
       <c r="A67" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B67" s="7" t="n"/>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>Rhamondre Stevenson</t>
+        </is>
+      </c>
       <c r="C67" s="7" t="n"/>
       <c r="D67" s="7" t="n"/>
       <c r="E67" s="7" t="n"/>
       <c r="F67" s="7" t="n"/>
       <c r="G67" s="7" t="n"/>
-      <c r="H67" s="7" t="inlineStr">
-        <is>
-          <t>Drake Maye</t>
-        </is>
-      </c>
+      <c r="H67" s="7" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B68" s="7" t="inlineStr">
-        <is>
-          <t>Rhamondre Stevenson</t>
-        </is>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="B68" s="7" t="n"/>
       <c r="C68" s="7" t="n"/>
-      <c r="D68" s="7" t="n"/>
+      <c r="D68" s="7" t="inlineStr">
+        <is>
+          <t>Carnell Tate</t>
+        </is>
+      </c>
       <c r="E68" s="7" t="n"/>
       <c r="F68" s="7" t="n"/>
       <c r="G68" s="7" t="n"/>
@@ -1644,13 +1644,13 @@
       <c r="A69" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B69" s="7" t="n"/>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>Jadarian Price</t>
+        </is>
+      </c>
       <c r="C69" s="7" t="n"/>
-      <c r="D69" s="7" t="inlineStr">
-        <is>
-          <t>Carnell Tate</t>
-        </is>
-      </c>
+      <c r="D69" s="7" t="n"/>
       <c r="E69" s="7" t="n"/>
       <c r="F69" s="7" t="n"/>
       <c r="G69" s="7" t="n"/>
@@ -1664,7 +1664,7 @@
       <c r="C70" s="7" t="n"/>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>Stefon Diggs</t>
+          <t>Alec Pierce</t>
         </is>
       </c>
       <c r="E70" s="7" t="n"/>
@@ -1674,15 +1674,15 @@
     </row>
     <row r="71">
       <c r="A71" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B71" s="7" t="inlineStr">
-        <is>
-          <t>Josh Jacobs</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="B71" s="7" t="n"/>
       <c r="C71" s="7" t="n"/>
-      <c r="D71" s="7" t="n"/>
+      <c r="D71" s="7" t="inlineStr">
+        <is>
+          <t>Stefon Diggs</t>
+        </is>
+      </c>
       <c r="E71" s="7" t="n"/>
       <c r="F71" s="7" t="n"/>
       <c r="G71" s="7" t="n"/>
@@ -1690,99 +1690,99 @@
     </row>
     <row r="72">
       <c r="A72" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B72" s="7" t="n"/>
       <c r="C72" s="7" t="n"/>
-      <c r="D72" s="7" t="inlineStr">
-        <is>
-          <t>Jameson Williams</t>
-        </is>
-      </c>
+      <c r="D72" s="7" t="n"/>
       <c r="E72" s="7" t="n"/>
-      <c r="F72" s="7" t="n"/>
+      <c r="F72" s="7" t="inlineStr">
+        <is>
+          <t>Colston Loveland</t>
+        </is>
+      </c>
       <c r="G72" s="7" t="n"/>
       <c r="H72" s="7" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B73" s="7" t="n"/>
       <c r="C73" s="7" t="n"/>
-      <c r="D73" s="7" t="inlineStr">
-        <is>
-          <t>De'Zhaun Stribling</t>
-        </is>
-      </c>
+      <c r="D73" s="7" t="n"/>
       <c r="E73" s="7" t="n"/>
-      <c r="F73" s="7" t="n"/>
+      <c r="F73" s="7" t="inlineStr">
+        <is>
+          <t>George Kittle</t>
+        </is>
+      </c>
       <c r="G73" s="7" t="n"/>
       <c r="H73" s="7" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B74" s="7" t="n"/>
       <c r="C74" s="7" t="n"/>
       <c r="D74" s="7" t="n"/>
       <c r="E74" s="7" t="n"/>
-      <c r="F74" s="7" t="inlineStr">
-        <is>
-          <t>Colston Loveland</t>
-        </is>
-      </c>
+      <c r="F74" s="7" t="n"/>
       <c r="G74" s="7" t="n"/>
-      <c r="H74" s="7" t="n"/>
+      <c r="H74" s="7" t="inlineStr">
+        <is>
+          <t>Drake Maye</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B75" s="7" t="n"/>
+        <v>4</v>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>MarShawn Lloyd</t>
+        </is>
+      </c>
       <c r="C75" s="7" t="n"/>
       <c r="D75" s="7" t="n"/>
       <c r="E75" s="7" t="n"/>
-      <c r="F75" s="7" t="inlineStr">
-        <is>
-          <t>Isaiah Likely</t>
-        </is>
-      </c>
+      <c r="F75" s="7" t="n"/>
       <c r="G75" s="7" t="n"/>
       <c r="H75" s="7" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B76" s="7" t="n"/>
+        <v>4</v>
+      </c>
+      <c r="B76" s="7" t="inlineStr">
+        <is>
+          <t>TreVeyon Henderson</t>
+        </is>
+      </c>
       <c r="C76" s="7" t="n"/>
       <c r="D76" s="7" t="n"/>
       <c r="E76" s="7" t="n"/>
       <c r="F76" s="7" t="n"/>
       <c r="G76" s="7" t="n"/>
-      <c r="H76" s="7" t="inlineStr">
-        <is>
-          <t>Jayden Daniels</t>
-        </is>
-      </c>
+      <c r="H76" s="7" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B77" s="7" t="n"/>
+        <v>4</v>
+      </c>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>Josh Jacobs</t>
+        </is>
+      </c>
       <c r="C77" s="7" t="n"/>
       <c r="D77" s="7" t="n"/>
       <c r="E77" s="7" t="n"/>
       <c r="F77" s="7" t="n"/>
       <c r="G77" s="7" t="n"/>
-      <c r="H77" s="7" t="inlineStr">
-        <is>
-          <t>Dak Prescott</t>
-        </is>
-      </c>
+      <c r="H77" s="7" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="6" t="n">
@@ -1790,7 +1790,7 @@
       </c>
       <c r="B78" s="7" t="inlineStr">
         <is>
-          <t>Tony Pollard</t>
+          <t>Kenny Gainwell</t>
         </is>
       </c>
       <c r="C78" s="7" t="n"/>
@@ -1804,13 +1804,13 @@
       <c r="A79" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B79" s="7" t="inlineStr">
-        <is>
-          <t>Kenny Gainwell</t>
-        </is>
-      </c>
+      <c r="B79" s="7" t="n"/>
       <c r="C79" s="7" t="n"/>
-      <c r="D79" s="7" t="n"/>
+      <c r="D79" s="7" t="inlineStr">
+        <is>
+          <t>Rome Odunze</t>
+        </is>
+      </c>
       <c r="E79" s="7" t="n"/>
       <c r="F79" s="7" t="n"/>
       <c r="G79" s="7" t="n"/>
@@ -1824,7 +1824,7 @@
       <c r="C80" s="7" t="n"/>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>Rome Odunze</t>
+          <t>KC Concepcion</t>
         </is>
       </c>
       <c r="E80" s="7" t="n"/>
@@ -1838,27 +1838,27 @@
       </c>
       <c r="B81" s="7" t="n"/>
       <c r="C81" s="7" t="n"/>
-      <c r="D81" s="7" t="n"/>
+      <c r="D81" s="7" t="inlineStr">
+        <is>
+          <t>Jayden Reed</t>
+        </is>
+      </c>
       <c r="E81" s="7" t="n"/>
       <c r="F81" s="7" t="n"/>
       <c r="G81" s="7" t="n"/>
-      <c r="H81" s="7" t="inlineStr">
-        <is>
-          <t>Joe Burrow</t>
-        </is>
-      </c>
+      <c r="H81" s="7" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B82" s="7" t="inlineStr">
-        <is>
-          <t>MarShawn Lloyd</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="B82" s="7" t="n"/>
       <c r="C82" s="7" t="n"/>
-      <c r="D82" s="7" t="n"/>
+      <c r="D82" s="7" t="inlineStr">
+        <is>
+          <t>Jordyn Tyson</t>
+        </is>
+      </c>
       <c r="E82" s="7" t="n"/>
       <c r="F82" s="7" t="n"/>
       <c r="G82" s="7" t="n"/>
@@ -1866,35 +1866,35 @@
     </row>
     <row r="83">
       <c r="A83" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B83" s="7" t="inlineStr">
-        <is>
-          <t>TreVeyon Henderson</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="B83" s="7" t="n"/>
       <c r="C83" s="7" t="n"/>
       <c r="D83" s="7" t="n"/>
       <c r="E83" s="7" t="n"/>
       <c r="F83" s="7" t="n"/>
       <c r="G83" s="7" t="n"/>
-      <c r="H83" s="7" t="n"/>
+      <c r="H83" s="7" t="inlineStr">
+        <is>
+          <t>Joe Burrow</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B84" s="7" t="inlineStr">
-        <is>
-          <t>Jordan Mason</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="B84" s="7" t="n"/>
       <c r="C84" s="7" t="n"/>
       <c r="D84" s="7" t="n"/>
       <c r="E84" s="7" t="n"/>
       <c r="F84" s="7" t="n"/>
       <c r="G84" s="7" t="n"/>
-      <c r="H84" s="7" t="n"/>
+      <c r="H84" s="7" t="inlineStr">
+        <is>
+          <t>Jayden Daniels</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="6" t="n">
@@ -1920,7 +1920,7 @@
       <c r="C86" s="7" t="n"/>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>Alec Pierce</t>
+          <t>DK Metcalf</t>
         </is>
       </c>
       <c r="E86" s="7" t="n"/>
@@ -1930,43 +1930,43 @@
     </row>
     <row r="87">
       <c r="A87" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B87" s="7" t="inlineStr">
-        <is>
-          <t>Jonathon Brooks</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="B87" s="7" t="n"/>
       <c r="C87" s="7" t="n"/>
       <c r="D87" s="7" t="n"/>
       <c r="E87" s="7" t="n"/>
-      <c r="F87" s="7" t="n"/>
+      <c r="F87" s="7" t="inlineStr">
+        <is>
+          <t>Isaiah Likely</t>
+        </is>
+      </c>
       <c r="G87" s="7" t="n"/>
       <c r="H87" s="7" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B88" s="7" t="inlineStr">
-        <is>
-          <t>Mike Washington Jr.</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="B88" s="7" t="n"/>
       <c r="C88" s="7" t="n"/>
       <c r="D88" s="7" t="n"/>
       <c r="E88" s="7" t="n"/>
       <c r="F88" s="7" t="n"/>
       <c r="G88" s="7" t="n"/>
-      <c r="H88" s="7" t="n"/>
+      <c r="H88" s="7" t="inlineStr">
+        <is>
+          <t>Dak Prescott</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B89" s="7" t="inlineStr">
         <is>
-          <t>Rico Dowdle</t>
+          <t>Jordan Mason</t>
         </is>
       </c>
       <c r="C89" s="7" t="n"/>
@@ -1978,11 +1978,11 @@
     </row>
     <row r="90">
       <c r="A90" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B90" s="7" t="inlineStr">
         <is>
-          <t>Jacory Croskey-Merritt</t>
+          <t>J.K. Dobbins</t>
         </is>
       </c>
       <c r="C90" s="7" t="n"/>
@@ -1994,11 +1994,11 @@
     </row>
     <row r="91">
       <c r="A91" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B91" s="7" t="inlineStr">
         <is>
-          <t>J.K. Dobbins</t>
+          <t>Jacory Croskey-Merritt</t>
         </is>
       </c>
       <c r="C91" s="7" t="n"/>
@@ -2014,7 +2014,7 @@
       </c>
       <c r="B92" s="7" t="inlineStr">
         <is>
-          <t>Blake Corum</t>
+          <t>Tony Pollard</t>
         </is>
       </c>
       <c r="C92" s="7" t="n"/>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="B93" s="7" t="inlineStr">
         <is>
-          <t>Woody Marks</t>
+          <t>Jonathon Brooks</t>
         </is>
       </c>
       <c r="C93" s="7" t="n"/>
@@ -2044,13 +2044,13 @@
       <c r="A94" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B94" s="7" t="n"/>
+      <c r="B94" s="7" t="inlineStr">
+        <is>
+          <t>Mike Washington Jr.</t>
+        </is>
+      </c>
       <c r="C94" s="7" t="n"/>
-      <c r="D94" s="7" t="inlineStr">
-        <is>
-          <t>Marvin Harrison Jr.</t>
-        </is>
-      </c>
+      <c r="D94" s="7" t="n"/>
       <c r="E94" s="7" t="n"/>
       <c r="F94" s="7" t="n"/>
       <c r="G94" s="7" t="n"/>
@@ -2060,13 +2060,13 @@
       <c r="A95" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B95" s="7" t="n"/>
+      <c r="B95" s="7" t="inlineStr">
+        <is>
+          <t>Rico Dowdle</t>
+        </is>
+      </c>
       <c r="C95" s="7" t="n"/>
-      <c r="D95" s="7" t="inlineStr">
-        <is>
-          <t>KC Concepcion</t>
-        </is>
-      </c>
+      <c r="D95" s="7" t="n"/>
       <c r="E95" s="7" t="n"/>
       <c r="F95" s="7" t="n"/>
       <c r="G95" s="7" t="n"/>
@@ -2076,13 +2076,13 @@
       <c r="A96" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B96" s="7" t="n"/>
+      <c r="B96" s="7" t="inlineStr">
+        <is>
+          <t>Blake Corum</t>
+        </is>
+      </c>
       <c r="C96" s="7" t="n"/>
-      <c r="D96" s="7" t="inlineStr">
-        <is>
-          <t>Quentin Johnston</t>
-        </is>
-      </c>
+      <c r="D96" s="7" t="n"/>
       <c r="E96" s="7" t="n"/>
       <c r="F96" s="7" t="n"/>
       <c r="G96" s="7" t="n"/>
@@ -2092,13 +2092,13 @@
       <c r="A97" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B97" s="7" t="n"/>
+      <c r="B97" s="7" t="inlineStr">
+        <is>
+          <t>Woody Marks</t>
+        </is>
+      </c>
       <c r="C97" s="7" t="n"/>
-      <c r="D97" s="7" t="inlineStr">
-        <is>
-          <t>Chris Godwin Jr.</t>
-        </is>
-      </c>
+      <c r="D97" s="7" t="n"/>
       <c r="E97" s="7" t="n"/>
       <c r="F97" s="7" t="n"/>
       <c r="G97" s="7" t="n"/>
@@ -2112,7 +2112,7 @@
       <c r="C98" s="7" t="n"/>
       <c r="D98" s="7" t="inlineStr">
         <is>
-          <t>Jayden Reed</t>
+          <t>Brian Thomas Jr.</t>
         </is>
       </c>
       <c r="E98" s="7" t="n"/>
@@ -2128,7 +2128,7 @@
       <c r="C99" s="7" t="n"/>
       <c r="D99" s="7" t="inlineStr">
         <is>
-          <t>Jordyn Tyson</t>
+          <t>Marvin Harrison Jr.</t>
         </is>
       </c>
       <c r="E99" s="7" t="n"/>
@@ -2144,7 +2144,7 @@
       <c r="C100" s="7" t="n"/>
       <c r="D100" s="7" t="inlineStr">
         <is>
-          <t>Brian Thomas Jr.</t>
+          <t>Quentin Johnston</t>
         </is>
       </c>
       <c r="E100" s="7" t="n"/>
@@ -2160,7 +2160,7 @@
       <c r="C101" s="7" t="n"/>
       <c r="D101" s="7" t="inlineStr">
         <is>
-          <t>DK Metcalf</t>
+          <t>Chris Godwin Jr.</t>
         </is>
       </c>
       <c r="E101" s="7" t="n"/>
@@ -2311,7 +2311,7 @@
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>Baseline: the live Trade Values Google Sheet (Half PPR, 10-team), 105 players, top value 77.</t>
+          <t>Baseline: the live Trade Values Google Sheet (Half PPR, 10-team), 105 players, top value 76.</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2335,7 @@
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   (Projections page snapshot 0; 32 players used week 3 medians): implied = 0.7 x the seed value at the player's projection-rank slot among the projected players at the position + 0.3 x</t>
+          <t xml:space="preserve">   (Projections page snapshot 1; 13 players used week 3 medians): implied = 0.7 x the seed value at the player's projection-rank slot among the projected players at the position + 0.3 x</t>
         </is>
       </c>
     </row>
@@ -2349,14 +2349,14 @@
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   new = sheet + 0.6 x (implied - sheet), then rescaled so the total equals the sheet total. 79 players moved.</t>
+          <t xml:space="preserve">   new = sheet + 0.45 x (implied - sheet), then rescaled so the total equals the sheet total. 83 players moved.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   No projection this week (value kept): Puka Nacua, Josh Jacobs, De'Zhaun Stribling, Jayden Daniels, Jordan Mason, Alec Pierce, Jonathon Brooks, Jayden Reed, Mike Washington Jr., Jordyn Tyson, Rico Dowdle, Jaxson Dart, Ja'Kobi Lane.</t>
+          <t xml:space="preserve">   No projection this week (value kept): Josh Jacobs, De'Zhaun Stribling, Jayden Daniels, Jordan Mason, Alec Pierce, Jonathon Brooks, Jayden Reed, Mike Washington Jr., Jordyn Tyson, Rico Dowdle, Jaxson Dart, Ja'Kobi Lane.</t>
         </is>
       </c>
     </row>
@@ -2408,7 +2408,7 @@
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Replacement level = average line of baseline players valued 5 or less at the position: RB 1.9, WR 3.1, TE 4.5, QB 0.0.</t>
+          <t xml:space="preserve">   Replacement level = average line of baseline players valued 5 or less at the position: RB 1.8, WR 2.9, TE 4.5, QB 0.0.</t>
         </is>
       </c>
     </row>
@@ -2435,7 +2435,7 @@
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>Largest moves vs. the baseline in this file: James Cook III 56-&gt;49, Derrick Henry 57-&gt;50, Josh Allen 37-&gt;31, Jonathan Taylor 63-&gt;58, Kenneth Walker III 62-&gt;57, Lamar Jackson 27-&gt;22, Bijan Robinson 72-&gt;68, Jahmyr Gibbs 77-&gt;73</t>
+          <t>Largest moves vs. the baseline in this file: James Cook III 52-&gt;44, Derrick Henry 57-&gt;49, Josh Allen 38-&gt;31, Omarion Hampton 27-&gt;21, Kyren Williams 26-&gt;20, Lamar Jackson 26-&gt;20, Bhayshul Tuten 12-&gt;7, Jonathan Taylor 63-&gt;59</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Trade values: manual overrides file; Allen 41, McBride 40, Bowers 35, Maye 7, Achane removed
overrides.json is applied on top of the Google Sheet every build (set a
baseline value or remove a player); unknown names stop the build.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TradeValueSheets/TradeValues_FullPPR_10team.xlsx
+++ b/TradeValueSheets/TradeValues_FullPPR_10team.xlsx
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H108"/>
+  <dimension ref="A1:H107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -876,15 +876,15 @@
       <c r="A21" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>De'Von Achane</t>
-        </is>
-      </c>
+      <c r="B21" s="7" t="n"/>
       <c r="C21" s="7" t="n"/>
       <c r="D21" s="7" t="n"/>
       <c r="E21" s="7" t="n"/>
-      <c r="F21" s="7" t="n"/>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>Trey McBride</t>
+        </is>
+      </c>
       <c r="G21" s="7" t="n"/>
       <c r="H21" s="7" t="n"/>
     </row>
@@ -944,13 +944,13 @@
       <c r="C25" s="7" t="n"/>
       <c r="D25" s="7" t="n"/>
       <c r="E25" s="7" t="n"/>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>Trey McBride</t>
-        </is>
-      </c>
+      <c r="F25" s="7" t="n"/>
       <c r="G25" s="7" t="n"/>
-      <c r="H25" s="7" t="n"/>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>Josh Allen</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="n">
@@ -970,7 +970,7 @@
     </row>
     <row r="27">
       <c r="A27" s="6" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B27" s="7" t="n"/>
       <c r="C27" s="7" t="n"/>
@@ -986,19 +986,19 @@
     </row>
     <row r="28">
       <c r="A28" s="6" t="n">
-        <v>31</v>
-      </c>
-      <c r="B28" s="7" t="n"/>
+        <v>30</v>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Jeremiyah Love</t>
+        </is>
+      </c>
       <c r="C28" s="7" t="n"/>
       <c r="D28" s="7" t="n"/>
       <c r="E28" s="7" t="n"/>
       <c r="F28" s="7" t="n"/>
       <c r="G28" s="7" t="n"/>
-      <c r="H28" s="7" t="inlineStr">
-        <is>
-          <t>Josh Allen</t>
-        </is>
-      </c>
+      <c r="H28" s="7" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="n">
@@ -1006,7 +1006,7 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Jeremiyah Love</t>
+          <t>Jaylen Warren</t>
         </is>
       </c>
       <c r="C29" s="7" t="n"/>
@@ -1018,11 +1018,11 @@
     </row>
     <row r="30">
       <c r="A30" s="6" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Jaylen Warren</t>
+          <t>Javonte Williams</t>
         </is>
       </c>
       <c r="C30" s="7" t="n"/>
@@ -1036,13 +1036,13 @@
       <c r="A31" s="6" t="n">
         <v>29</v>
       </c>
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>Javonte Williams</t>
-        </is>
-      </c>
+      <c r="B31" s="7" t="n"/>
       <c r="C31" s="7" t="n"/>
-      <c r="D31" s="7" t="n"/>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>George Pickens</t>
+        </is>
+      </c>
       <c r="E31" s="7" t="n"/>
       <c r="F31" s="7" t="n"/>
       <c r="G31" s="7" t="n"/>
@@ -1050,15 +1050,15 @@
     </row>
     <row r="32">
       <c r="A32" s="6" t="n">
-        <v>29</v>
-      </c>
-      <c r="B32" s="7" t="n"/>
+        <v>28</v>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>D'Andre Swift</t>
+        </is>
+      </c>
       <c r="C32" s="7" t="n"/>
-      <c r="D32" s="7" t="inlineStr">
-        <is>
-          <t>George Pickens</t>
-        </is>
-      </c>
+      <c r="D32" s="7" t="n"/>
       <c r="E32" s="7" t="n"/>
       <c r="F32" s="7" t="n"/>
       <c r="G32" s="7" t="n"/>
@@ -1068,13 +1068,13 @@
       <c r="A33" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="B33" s="7" t="inlineStr">
-        <is>
-          <t>D'Andre Swift</t>
-        </is>
-      </c>
+      <c r="B33" s="7" t="n"/>
       <c r="C33" s="7" t="n"/>
-      <c r="D33" s="7" t="n"/>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>DeVonta Smith</t>
+        </is>
+      </c>
       <c r="E33" s="7" t="n"/>
       <c r="F33" s="7" t="n"/>
       <c r="G33" s="7" t="n"/>
@@ -1088,7 +1088,7 @@
       <c r="C34" s="7" t="n"/>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>DeVonta Smith</t>
+          <t>Davante Adams</t>
         </is>
       </c>
       <c r="E34" s="7" t="n"/>
@@ -1098,13 +1098,13 @@
     </row>
     <row r="35">
       <c r="A35" s="6" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B35" s="7" t="n"/>
       <c r="C35" s="7" t="n"/>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>Davante Adams</t>
+          <t>A.J. Brown</t>
         </is>
       </c>
       <c r="E35" s="7" t="n"/>
@@ -1120,7 +1120,7 @@
       <c r="C36" s="7" t="n"/>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>A.J. Brown</t>
+          <t>Zay Flowers</t>
         </is>
       </c>
       <c r="E36" s="7" t="n"/>
@@ -1130,15 +1130,15 @@
     </row>
     <row r="37">
       <c r="A37" s="6" t="n">
-        <v>27</v>
-      </c>
-      <c r="B37" s="7" t="n"/>
+        <v>25</v>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Aaron Jones Sr.</t>
+        </is>
+      </c>
       <c r="C37" s="7" t="n"/>
-      <c r="D37" s="7" t="inlineStr">
-        <is>
-          <t>Zay Flowers</t>
-        </is>
-      </c>
+      <c r="D37" s="7" t="n"/>
       <c r="E37" s="7" t="n"/>
       <c r="F37" s="7" t="n"/>
       <c r="G37" s="7" t="n"/>
@@ -1148,13 +1148,13 @@
       <c r="A38" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="B38" s="7" t="inlineStr">
-        <is>
-          <t>Aaron Jones Sr.</t>
-        </is>
-      </c>
+      <c r="B38" s="7" t="n"/>
       <c r="C38" s="7" t="n"/>
-      <c r="D38" s="7" t="n"/>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>Tetairoa McMillan</t>
+        </is>
+      </c>
       <c r="E38" s="7" t="n"/>
       <c r="F38" s="7" t="n"/>
       <c r="G38" s="7" t="n"/>
@@ -1168,7 +1168,7 @@
       <c r="C39" s="7" t="n"/>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>Tetairoa McMillan</t>
+          <t>Parker Washington</t>
         </is>
       </c>
       <c r="E39" s="7" t="n"/>
@@ -1178,13 +1178,13 @@
     </row>
     <row r="40">
       <c r="A40" s="6" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B40" s="7" t="n"/>
       <c r="C40" s="7" t="n"/>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>Parker Washington</t>
+          <t>Tee Higgins</t>
         </is>
       </c>
       <c r="E40" s="7" t="n"/>
@@ -1194,13 +1194,13 @@
     </row>
     <row r="41">
       <c r="A41" s="6" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B41" s="7" t="n"/>
       <c r="C41" s="7" t="n"/>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>Tee Higgins</t>
+          <t>Rashee Rice</t>
         </is>
       </c>
       <c r="E41" s="7" t="n"/>
@@ -1210,15 +1210,15 @@
     </row>
     <row r="42">
       <c r="A42" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="B42" s="7" t="n"/>
+        <v>21</v>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Omarion Hampton</t>
+        </is>
+      </c>
       <c r="C42" s="7" t="n"/>
-      <c r="D42" s="7" t="inlineStr">
-        <is>
-          <t>Rashee Rice</t>
-        </is>
-      </c>
+      <c r="D42" s="7" t="n"/>
       <c r="E42" s="7" t="n"/>
       <c r="F42" s="7" t="n"/>
       <c r="G42" s="7" t="n"/>
@@ -1230,7 +1230,7 @@
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Omarion Hampton</t>
+          <t>Cam Skattebo</t>
         </is>
       </c>
       <c r="C43" s="7" t="n"/>
@@ -1244,13 +1244,13 @@
       <c r="A44" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="B44" s="7" t="inlineStr">
-        <is>
-          <t>Cam Skattebo</t>
-        </is>
-      </c>
+      <c r="B44" s="7" t="n"/>
       <c r="C44" s="7" t="n"/>
-      <c r="D44" s="7" t="n"/>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>Malik Nabers</t>
+        </is>
+      </c>
       <c r="E44" s="7" t="n"/>
       <c r="F44" s="7" t="n"/>
       <c r="G44" s="7" t="n"/>
@@ -1258,15 +1258,15 @@
     </row>
     <row r="45">
       <c r="A45" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="B45" s="7" t="n"/>
+        <v>20</v>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Kyren Williams</t>
+        </is>
+      </c>
       <c r="C45" s="7" t="n"/>
-      <c r="D45" s="7" t="inlineStr">
-        <is>
-          <t>Malik Nabers</t>
-        </is>
-      </c>
+      <c r="D45" s="7" t="n"/>
       <c r="E45" s="7" t="n"/>
       <c r="F45" s="7" t="n"/>
       <c r="G45" s="7" t="n"/>
@@ -1276,45 +1276,45 @@
       <c r="A46" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="B46" s="7" t="inlineStr">
-        <is>
-          <t>Kyren Williams</t>
-        </is>
-      </c>
+      <c r="B46" s="7" t="n"/>
       <c r="C46" s="7" t="n"/>
       <c r="D46" s="7" t="n"/>
       <c r="E46" s="7" t="n"/>
       <c r="F46" s="7" t="n"/>
       <c r="G46" s="7" t="n"/>
-      <c r="H46" s="7" t="n"/>
+      <c r="H46" s="7" t="inlineStr">
+        <is>
+          <t>Lamar Jackson</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B47" s="7" t="n"/>
       <c r="C47" s="7" t="n"/>
-      <c r="D47" s="7" t="n"/>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>Christian Watson</t>
+        </is>
+      </c>
       <c r="E47" s="7" t="n"/>
       <c r="F47" s="7" t="n"/>
       <c r="G47" s="7" t="n"/>
-      <c r="H47" s="7" t="inlineStr">
-        <is>
-          <t>Lamar Jackson</t>
-        </is>
-      </c>
+      <c r="H47" s="7" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="B48" s="7" t="n"/>
+        <v>17</v>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Chuba Hubbard</t>
+        </is>
+      </c>
       <c r="C48" s="7" t="n"/>
-      <c r="D48" s="7" t="inlineStr">
-        <is>
-          <t>Christian Watson</t>
-        </is>
-      </c>
+      <c r="D48" s="7" t="n"/>
       <c r="E48" s="7" t="n"/>
       <c r="F48" s="7" t="n"/>
       <c r="G48" s="7" t="n"/>
@@ -1324,13 +1324,13 @@
       <c r="A49" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="B49" s="7" t="inlineStr">
-        <is>
-          <t>Chuba Hubbard</t>
-        </is>
-      </c>
+      <c r="B49" s="7" t="n"/>
       <c r="C49" s="7" t="n"/>
-      <c r="D49" s="7" t="n"/>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>Jaylen Waddle</t>
+        </is>
+      </c>
       <c r="E49" s="7" t="n"/>
       <c r="F49" s="7" t="n"/>
       <c r="G49" s="7" t="n"/>
@@ -1338,15 +1338,15 @@
     </row>
     <row r="50">
       <c r="A50" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="B50" s="7" t="n"/>
+        <v>16</v>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>Bucky Irving</t>
+        </is>
+      </c>
       <c r="C50" s="7" t="n"/>
-      <c r="D50" s="7" t="inlineStr">
-        <is>
-          <t>Jaylen Waddle</t>
-        </is>
-      </c>
+      <c r="D50" s="7" t="n"/>
       <c r="E50" s="7" t="n"/>
       <c r="F50" s="7" t="n"/>
       <c r="G50" s="7" t="n"/>
@@ -1356,31 +1356,31 @@
       <c r="A51" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="B51" s="7" t="inlineStr">
-        <is>
-          <t>Bucky Irving</t>
-        </is>
-      </c>
+      <c r="B51" s="7" t="n"/>
       <c r="C51" s="7" t="n"/>
       <c r="D51" s="7" t="n"/>
       <c r="E51" s="7" t="n"/>
-      <c r="F51" s="7" t="n"/>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>Tyler Warren</t>
+        </is>
+      </c>
       <c r="G51" s="7" t="n"/>
       <c r="H51" s="7" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="B52" s="7" t="n"/>
+        <v>14</v>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>Quinshon Judkins</t>
+        </is>
+      </c>
       <c r="C52" s="7" t="n"/>
       <c r="D52" s="7" t="n"/>
       <c r="E52" s="7" t="n"/>
-      <c r="F52" s="7" t="inlineStr">
-        <is>
-          <t>Tyler Warren</t>
-        </is>
-      </c>
+      <c r="F52" s="7" t="n"/>
       <c r="G52" s="7" t="n"/>
       <c r="H52" s="7" t="n"/>
     </row>
@@ -1388,13 +1388,13 @@
       <c r="A53" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B53" s="7" t="inlineStr">
-        <is>
-          <t>Quinshon Judkins</t>
-        </is>
-      </c>
+      <c r="B53" s="7" t="n"/>
       <c r="C53" s="7" t="n"/>
-      <c r="D53" s="7" t="n"/>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>Ladd McConkey</t>
+        </is>
+      </c>
       <c r="E53" s="7" t="n"/>
       <c r="F53" s="7" t="n"/>
       <c r="G53" s="7" t="n"/>
@@ -1402,15 +1402,15 @@
     </row>
     <row r="54">
       <c r="A54" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="B54" s="7" t="n"/>
+        <v>12</v>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>Travis Etienne Jr.</t>
+        </is>
+      </c>
       <c r="C54" s="7" t="n"/>
-      <c r="D54" s="7" t="inlineStr">
-        <is>
-          <t>Ladd McConkey</t>
-        </is>
-      </c>
+      <c r="D54" s="7" t="n"/>
       <c r="E54" s="7" t="n"/>
       <c r="F54" s="7" t="n"/>
       <c r="G54" s="7" t="n"/>
@@ -1420,13 +1420,13 @@
       <c r="A55" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B55" s="7" t="inlineStr">
-        <is>
-          <t>Travis Etienne Jr.</t>
-        </is>
-      </c>
+      <c r="B55" s="7" t="n"/>
       <c r="C55" s="7" t="n"/>
-      <c r="D55" s="7" t="n"/>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>Mike Evans</t>
+        </is>
+      </c>
       <c r="E55" s="7" t="n"/>
       <c r="F55" s="7" t="n"/>
       <c r="G55" s="7" t="n"/>
@@ -1440,7 +1440,7 @@
       <c r="C56" s="7" t="n"/>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>Mike Evans</t>
+          <t>Michael Wilson</t>
         </is>
       </c>
       <c r="E56" s="7" t="n"/>
@@ -1450,15 +1450,15 @@
     </row>
     <row r="57">
       <c r="A57" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="B57" s="7" t="n"/>
+        <v>11</v>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>David Montgomery</t>
+        </is>
+      </c>
       <c r="C57" s="7" t="n"/>
-      <c r="D57" s="7" t="inlineStr">
-        <is>
-          <t>Michael Wilson</t>
-        </is>
-      </c>
+      <c r="D57" s="7" t="n"/>
       <c r="E57" s="7" t="n"/>
       <c r="F57" s="7" t="n"/>
       <c r="G57" s="7" t="n"/>
@@ -1468,13 +1468,13 @@
       <c r="A58" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="B58" s="7" t="inlineStr">
-        <is>
-          <t>David Montgomery</t>
-        </is>
-      </c>
+      <c r="B58" s="7" t="n"/>
       <c r="C58" s="7" t="n"/>
-      <c r="D58" s="7" t="n"/>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>Emeka Egbuka</t>
+        </is>
+      </c>
       <c r="E58" s="7" t="n"/>
       <c r="F58" s="7" t="n"/>
       <c r="G58" s="7" t="n"/>
@@ -1482,13 +1482,13 @@
     </row>
     <row r="59">
       <c r="A59" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B59" s="7" t="n"/>
       <c r="C59" s="7" t="n"/>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>Emeka Egbuka</t>
+          <t>Luther Burden III</t>
         </is>
       </c>
       <c r="E59" s="7" t="n"/>
@@ -1504,7 +1504,7 @@
       <c r="C60" s="7" t="n"/>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>Luther Burden III</t>
+          <t>Terry McLaurin</t>
         </is>
       </c>
       <c r="E60" s="7" t="n"/>
@@ -1514,13 +1514,13 @@
     </row>
     <row r="61">
       <c r="A61" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B61" s="7" t="n"/>
       <c r="C61" s="7" t="n"/>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>Terry McLaurin</t>
+          <t>DJ Moore</t>
         </is>
       </c>
       <c r="E61" s="7" t="n"/>
@@ -1536,7 +1536,7 @@
       <c r="C62" s="7" t="n"/>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>DJ Moore</t>
+          <t>Matthew Golden</t>
         </is>
       </c>
       <c r="E62" s="7" t="n"/>
@@ -1546,15 +1546,15 @@
     </row>
     <row r="63">
       <c r="A63" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="B63" s="7" t="n"/>
+        <v>8</v>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>Bhayshul Tuten</t>
+        </is>
+      </c>
       <c r="C63" s="7" t="n"/>
-      <c r="D63" s="7" t="inlineStr">
-        <is>
-          <t>Matthew Golden</t>
-        </is>
-      </c>
+      <c r="D63" s="7" t="n"/>
       <c r="E63" s="7" t="n"/>
       <c r="F63" s="7" t="n"/>
       <c r="G63" s="7" t="n"/>
@@ -1598,7 +1598,7 @@
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>Bhayshul Tuten</t>
+          <t>Rhamondre Stevenson</t>
         </is>
       </c>
       <c r="C66" s="7" t="n"/>
@@ -1612,13 +1612,13 @@
       <c r="A67" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B67" s="7" t="inlineStr">
-        <is>
-          <t>Rhamondre Stevenson</t>
-        </is>
-      </c>
+      <c r="B67" s="7" t="n"/>
       <c r="C67" s="7" t="n"/>
-      <c r="D67" s="7" t="n"/>
+      <c r="D67" s="7" t="inlineStr">
+        <is>
+          <t>Carnell Tate</t>
+        </is>
+      </c>
       <c r="E67" s="7" t="n"/>
       <c r="F67" s="7" t="n"/>
       <c r="G67" s="7" t="n"/>
@@ -1626,15 +1626,15 @@
     </row>
     <row r="68">
       <c r="A68" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="B68" s="7" t="n"/>
+        <v>6</v>
+      </c>
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>Jadarian Price</t>
+        </is>
+      </c>
       <c r="C68" s="7" t="n"/>
-      <c r="D68" s="7" t="inlineStr">
-        <is>
-          <t>Carnell Tate</t>
-        </is>
-      </c>
+      <c r="D68" s="7" t="n"/>
       <c r="E68" s="7" t="n"/>
       <c r="F68" s="7" t="n"/>
       <c r="G68" s="7" t="n"/>
@@ -1644,13 +1644,13 @@
       <c r="A69" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B69" s="7" t="inlineStr">
-        <is>
-          <t>Jadarian Price</t>
-        </is>
-      </c>
+      <c r="B69" s="7" t="n"/>
       <c r="C69" s="7" t="n"/>
-      <c r="D69" s="7" t="n"/>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>Alec Pierce</t>
+        </is>
+      </c>
       <c r="E69" s="7" t="n"/>
       <c r="F69" s="7" t="n"/>
       <c r="G69" s="7" t="n"/>
@@ -1664,7 +1664,7 @@
       <c r="C70" s="7" t="n"/>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>Alec Pierce</t>
+          <t>Stefon Diggs</t>
         </is>
       </c>
       <c r="E70" s="7" t="n"/>
@@ -1678,13 +1678,13 @@
       </c>
       <c r="B71" s="7" t="n"/>
       <c r="C71" s="7" t="n"/>
-      <c r="D71" s="7" t="inlineStr">
-        <is>
-          <t>Stefon Diggs</t>
-        </is>
-      </c>
+      <c r="D71" s="7" t="n"/>
       <c r="E71" s="7" t="n"/>
-      <c r="F71" s="7" t="n"/>
+      <c r="F71" s="7" t="inlineStr">
+        <is>
+          <t>Colston Loveland</t>
+        </is>
+      </c>
       <c r="G71" s="7" t="n"/>
       <c r="H71" s="7" t="n"/>
     </row>
@@ -1698,7 +1698,7 @@
       <c r="E72" s="7" t="n"/>
       <c r="F72" s="7" t="inlineStr">
         <is>
-          <t>Colston Loveland</t>
+          <t>George Kittle</t>
         </is>
       </c>
       <c r="G72" s="7" t="n"/>
@@ -1706,35 +1706,35 @@
     </row>
     <row r="73">
       <c r="A73" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B73" s="7" t="n"/>
+        <v>4</v>
+      </c>
+      <c r="B73" s="7" t="inlineStr">
+        <is>
+          <t>MarShawn Lloyd</t>
+        </is>
+      </c>
       <c r="C73" s="7" t="n"/>
       <c r="D73" s="7" t="n"/>
       <c r="E73" s="7" t="n"/>
-      <c r="F73" s="7" t="inlineStr">
-        <is>
-          <t>George Kittle</t>
-        </is>
-      </c>
+      <c r="F73" s="7" t="n"/>
       <c r="G73" s="7" t="n"/>
       <c r="H73" s="7" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B74" s="7" t="n"/>
+        <v>4</v>
+      </c>
+      <c r="B74" s="7" t="inlineStr">
+        <is>
+          <t>TreVeyon Henderson</t>
+        </is>
+      </c>
       <c r="C74" s="7" t="n"/>
       <c r="D74" s="7" t="n"/>
       <c r="E74" s="7" t="n"/>
       <c r="F74" s="7" t="n"/>
       <c r="G74" s="7" t="n"/>
-      <c r="H74" s="7" t="inlineStr">
-        <is>
-          <t>Drake Maye</t>
-        </is>
-      </c>
+      <c r="H74" s="7" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="6" t="n">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="B75" s="7" t="inlineStr">
         <is>
-          <t>MarShawn Lloyd</t>
+          <t>Josh Jacobs</t>
         </is>
       </c>
       <c r="C75" s="7" t="n"/>
@@ -1758,7 +1758,7 @@
       </c>
       <c r="B76" s="7" t="inlineStr">
         <is>
-          <t>TreVeyon Henderson</t>
+          <t>Kenny Gainwell</t>
         </is>
       </c>
       <c r="C76" s="7" t="n"/>
@@ -1772,13 +1772,13 @@
       <c r="A77" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B77" s="7" t="inlineStr">
-        <is>
-          <t>Josh Jacobs</t>
-        </is>
-      </c>
+      <c r="B77" s="7" t="n"/>
       <c r="C77" s="7" t="n"/>
-      <c r="D77" s="7" t="n"/>
+      <c r="D77" s="7" t="inlineStr">
+        <is>
+          <t>Rome Odunze</t>
+        </is>
+      </c>
       <c r="E77" s="7" t="n"/>
       <c r="F77" s="7" t="n"/>
       <c r="G77" s="7" t="n"/>
@@ -1788,13 +1788,13 @@
       <c r="A78" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B78" s="7" t="inlineStr">
-        <is>
-          <t>Kenny Gainwell</t>
-        </is>
-      </c>
+      <c r="B78" s="7" t="n"/>
       <c r="C78" s="7" t="n"/>
-      <c r="D78" s="7" t="n"/>
+      <c r="D78" s="7" t="inlineStr">
+        <is>
+          <t>KC Concepcion</t>
+        </is>
+      </c>
       <c r="E78" s="7" t="n"/>
       <c r="F78" s="7" t="n"/>
       <c r="G78" s="7" t="n"/>
@@ -1808,7 +1808,7 @@
       <c r="C79" s="7" t="n"/>
       <c r="D79" s="7" t="inlineStr">
         <is>
-          <t>Rome Odunze</t>
+          <t>Jayden Reed</t>
         </is>
       </c>
       <c r="E79" s="7" t="n"/>
@@ -1824,7 +1824,7 @@
       <c r="C80" s="7" t="n"/>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>KC Concepcion</t>
+          <t>Jordyn Tyson</t>
         </is>
       </c>
       <c r="E80" s="7" t="n"/>
@@ -1838,15 +1838,15 @@
       </c>
       <c r="B81" s="7" t="n"/>
       <c r="C81" s="7" t="n"/>
-      <c r="D81" s="7" t="inlineStr">
-        <is>
-          <t>Jayden Reed</t>
-        </is>
-      </c>
+      <c r="D81" s="7" t="n"/>
       <c r="E81" s="7" t="n"/>
       <c r="F81" s="7" t="n"/>
       <c r="G81" s="7" t="n"/>
-      <c r="H81" s="7" t="n"/>
+      <c r="H81" s="7" t="inlineStr">
+        <is>
+          <t>Joe Burrow</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="6" t="n">
@@ -1854,61 +1854,61 @@
       </c>
       <c r="B82" s="7" t="n"/>
       <c r="C82" s="7" t="n"/>
-      <c r="D82" s="7" t="inlineStr">
-        <is>
-          <t>Jordyn Tyson</t>
-        </is>
-      </c>
+      <c r="D82" s="7" t="n"/>
       <c r="E82" s="7" t="n"/>
       <c r="F82" s="7" t="n"/>
       <c r="G82" s="7" t="n"/>
-      <c r="H82" s="7" t="n"/>
+      <c r="H82" s="7" t="inlineStr">
+        <is>
+          <t>Jayden Daniels</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B83" s="7" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="B83" s="7" t="inlineStr">
+        <is>
+          <t>Rachaad White</t>
+        </is>
+      </c>
       <c r="C83" s="7" t="n"/>
       <c r="D83" s="7" t="n"/>
       <c r="E83" s="7" t="n"/>
       <c r="F83" s="7" t="n"/>
       <c r="G83" s="7" t="n"/>
-      <c r="H83" s="7" t="inlineStr">
-        <is>
-          <t>Joe Burrow</t>
-        </is>
-      </c>
+      <c r="H83" s="7" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B84" s="7" t="n"/>
       <c r="C84" s="7" t="n"/>
-      <c r="D84" s="7" t="n"/>
+      <c r="D84" s="7" t="inlineStr">
+        <is>
+          <t>DK Metcalf</t>
+        </is>
+      </c>
       <c r="E84" s="7" t="n"/>
       <c r="F84" s="7" t="n"/>
       <c r="G84" s="7" t="n"/>
-      <c r="H84" s="7" t="inlineStr">
-        <is>
-          <t>Jayden Daniels</t>
-        </is>
-      </c>
+      <c r="H84" s="7" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B85" s="7" t="inlineStr">
-        <is>
-          <t>Rachaad White</t>
-        </is>
-      </c>
+      <c r="B85" s="7" t="n"/>
       <c r="C85" s="7" t="n"/>
       <c r="D85" s="7" t="n"/>
       <c r="E85" s="7" t="n"/>
-      <c r="F85" s="7" t="n"/>
+      <c r="F85" s="7" t="inlineStr">
+        <is>
+          <t>Isaiah Likely</t>
+        </is>
+      </c>
       <c r="G85" s="7" t="n"/>
       <c r="H85" s="7" t="n"/>
     </row>
@@ -1918,15 +1918,15 @@
       </c>
       <c r="B86" s="7" t="n"/>
       <c r="C86" s="7" t="n"/>
-      <c r="D86" s="7" t="inlineStr">
-        <is>
-          <t>DK Metcalf</t>
-        </is>
-      </c>
+      <c r="D86" s="7" t="n"/>
       <c r="E86" s="7" t="n"/>
       <c r="F86" s="7" t="n"/>
       <c r="G86" s="7" t="n"/>
-      <c r="H86" s="7" t="n"/>
+      <c r="H86" s="7" t="inlineStr">
+        <is>
+          <t>Drake Maye</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="6" t="n">
@@ -1936,29 +1936,29 @@
       <c r="C87" s="7" t="n"/>
       <c r="D87" s="7" t="n"/>
       <c r="E87" s="7" t="n"/>
-      <c r="F87" s="7" t="inlineStr">
-        <is>
-          <t>Isaiah Likely</t>
-        </is>
-      </c>
+      <c r="F87" s="7" t="n"/>
       <c r="G87" s="7" t="n"/>
-      <c r="H87" s="7" t="n"/>
+      <c r="H87" s="7" t="inlineStr">
+        <is>
+          <t>Dak Prescott</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B88" s="7" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="B88" s="7" t="inlineStr">
+        <is>
+          <t>Jordan Mason</t>
+        </is>
+      </c>
       <c r="C88" s="7" t="n"/>
       <c r="D88" s="7" t="n"/>
       <c r="E88" s="7" t="n"/>
       <c r="F88" s="7" t="n"/>
       <c r="G88" s="7" t="n"/>
-      <c r="H88" s="7" t="inlineStr">
-        <is>
-          <t>Dak Prescott</t>
-        </is>
-      </c>
+      <c r="H88" s="7" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="6" t="n">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="B89" s="7" t="inlineStr">
         <is>
-          <t>Jordan Mason</t>
+          <t>J.K. Dobbins</t>
         </is>
       </c>
       <c r="C89" s="7" t="n"/>
@@ -1982,7 +1982,7 @@
       </c>
       <c r="B90" s="7" t="inlineStr">
         <is>
-          <t>J.K. Dobbins</t>
+          <t>Jacory Croskey-Merritt</t>
         </is>
       </c>
       <c r="C90" s="7" t="n"/>
@@ -1994,11 +1994,11 @@
     </row>
     <row r="91">
       <c r="A91" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B91" s="7" t="inlineStr">
         <is>
-          <t>Jacory Croskey-Merritt</t>
+          <t>Tony Pollard</t>
         </is>
       </c>
       <c r="C91" s="7" t="n"/>
@@ -2014,7 +2014,7 @@
       </c>
       <c r="B92" s="7" t="inlineStr">
         <is>
-          <t>Tony Pollard</t>
+          <t>Jonathon Brooks</t>
         </is>
       </c>
       <c r="C92" s="7" t="n"/>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="B93" s="7" t="inlineStr">
         <is>
-          <t>Jonathon Brooks</t>
+          <t>Mike Washington Jr.</t>
         </is>
       </c>
       <c r="C93" s="7" t="n"/>
@@ -2046,7 +2046,7 @@
       </c>
       <c r="B94" s="7" t="inlineStr">
         <is>
-          <t>Mike Washington Jr.</t>
+          <t>Rico Dowdle</t>
         </is>
       </c>
       <c r="C94" s="7" t="n"/>
@@ -2062,7 +2062,7 @@
       </c>
       <c r="B95" s="7" t="inlineStr">
         <is>
-          <t>Rico Dowdle</t>
+          <t>Blake Corum</t>
         </is>
       </c>
       <c r="C95" s="7" t="n"/>
@@ -2078,7 +2078,7 @@
       </c>
       <c r="B96" s="7" t="inlineStr">
         <is>
-          <t>Blake Corum</t>
+          <t>Woody Marks</t>
         </is>
       </c>
       <c r="C96" s="7" t="n"/>
@@ -2092,13 +2092,13 @@
       <c r="A97" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B97" s="7" t="inlineStr">
-        <is>
-          <t>Woody Marks</t>
-        </is>
-      </c>
+      <c r="B97" s="7" t="n"/>
       <c r="C97" s="7" t="n"/>
-      <c r="D97" s="7" t="n"/>
+      <c r="D97" s="7" t="inlineStr">
+        <is>
+          <t>Brian Thomas Jr.</t>
+        </is>
+      </c>
       <c r="E97" s="7" t="n"/>
       <c r="F97" s="7" t="n"/>
       <c r="G97" s="7" t="n"/>
@@ -2112,7 +2112,7 @@
       <c r="C98" s="7" t="n"/>
       <c r="D98" s="7" t="inlineStr">
         <is>
-          <t>Brian Thomas Jr.</t>
+          <t>Marvin Harrison Jr.</t>
         </is>
       </c>
       <c r="E98" s="7" t="n"/>
@@ -2128,7 +2128,7 @@
       <c r="C99" s="7" t="n"/>
       <c r="D99" s="7" t="inlineStr">
         <is>
-          <t>Marvin Harrison Jr.</t>
+          <t>Quentin Johnston</t>
         </is>
       </c>
       <c r="E99" s="7" t="n"/>
@@ -2144,7 +2144,7 @@
       <c r="C100" s="7" t="n"/>
       <c r="D100" s="7" t="inlineStr">
         <is>
-          <t>Quentin Johnston</t>
+          <t>Chris Godwin Jr.</t>
         </is>
       </c>
       <c r="E100" s="7" t="n"/>
@@ -2160,7 +2160,7 @@
       <c r="C101" s="7" t="n"/>
       <c r="D101" s="7" t="inlineStr">
         <is>
-          <t>Chris Godwin Jr.</t>
+          <t>Ja'Kobi Lane</t>
         </is>
       </c>
       <c r="E101" s="7" t="n"/>
@@ -2174,13 +2174,13 @@
       </c>
       <c r="B102" s="7" t="n"/>
       <c r="C102" s="7" t="n"/>
-      <c r="D102" s="7" t="inlineStr">
-        <is>
-          <t>Ja'Kobi Lane</t>
-        </is>
-      </c>
+      <c r="D102" s="7" t="n"/>
       <c r="E102" s="7" t="n"/>
-      <c r="F102" s="7" t="n"/>
+      <c r="F102" s="7" t="inlineStr">
+        <is>
+          <t>Tucker Kraft</t>
+        </is>
+      </c>
       <c r="G102" s="7" t="n"/>
       <c r="H102" s="7" t="n"/>
     </row>
@@ -2194,7 +2194,7 @@
       <c r="E103" s="7" t="n"/>
       <c r="F103" s="7" t="inlineStr">
         <is>
-          <t>Tucker Kraft</t>
+          <t>Harold Fannin Jr.</t>
         </is>
       </c>
       <c r="G103" s="7" t="n"/>
@@ -2208,13 +2208,13 @@
       <c r="C104" s="7" t="n"/>
       <c r="D104" s="7" t="n"/>
       <c r="E104" s="7" t="n"/>
-      <c r="F104" s="7" t="inlineStr">
-        <is>
-          <t>Harold Fannin Jr.</t>
-        </is>
-      </c>
+      <c r="F104" s="7" t="n"/>
       <c r="G104" s="7" t="n"/>
-      <c r="H104" s="7" t="n"/>
+      <c r="H104" s="7" t="inlineStr">
+        <is>
+          <t>Trevor Lawrence</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="6" t="n">
@@ -2228,7 +2228,7 @@
       <c r="G105" s="7" t="n"/>
       <c r="H105" s="7" t="inlineStr">
         <is>
-          <t>Trevor Lawrence</t>
+          <t>Jalen Hurts</t>
         </is>
       </c>
     </row>
@@ -2244,7 +2244,7 @@
       <c r="G106" s="7" t="n"/>
       <c r="H106" s="7" t="inlineStr">
         <is>
-          <t>Jalen Hurts</t>
+          <t>Justin Herbert</t>
         </is>
       </c>
     </row>
@@ -2259,22 +2259,6 @@
       <c r="F107" s="7" t="n"/>
       <c r="G107" s="7" t="n"/>
       <c r="H107" s="7" t="inlineStr">
-        <is>
-          <t>Justin Herbert</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B108" s="7" t="n"/>
-      <c r="C108" s="7" t="n"/>
-      <c r="D108" s="7" t="n"/>
-      <c r="E108" s="7" t="n"/>
-      <c r="F108" s="7" t="n"/>
-      <c r="G108" s="7" t="n"/>
-      <c r="H108" s="7" t="inlineStr">
         <is>
           <t>Jaxson Dart</t>
         </is>
@@ -2311,7 +2295,7 @@
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>Baseline: the live Trade Values Google Sheet (Half PPR, 10-team), 105 players, top value 76.</t>
+          <t>Baseline: the live Trade Values Google Sheet (Half PPR, 10-team), 104 players, top value 76.</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2319,7 @@
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   (Projections page snapshot 1; 13 players used week 3 medians): implied = 0.7 x the seed value at the player's projection-rank slot among the projected players at the position + 0.3 x</t>
+          <t xml:space="preserve">   (Projections page snapshot 1; 12 players used week 3 medians): implied = 0.7 x the seed value at the player's projection-rank slot among the projected players at the position + 0.3 x</t>
         </is>
       </c>
     </row>
@@ -2349,7 +2333,7 @@
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   new = sheet + 0.45 x (implied - sheet), then rescaled so the total equals the sheet total. 83 players moved.</t>
+          <t xml:space="preserve">   new = sheet + 0.45 x (implied - sheet), then rescaled so the total equals the sheet total. 81 players moved.</t>
         </is>
       </c>
     </row>
@@ -2435,7 +2419,7 @@
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>Largest moves vs. the baseline in this file: James Cook III 52-&gt;44, Derrick Henry 57-&gt;49, Josh Allen 38-&gt;31, Omarion Hampton 27-&gt;21, Kyren Williams 26-&gt;20, Lamar Jackson 26-&gt;20, Bhayshul Tuten 12-&gt;7, Jonathan Taylor 63-&gt;59</t>
+          <t>Largest moves vs. the baseline in this file: James Cook III 52-&gt;44, Derrick Henry 57-&gt;49, Josh Allen 42-&gt;35, Omarion Hampton 27-&gt;21, Kyren Williams 26-&gt;20, Lamar Jackson 26-&gt;20, Jonathan Taylor 63-&gt;59, Kenneth Walker III 64-&gt;60</t>
         </is>
       </c>
     </row>

</xml_diff>